<commit_message>
Add daily task record for 2026-05-14
Notable: 31% external affairs (三菱協同組合 会合・懇親会),
KES meeting 67min, forklift monthly inspection.

https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11,14 +11,15 @@
     <sheet name="1週間（例）" sheetId="3" state="visible" r:id="rId3"/>
     <sheet name="2026-05-12" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-05-13" sheetId="5" state="visible" r:id="rId5"/>
+    <sheet name="2026-05-14" sheetId="6" state="visible" r:id="rId6"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId6"/>
     <externalReference r:id="rId7"/>
     <externalReference r:id="rId8"/>
     <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
     <externalReference r:id="rId11"/>
+    <externalReference r:id="rId12"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -588,7 +589,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="41">
+  <borders count="42">
     <border>
       <left/>
       <right/>
@@ -1025,11 +1026,18 @@
       <bottom style="thin"/>
       <diagonal/>
     </border>
+    <border>
+      <left/>
+      <right/>
+      <top/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
   </borders>
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="116">
+  <cellXfs count="117">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1314,6 +1322,7 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="39" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -10983,11 +10992,11 @@
     </row>
     <row r="4" ht="20" customHeight="1" thickBot="1">
       <c r="B4" s="113" t="n"/>
-      <c r="C4" s="110" t="n"/>
-      <c r="D4" s="110" t="n"/>
-      <c r="E4" s="110" t="n"/>
-      <c r="F4" s="110" t="n"/>
-      <c r="G4" s="111" t="n"/>
+      <c r="C4" s="116" t="n"/>
+      <c r="D4" s="116" t="n"/>
+      <c r="E4" s="116" t="n"/>
+      <c r="F4" s="116" t="n"/>
+      <c r="G4" s="112" t="n"/>
     </row>
     <row r="5" ht="18" customHeight="1">
       <c r="B5" s="113" t="n"/>
@@ -11109,11 +11118,11 @@
     </row>
     <row r="14" ht="20" customHeight="1">
       <c r="B14" s="112" t="n"/>
-      <c r="C14" s="110" t="n"/>
-      <c r="D14" s="110" t="n"/>
-      <c r="E14" s="110" t="n"/>
-      <c r="F14" s="110" t="n"/>
-      <c r="G14" s="111" t="n"/>
+      <c r="C14" s="116" t="n"/>
+      <c r="D14" s="116" t="n"/>
+      <c r="E14" s="116" t="n"/>
+      <c r="F14" s="116" t="n"/>
+      <c r="G14" s="112" t="n"/>
     </row>
     <row r="15" ht="22" customHeight="1">
       <c r="B15" s="52" t="inlineStr">
@@ -11436,8 +11445,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="R3:T3"/>
     <mergeCell ref="E11:G11"/>
-    <mergeCell ref="R3:T3"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -15445,6 +15454,11 @@
           <t>2026年5月13日（水）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -16024,6 +16038,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C23" s="110" t="n"/>
+      <c r="D23" s="110" t="n"/>
+      <c r="E23" s="110" t="n"/>
+      <c r="F23" s="110" t="n"/>
+      <c r="G23" s="111" t="n"/>
     </row>
     <row r="24">
       <c r="B24" s="52" t="inlineStr">
@@ -16210,4 +16229,764 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet6.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月14日（木）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="inlineStr">
+        <is>
+          <t>8:02</t>
+        </is>
+      </c>
+      <c r="G4" s="98" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E5" s="100" t="inlineStr">
+        <is>
+          <t>8:02</t>
+        </is>
+      </c>
+      <c r="F5" s="100" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="G5" s="100" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D6" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E6" s="106" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="F6" s="106" t="inlineStr">
+        <is>
+          <t>8:12</t>
+        </is>
+      </c>
+      <c r="G6" s="106" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D7" s="105" t="inlineStr">
+        <is>
+          <t>フォークリフト月次点検</t>
+        </is>
+      </c>
+      <c r="E7" s="106" t="inlineStr">
+        <is>
+          <t>8:12</t>
+        </is>
+      </c>
+      <c r="F7" s="106" t="inlineStr">
+        <is>
+          <t>8:30</t>
+        </is>
+      </c>
+      <c r="G7" s="106" t="n">
+        <v>18</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C8" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D8" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（見積・客先メール・作業時間検討・人事評価検討）</t>
+        </is>
+      </c>
+      <c r="E8" s="102" t="inlineStr">
+        <is>
+          <t>8:30</t>
+        </is>
+      </c>
+      <c r="F8" s="102" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="G8" s="102" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D9" s="97" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E9" s="98" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F9" s="98" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G9" s="98" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C10" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D10" s="97" t="inlineStr">
+        <is>
+          <t>中央通路 冷蔵庫掃除</t>
+        </is>
+      </c>
+      <c r="E10" s="98" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F10" s="98" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="G10" s="98" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C11" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D11" s="99" t="inlineStr">
+        <is>
+          <t>KES会議</t>
+        </is>
+      </c>
+      <c r="E11" s="100" t="inlineStr">
+        <is>
+          <t>10:18</t>
+        </is>
+      </c>
+      <c r="F11" s="100" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="G11" s="100" t="n">
+        <v>67</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C12" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D12" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（見積もり検討）</t>
+        </is>
+      </c>
+      <c r="E12" s="102" t="inlineStr">
+        <is>
+          <t>11:25</t>
+        </is>
+      </c>
+      <c r="F12" s="102" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="G12" s="102" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="97" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E13" s="98" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F13" s="98" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="G13" s="98" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C14" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D14" s="97" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E14" s="98" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F14" s="98" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="G14" s="98" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C15" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D15" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E15" s="106" t="inlineStr">
+        <is>
+          <t>12:54</t>
+        </is>
+      </c>
+      <c r="F15" s="106" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G15" s="106" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C16" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D16" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（社内回覧作成・客先納品引き取り事前連絡）</t>
+        </is>
+      </c>
+      <c r="E16" s="102" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F16" s="102" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="G16" s="102" t="n">
+        <v>71</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C17" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
+        <is>
+          <t>着替え・移動（伊丹菱栄会）</t>
+        </is>
+      </c>
+      <c r="E17" s="98" t="inlineStr">
+        <is>
+          <t>14:11</t>
+        </is>
+      </c>
+      <c r="F17" s="98" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="G17" s="98" t="n">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C18" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D18" s="97" t="inlineStr">
+        <is>
+          <t>現地待機</t>
+        </is>
+      </c>
+      <c r="E18" s="98" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="F18" s="98" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G18" s="98" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D19" s="107" t="inlineStr">
+        <is>
+          <t>伊丹菱栄会（三菱協同組合 会合）</t>
+        </is>
+      </c>
+      <c r="E19" s="108" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="F19" s="108" t="inlineStr">
+        <is>
+          <t>18:06</t>
+        </is>
+      </c>
+      <c r="G19" s="108" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C20" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D20" s="107" t="inlineStr">
+        <is>
+          <t>伊丹菱栄会 懇親会・会食（移動含む）</t>
+        </is>
+      </c>
+      <c r="E20" s="108" t="inlineStr">
+        <is>
+          <t>18:06</t>
+        </is>
+      </c>
+      <c r="F20" s="108" t="inlineStr">
+        <is>
+          <t>20:40</t>
+        </is>
+      </c>
+      <c r="G20" s="108" t="n">
+        <v>154</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C23" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D23" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E23" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F23" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G23" s="53" t="n"/>
+    </row>
+    <row r="24" ht="18" customHeight="1">
+      <c r="B24" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C24" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D24" s="108" t="n">
+        <v>220</v>
+      </c>
+      <c r="E24" s="108" t="n">
+        <v>3.7</v>
+      </c>
+      <c r="F24" s="108" t="n">
+        <v>31.4</v>
+      </c>
+      <c r="G24" s="57" t="n"/>
+    </row>
+    <row r="25" ht="18" customHeight="1">
+      <c r="B25" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C25" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D25" s="100" t="n">
+        <v>70</v>
+      </c>
+      <c r="E25" s="100" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F25" s="100" t="n">
+        <v>10</v>
+      </c>
+      <c r="G25" s="61" t="n"/>
+    </row>
+    <row r="26" ht="18" customHeight="1">
+      <c r="B26" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D26" s="106" t="n">
+        <v>31</v>
+      </c>
+      <c r="E26" s="106" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F26" s="106" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="G26" s="65" t="n"/>
+    </row>
+    <row r="27" ht="18" customHeight="1">
+      <c r="B27" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C27" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D27" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="69" t="n"/>
+    </row>
+    <row r="28" ht="18" customHeight="1">
+      <c r="B28" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C28" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D28" s="102" t="n">
+        <v>211</v>
+      </c>
+      <c r="E28" s="102" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F28" s="102" t="n">
+        <v>30.1</v>
+      </c>
+      <c r="G28" s="73" t="n"/>
+    </row>
+    <row r="29" ht="18" customHeight="1">
+      <c r="B29" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C29" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D29" s="98" t="n">
+        <v>168</v>
+      </c>
+      <c r="E29" s="98" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F29" s="98" t="n">
+        <v>24</v>
+      </c>
+      <c r="G29" s="77" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C30" s="86" t="inlineStr"/>
+      <c r="D30" s="86" t="n">
+        <v>700</v>
+      </c>
+      <c r="E30" s="86" t="n">
+        <v>11.7</v>
+      </c>
+      <c r="F30" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G30" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add daily task records for 2026-05-15 and 2026-05-18
5/15: 笠取工場 治具整理・FL点検、現場直接作業27%
5/18: 週初め朝礼・昼礼、来客対応、見積・パワポ・AI実験

https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -12,14 +12,16 @@
     <sheet name="2026-05-12" sheetId="4" state="visible" r:id="rId4"/>
     <sheet name="2026-05-13" sheetId="5" state="visible" r:id="rId5"/>
     <sheet name="2026-05-14" sheetId="6" state="visible" r:id="rId6"/>
+    <sheet name="2026-05-15" sheetId="7" state="visible" r:id="rId7"/>
+    <sheet name="2026-05-18" sheetId="8" state="visible" r:id="rId8"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId7"/>
-    <externalReference r:id="rId8"/>
     <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
     <externalReference r:id="rId11"/>
     <externalReference r:id="rId12"/>
+    <externalReference r:id="rId13"/>
+    <externalReference r:id="rId14"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -11445,8 +11447,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="R3:T3"/>
-    <mergeCell ref="E11:G11"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -16254,6 +16256,11 @@
           <t>2026年5月14日（木）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -16803,6 +16810,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C22" s="110" t="n"/>
+      <c r="D22" s="110" t="n"/>
+      <c r="E22" s="110" t="n"/>
+      <c r="F22" s="110" t="n"/>
+      <c r="G22" s="111" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="52" t="inlineStr">
@@ -16976,6 +16988,1586 @@
       </c>
       <c r="E30" s="86" t="n">
         <v>11.7</v>
+      </c>
+      <c r="F30" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G30" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet7.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G32"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月15日（金）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C4" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D4" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック</t>
+        </is>
+      </c>
+      <c r="E4" s="102" t="inlineStr">
+        <is>
+          <t>7:37</t>
+        </is>
+      </c>
+      <c r="F4" s="102" t="inlineStr">
+        <is>
+          <t>7:52</t>
+        </is>
+      </c>
+      <c r="G4" s="102" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C5" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D5" s="97" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E5" s="98" t="inlineStr">
+        <is>
+          <t>7:52</t>
+        </is>
+      </c>
+      <c r="F5" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="G5" s="98" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C6" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D6" s="97" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E6" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F6" s="98" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G6" s="98" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C7" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D7" s="99" t="inlineStr">
+        <is>
+          <t>各作業場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E7" s="100" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F7" s="100" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G7" s="100" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C8" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D8" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E8" s="106" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F8" s="106" t="inlineStr">
+        <is>
+          <t>8:26</t>
+        </is>
+      </c>
+      <c r="G8" s="106" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D9" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メールチェック・見積・仕組みづくり）</t>
+        </is>
+      </c>
+      <c r="E9" s="102" t="inlineStr">
+        <is>
+          <t>8:26</t>
+        </is>
+      </c>
+      <c r="F9" s="102" t="inlineStr">
+        <is>
+          <t>8:53</t>
+        </is>
+      </c>
+      <c r="G9" s="102" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C10" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D10" s="99" t="inlineStr">
+        <is>
+          <t>社長と雑談</t>
+        </is>
+      </c>
+      <c r="E10" s="100" t="inlineStr">
+        <is>
+          <t>8:53</t>
+        </is>
+      </c>
+      <c r="F10" s="100" t="inlineStr">
+        <is>
+          <t>9:19</t>
+        </is>
+      </c>
+      <c r="G10" s="100" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C11" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D11" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（支給品材料確認等）</t>
+        </is>
+      </c>
+      <c r="E11" s="102" t="inlineStr">
+        <is>
+          <t>9:19</t>
+        </is>
+      </c>
+      <c r="F11" s="102" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="G11" s="102" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E12" s="98" t="inlineStr">
+        <is>
+          <t>10:07</t>
+        </is>
+      </c>
+      <c r="F12" s="98" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="G12" s="98" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C13" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D13" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（支給品支給日確認・見積作業）</t>
+        </is>
+      </c>
+      <c r="E13" s="102" t="inlineStr">
+        <is>
+          <t>10:09</t>
+        </is>
+      </c>
+      <c r="F13" s="102" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="G13" s="102" t="n">
+        <v>126</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C14" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D14" s="97" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E14" s="98" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F14" s="98" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="G14" s="98" t="n">
+        <v>27</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C15" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D15" s="97" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E15" s="98" t="inlineStr">
+        <is>
+          <t>12:42</t>
+        </is>
+      </c>
+      <c r="F15" s="98" t="inlineStr">
+        <is>
+          <t>12:52</t>
+        </is>
+      </c>
+      <c r="G15" s="98" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C16" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D16" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（PC整理・メールチェック）</t>
+        </is>
+      </c>
+      <c r="E16" s="102" t="inlineStr">
+        <is>
+          <t>12:52</t>
+        </is>
+      </c>
+      <c r="F16" s="102" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="G16" s="102" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C17" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
+        <is>
+          <t>笠取工場へ移動</t>
+        </is>
+      </c>
+      <c r="E17" s="98" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="F17" s="98" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="G17" s="98" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C18" s="66" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D18" s="103" t="inlineStr">
+        <is>
+          <t>治具・金型・保管品整理・FL点検記録・メール対応</t>
+        </is>
+      </c>
+      <c r="E18" s="104" t="inlineStr">
+        <is>
+          <t>13:25</t>
+        </is>
+      </c>
+      <c r="F18" s="104" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="G18" s="104" t="n">
+        <v>99</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C19" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D19" s="97" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E19" s="98" t="inlineStr">
+        <is>
+          <t>15:04</t>
+        </is>
+      </c>
+      <c r="F19" s="98" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="G19" s="98" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C20" s="66" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D20" s="103" t="inlineStr">
+        <is>
+          <t>治具・金型・保管品整理（再開）</t>
+        </is>
+      </c>
+      <c r="E20" s="104" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="F20" s="104" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="G20" s="104" t="n">
+        <v>70</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1">
+      <c r="B21" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C21" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D21" s="97" t="inlineStr">
+        <is>
+          <t>笠取→本社工場 移動</t>
+        </is>
+      </c>
+      <c r="E21" s="98" t="inlineStr">
+        <is>
+          <t>16:20</t>
+        </is>
+      </c>
+      <c r="F21" s="98" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="G21" s="98" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="22" ht="18" customHeight="1">
+      <c r="B22" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C22" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D22" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック・客先へメール送信</t>
+        </is>
+      </c>
+      <c r="E22" s="102" t="inlineStr">
+        <is>
+          <t>16:35</t>
+        </is>
+      </c>
+      <c r="F22" s="102" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="G22" s="102" t="n">
+        <v>85</v>
+      </c>
+    </row>
+    <row r="24" ht="20" customHeight="1">
+      <c r="B24" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C25" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D25" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E25" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F25" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G25" s="53" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C26" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D26" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="57" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C27" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D27" s="100" t="n">
+        <v>29</v>
+      </c>
+      <c r="E27" s="100" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F27" s="100" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="G27" s="61" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C28" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D28" s="106" t="n">
+        <v>20</v>
+      </c>
+      <c r="E28" s="106" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F28" s="106" t="n">
+        <v>3.2</v>
+      </c>
+      <c r="G28" s="65" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C29" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D29" s="104" t="n">
+        <v>169</v>
+      </c>
+      <c r="E29" s="104" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="F29" s="104" t="n">
+        <v>27.1</v>
+      </c>
+      <c r="G29" s="69" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C30" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D30" s="102" t="n">
+        <v>314</v>
+      </c>
+      <c r="E30" s="102" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F30" s="102" t="n">
+        <v>50.4</v>
+      </c>
+      <c r="G30" s="73" t="n"/>
+    </row>
+    <row r="31">
+      <c r="B31" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C31" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D31" s="98" t="n">
+        <v>91</v>
+      </c>
+      <c r="E31" s="98" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F31" s="98" t="n">
+        <v>14.6</v>
+      </c>
+      <c r="G31" s="77" t="n"/>
+    </row>
+    <row r="32" ht="22" customHeight="1">
+      <c r="B32" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C32" s="86" t="inlineStr"/>
+      <c r="D32" s="86" t="n">
+        <v>623</v>
+      </c>
+      <c r="E32" s="86" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="F32" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G32" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B24:G24"/>
+    <mergeCell ref="B2:G2"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet8.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G30"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月18日（月）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G4" s="98" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>各作業場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E5" s="100" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F5" s="100" t="inlineStr">
+        <is>
+          <t>8:08</t>
+        </is>
+      </c>
+      <c r="G5" s="100" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D6" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E6" s="106" t="inlineStr">
+        <is>
+          <t>8:08</t>
+        </is>
+      </c>
+      <c r="F6" s="106" t="inlineStr">
+        <is>
+          <t>8:18</t>
+        </is>
+      </c>
+      <c r="G6" s="106" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D7" s="101" t="inlineStr">
+        <is>
+          <t>事務作業</t>
+        </is>
+      </c>
+      <c r="E7" s="102" t="inlineStr">
+        <is>
+          <t>8:18</t>
+        </is>
+      </c>
+      <c r="F7" s="102" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="G7" s="102" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C8" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D8" s="99" t="inlineStr">
+        <is>
+          <t>週初め朝礼（関係者）</t>
+        </is>
+      </c>
+      <c r="E8" s="100" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="F8" s="100" t="inlineStr">
+        <is>
+          <t>9:45</t>
+        </is>
+      </c>
+      <c r="G8" s="100" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D9" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック</t>
+        </is>
+      </c>
+      <c r="E9" s="102" t="inlineStr">
+        <is>
+          <t>9:45</t>
+        </is>
+      </c>
+      <c r="F9" s="102" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="G9" s="102" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C10" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D10" s="97" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E10" s="98" t="inlineStr">
+        <is>
+          <t>10:01</t>
+        </is>
+      </c>
+      <c r="F10" s="98" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G10" s="98" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="97" t="inlineStr">
+        <is>
+          <t>客先へ移動（打ち合わせ・支給品引き取り）</t>
+        </is>
+      </c>
+      <c r="E11" s="98" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F11" s="98" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="G11" s="98" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D12" s="107" t="inlineStr">
+        <is>
+          <t>客先打ち合わせ・支給品引き取り</t>
+        </is>
+      </c>
+      <c r="E12" s="108" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F12" s="108" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G12" s="108" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="97" t="inlineStr">
+        <is>
+          <t>帰社移動</t>
+        </is>
+      </c>
+      <c r="E13" s="98" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="F13" s="98" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="G13" s="98" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C14" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D14" s="97" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E14" s="98" t="inlineStr">
+        <is>
+          <t>12:14</t>
+        </is>
+      </c>
+      <c r="F14" s="98" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="G14" s="98" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C15" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D15" s="99" t="inlineStr">
+        <is>
+          <t>週初め昼礼</t>
+        </is>
+      </c>
+      <c r="E15" s="100" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F15" s="100" t="inlineStr">
+        <is>
+          <t>12:52</t>
+        </is>
+      </c>
+      <c r="G15" s="100" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C16" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D16" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E16" s="106" t="inlineStr">
+        <is>
+          <t>12:52</t>
+        </is>
+      </c>
+      <c r="F16" s="106" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="G16" s="106" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C17" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D17" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メール確認・返信・見積）</t>
+        </is>
+      </c>
+      <c r="E17" s="102" t="inlineStr">
+        <is>
+          <t>13:03</t>
+        </is>
+      </c>
+      <c r="F17" s="102" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="G17" s="102" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C18" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D18" s="107" t="inlineStr">
+        <is>
+          <t>来客対応</t>
+        </is>
+      </c>
+      <c r="E18" s="108" t="inlineStr">
+        <is>
+          <t>13:31</t>
+        </is>
+      </c>
+      <c r="F18" s="108" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="G18" s="108" t="n">
+        <v>79</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（一般）</t>
+        </is>
+      </c>
+      <c r="E19" s="102" t="inlineStr">
+        <is>
+          <t>14:50</t>
+        </is>
+      </c>
+      <c r="F19" s="102" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="G19" s="102" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1">
+      <c r="B20" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C20" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D20" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（見積・仕組み構築・パワポ作成・AI実験）</t>
+        </is>
+      </c>
+      <c r="E20" s="102" t="inlineStr">
+        <is>
+          <t>15:30</t>
+        </is>
+      </c>
+      <c r="F20" s="102" t="inlineStr">
+        <is>
+          <t>18:08</t>
+        </is>
+      </c>
+      <c r="G20" s="102" t="n">
+        <v>158</v>
+      </c>
+    </row>
+    <row r="22" ht="20" customHeight="1">
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C23" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D23" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E23" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F23" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G23" s="53" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C24" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D24" s="108" t="n">
+        <v>109</v>
+      </c>
+      <c r="E24" s="108" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F24" s="108" t="n">
+        <v>17.9</v>
+      </c>
+      <c r="G24" s="57" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C25" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D25" s="100" t="n">
+        <v>57</v>
+      </c>
+      <c r="E25" s="100" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F25" s="100" t="n">
+        <v>9.4</v>
+      </c>
+      <c r="G25" s="61" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C26" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D26" s="106" t="n">
+        <v>21</v>
+      </c>
+      <c r="E26" s="106" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F26" s="106" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="G26" s="65" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C27" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D27" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E27" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F27" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G27" s="69" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C28" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D28" s="102" t="n">
+        <v>284</v>
+      </c>
+      <c r="E28" s="102" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F28" s="102" t="n">
+        <v>46.7</v>
+      </c>
+      <c r="G28" s="73" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C29" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D29" s="98" t="n">
+        <v>137</v>
+      </c>
+      <c r="E29" s="98" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F29" s="98" t="n">
+        <v>22.5</v>
+      </c>
+      <c r="G29" s="77" t="n"/>
+    </row>
+    <row r="30" ht="22" customHeight="1">
+      <c r="B30" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C30" s="86" t="inlineStr"/>
+      <c r="D30" s="86" t="n">
+        <v>608</v>
+      </c>
+      <c r="E30" s="86" t="n">
+        <v>10.1</v>
       </c>
       <c r="F30" s="86" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add daily task record for 2026-05-19
Notable: 61.6% external affairs (来客対応・協力会社訪問),
PC replacement setup 115min after hours.

https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14,14 +14,15 @@
     <sheet name="2026-05-14" sheetId="6" state="visible" r:id="rId6"/>
     <sheet name="2026-05-15" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-05-18" sheetId="8" state="visible" r:id="rId8"/>
+    <sheet name="2026-05-19" sheetId="9" state="visible" r:id="rId9"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId9"/>
     <externalReference r:id="rId10"/>
     <externalReference r:id="rId11"/>
     <externalReference r:id="rId12"/>
     <externalReference r:id="rId13"/>
     <externalReference r:id="rId14"/>
+    <externalReference r:id="rId15"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -11447,8 +11448,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="R3:T3"/>
     <mergeCell ref="E11:G11"/>
-    <mergeCell ref="R3:T3"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -17026,6 +17027,11 @@
           <t>2026年5月15日（金）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -17635,6 +17641,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C24" s="110" t="n"/>
+      <c r="D24" s="110" t="n"/>
+      <c r="E24" s="110" t="n"/>
+      <c r="F24" s="110" t="n"/>
+      <c r="G24" s="111" t="n"/>
     </row>
     <row r="25">
       <c r="B25" s="52" t="inlineStr">
@@ -17846,6 +17857,11 @@
           <t>2026年5月18日（月）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -18395,6 +18411,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C22" s="110" t="n"/>
+      <c r="D22" s="110" t="n"/>
+      <c r="E22" s="110" t="n"/>
+      <c r="F22" s="110" t="n"/>
+      <c r="G22" s="111" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="52" t="inlineStr">
@@ -18581,4 +18602,554 @@
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G23"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="40" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月19日（火）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G4" s="98" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>各作業場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E5" s="100" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F5" s="100" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G5" s="100" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D6" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E6" s="106" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F6" s="106" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="G6" s="106" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D7" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メールチェック・見積）</t>
+        </is>
+      </c>
+      <c r="E7" s="102" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="F7" s="102" t="inlineStr">
+        <is>
+          <t>9:30</t>
+        </is>
+      </c>
+      <c r="G7" s="102" t="n">
+        <v>75</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C8" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D8" s="107" t="inlineStr">
+        <is>
+          <t>来客対応</t>
+        </is>
+      </c>
+      <c r="E8" s="108" t="inlineStr">
+        <is>
+          <t>9:30</t>
+        </is>
+      </c>
+      <c r="F8" s="108" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="G8" s="108" t="n">
+        <v>292</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D9" s="97" t="inlineStr">
+        <is>
+          <t>協力会社訪問へ移動</t>
+        </is>
+      </c>
+      <c r="E9" s="98" t="inlineStr">
+        <is>
+          <t>14:22</t>
+        </is>
+      </c>
+      <c r="F9" s="98" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="G9" s="98" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C10" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D10" s="107" t="inlineStr">
+        <is>
+          <t>協力会社訪問・見学・打ち合わせ</t>
+        </is>
+      </c>
+      <c r="E10" s="108" t="inlineStr">
+        <is>
+          <t>14:30</t>
+        </is>
+      </c>
+      <c r="F10" s="108" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="G10" s="108" t="n">
+        <v>130</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="97" t="inlineStr">
+        <is>
+          <t>帰社移動</t>
+        </is>
+      </c>
+      <c r="E11" s="98" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="F11" s="98" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="G11" s="98" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C12" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D12" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メールチェック）</t>
+        </is>
+      </c>
+      <c r="E12" s="102" t="inlineStr">
+        <is>
+          <t>16:50</t>
+        </is>
+      </c>
+      <c r="F12" s="102" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="G12" s="102" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C13" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D13" s="101" t="inlineStr">
+        <is>
+          <t>PC入れ替え・セットアップ</t>
+        </is>
+      </c>
+      <c r="E13" s="102" t="inlineStr">
+        <is>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="F13" s="102" t="inlineStr">
+        <is>
+          <t>19:25</t>
+        </is>
+      </c>
+      <c r="G13" s="102" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="15" ht="20" customHeight="1">
+      <c r="B15" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C16" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D16" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E16" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F16" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G16" s="53" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C17" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D17" s="108" t="n">
+        <v>422</v>
+      </c>
+      <c r="E17" s="108" t="n">
+        <v>7</v>
+      </c>
+      <c r="F17" s="108" t="n">
+        <v>61.6</v>
+      </c>
+      <c r="G17" s="57" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C18" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D18" s="100" t="n">
+        <v>3</v>
+      </c>
+      <c r="E18" s="100" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F18" s="100" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="G18" s="61" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C19" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D19" s="106" t="n">
+        <v>9</v>
+      </c>
+      <c r="E19" s="106" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F19" s="106" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G19" s="65" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C20" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D20" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E20" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F20" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G20" s="69" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C21" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D21" s="102" t="n">
+        <v>230</v>
+      </c>
+      <c r="E21" s="102" t="n">
+        <v>3.8</v>
+      </c>
+      <c r="F21" s="102" t="n">
+        <v>33.6</v>
+      </c>
+      <c r="G21" s="73" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C22" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D22" s="98" t="n">
+        <v>21</v>
+      </c>
+      <c r="E22" s="98" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F22" s="98" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G22" s="77" t="n"/>
+    </row>
+    <row r="23" ht="22" customHeight="1">
+      <c r="B23" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C23" s="86" t="inlineStr"/>
+      <c r="D23" s="86" t="n">
+        <v>685</v>
+      </c>
+      <c r="E23" s="86" t="n">
+        <v>11.4</v>
+      </c>
+      <c r="F23" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G23" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B15:G15"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add daily task record for 2026-05-20
Notable: 交流会(5/23)買い出し・笠取運搬240min,
人事評価システムアプリ製作, PC設定続き.

https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -15,14 +15,15 @@
     <sheet name="2026-05-15" sheetId="7" state="visible" r:id="rId7"/>
     <sheet name="2026-05-18" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-05-19" sheetId="9" state="visible" r:id="rId9"/>
+    <sheet name="2026-05-20" sheetId="10" state="visible" r:id="rId10"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId10"/>
     <externalReference r:id="rId11"/>
     <externalReference r:id="rId12"/>
     <externalReference r:id="rId13"/>
     <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
+    <externalReference r:id="rId16"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -11448,8 +11449,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="R3:T3"/>
-    <mergeCell ref="E11:G11"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -11471,6 +11472,616 @@
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup orientation="portrait" paperSize="9" horizontalDpi="1200" verticalDpi="1200"/>
   <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId1"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet10.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G25"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月20日（水）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C4" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D4" s="101" t="inlineStr">
+        <is>
+          <t>PCセッティング（続き）</t>
+        </is>
+      </c>
+      <c r="E4" s="102" t="inlineStr">
+        <is>
+          <t>7:36</t>
+        </is>
+      </c>
+      <c r="F4" s="102" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="G4" s="102" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C5" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D5" s="97" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E5" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F5" s="98" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G5" s="98" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C6" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D6" s="99" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E6" s="100" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F6" s="100" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G6" s="100" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C7" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D7" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E7" s="106" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F7" s="106" t="inlineStr">
+        <is>
+          <t>8:20</t>
+        </is>
+      </c>
+      <c r="G7" s="106" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C8" s="66" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D8" s="103" t="inlineStr">
+        <is>
+          <t>本社治具の確認・整理</t>
+        </is>
+      </c>
+      <c r="E8" s="104" t="inlineStr">
+        <is>
+          <t>8:20</t>
+        </is>
+      </c>
+      <c r="F8" s="104" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="G8" s="104" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C9" s="66" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D9" s="103" t="inlineStr">
+        <is>
+          <t>社内設備の整理（突発・作業者依頼）</t>
+        </is>
+      </c>
+      <c r="E9" s="104" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="F9" s="104" t="inlineStr">
+        <is>
+          <t>8:55</t>
+        </is>
+      </c>
+      <c r="G9" s="104" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C10" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D10" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メールチェック・見積書・人事評価システムアプリ製作）</t>
+        </is>
+      </c>
+      <c r="E10" s="102" t="inlineStr">
+        <is>
+          <t>8:55</t>
+        </is>
+      </c>
+      <c r="F10" s="102" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="G10" s="102" t="n">
+        <v>198</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="97" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E11" s="98" t="inlineStr">
+        <is>
+          <t>12:13</t>
+        </is>
+      </c>
+      <c r="F11" s="98" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="G11" s="98" t="n">
+        <v>32</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E12" s="98" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F12" s="98" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="G12" s="98" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="97" t="inlineStr">
+        <is>
+          <t>準備</t>
+        </is>
+      </c>
+      <c r="E13" s="98" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="F13" s="98" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G13" s="98" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C14" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D14" s="99" t="inlineStr">
+        <is>
+          <t>交流会（5/23）買い出し・笠取工場へ運搬</t>
+        </is>
+      </c>
+      <c r="E14" s="100" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F14" s="100" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G14" s="100" t="n">
+        <v>240</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C15" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D15" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック・返信</t>
+        </is>
+      </c>
+      <c r="E15" s="102" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="F15" s="102" t="inlineStr">
+        <is>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="G15" s="102" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C18" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D18" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E18" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F18" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G18" s="53" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C19" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D19" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E19" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F19" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G19" s="57" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C20" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D20" s="100" t="n">
+        <v>243</v>
+      </c>
+      <c r="E20" s="100" t="n">
+        <v>4</v>
+      </c>
+      <c r="F20" s="100" t="n">
+        <v>38.9</v>
+      </c>
+      <c r="G20" s="61" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C21" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D21" s="106" t="n">
+        <v>14</v>
+      </c>
+      <c r="E21" s="106" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F21" s="106" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="G21" s="65" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C22" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D22" s="104" t="n">
+        <v>35</v>
+      </c>
+      <c r="E22" s="104" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F22" s="104" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G22" s="69" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C23" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D23" s="102" t="n">
+        <v>282</v>
+      </c>
+      <c r="E23" s="102" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F23" s="102" t="n">
+        <v>45.2</v>
+      </c>
+      <c r="G23" s="73" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C24" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D24" s="98" t="n">
+        <v>50</v>
+      </c>
+      <c r="E24" s="98" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F24" s="98" t="n">
+        <v>8</v>
+      </c>
+      <c r="G24" s="77" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C25" s="86" t="inlineStr"/>
+      <c r="D25" s="86" t="n">
+        <v>624</v>
+      </c>
+      <c r="E25" s="86" t="n">
+        <v>10.4</v>
+      </c>
+      <c r="F25" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G25" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B17:G17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
 
@@ -18627,6 +19238,11 @@
           <t>2026年5月19日（火）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -18966,6 +19582,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C15" s="110" t="n"/>
+      <c r="D15" s="110" t="n"/>
+      <c r="E15" s="110" t="n"/>
+      <c r="F15" s="110" t="n"/>
+      <c r="G15" s="111" t="n"/>
     </row>
     <row r="16">
       <c r="B16" s="52" t="inlineStr">

</xml_diff>

<commit_message>
Add daily task record for 2026-05-21
Notable: 製造計画会議, WEB打ち合わせ, 交流会(5/23)買い出し・笠取運搬.
夜間再出社あり（16:45-19:00は私的時間除く）.

https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -16,14 +16,15 @@
     <sheet name="2026-05-18" sheetId="8" state="visible" r:id="rId8"/>
     <sheet name="2026-05-19" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-05-20" sheetId="10" state="visible" r:id="rId10"/>
+    <sheet name="2026-05-21" sheetId="11" state="visible" r:id="rId11"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId11"/>
     <externalReference r:id="rId12"/>
     <externalReference r:id="rId13"/>
     <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
+    <externalReference r:id="rId17"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -11449,8 +11450,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="R3:T3"/>
     <mergeCell ref="E11:G11"/>
-    <mergeCell ref="R3:T3"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -11498,6 +11499,11 @@
           <t>2026年5月20日（水）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -11897,6 +11903,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C17" s="110" t="n"/>
+      <c r="D17" s="110" t="n"/>
+      <c r="E17" s="110" t="n"/>
+      <c r="F17" s="110" t="n"/>
+      <c r="G17" s="111" t="n"/>
     </row>
     <row r="18">
       <c r="B18" s="52" t="inlineStr">
@@ -12080,6 +12091,736 @@
   <mergeCells count="2">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B17:G17"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月21日（木）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G4" s="98" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E5" s="100" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F5" s="100" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G5" s="100" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D6" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E6" s="106" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F6" s="106" t="inlineStr">
+        <is>
+          <t>8:20</t>
+        </is>
+      </c>
+      <c r="G6" s="106" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D7" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メールチェック・システム整理）</t>
+        </is>
+      </c>
+      <c r="E7" s="102" t="inlineStr">
+        <is>
+          <t>8:20</t>
+        </is>
+      </c>
+      <c r="F7" s="102" t="inlineStr">
+        <is>
+          <t>9:03</t>
+        </is>
+      </c>
+      <c r="G7" s="102" t="n">
+        <v>43</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C8" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D8" s="99" t="inlineStr">
+        <is>
+          <t>製造計画会議</t>
+        </is>
+      </c>
+      <c r="E8" s="100" t="inlineStr">
+        <is>
+          <t>9:03</t>
+        </is>
+      </c>
+      <c r="F8" s="100" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="G8" s="100" t="n">
+        <v>57</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C9" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D9" s="97" t="inlineStr">
+        <is>
+          <t>応接室の片づけ</t>
+        </is>
+      </c>
+      <c r="E9" s="98" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F9" s="98" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="G9" s="98" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C10" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D10" s="105" t="inlineStr">
+        <is>
+          <t>現場周り・研修参加者確認</t>
+        </is>
+      </c>
+      <c r="E10" s="106" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="F10" s="106" t="inlineStr">
+        <is>
+          <t>10:39</t>
+        </is>
+      </c>
+      <c r="G10" s="106" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C11" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D11" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メールチェック）</t>
+        </is>
+      </c>
+      <c r="E11" s="102" t="inlineStr">
+        <is>
+          <t>10:39</t>
+        </is>
+      </c>
+      <c r="F11" s="102" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="G11" s="102" t="n">
+        <v>96</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E12" s="98" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F12" s="98" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="G12" s="98" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="97" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E13" s="98" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="F13" s="98" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="G13" s="98" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C14" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D14" s="99" t="inlineStr">
+        <is>
+          <t>WEB打ち合わせ準備</t>
+        </is>
+      </c>
+      <c r="E14" s="100" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="F14" s="100" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G14" s="100" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C15" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D15" s="107" t="inlineStr">
+        <is>
+          <t>WEB打ち合わせ</t>
+        </is>
+      </c>
+      <c r="E15" s="108" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F15" s="108" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="G15" s="108" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C16" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D16" s="99" t="inlineStr">
+        <is>
+          <t>交流会（5/23）買い出し</t>
+        </is>
+      </c>
+      <c r="E16" s="100" t="inlineStr">
+        <is>
+          <t>14:45</t>
+        </is>
+      </c>
+      <c r="F16" s="100" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="G16" s="100" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C17" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D17" s="99" t="inlineStr">
+        <is>
+          <t>買い出し続き・再出社</t>
+        </is>
+      </c>
+      <c r="E17" s="100" t="inlineStr">
+        <is>
+          <t>19:00</t>
+        </is>
+      </c>
+      <c r="F17" s="100" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="G17" s="100" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C18" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D18" s="99" t="inlineStr">
+        <is>
+          <t>笠取工場 荷物運搬・持ち帰り</t>
+        </is>
+      </c>
+      <c r="E18" s="100" t="inlineStr">
+        <is>
+          <t>19:45</t>
+        </is>
+      </c>
+      <c r="F18" s="100" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="G18" s="100" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="101" t="inlineStr">
+        <is>
+          <t>事務作業</t>
+        </is>
+      </c>
+      <c r="E19" s="102" t="inlineStr">
+        <is>
+          <t>20:30</t>
+        </is>
+      </c>
+      <c r="F19" s="102" t="inlineStr">
+        <is>
+          <t>21:32</t>
+        </is>
+      </c>
+      <c r="G19" s="102" t="n">
+        <v>62</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C22" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D22" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E22" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F22" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G22" s="53" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C23" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D23" s="108" t="n">
+        <v>105</v>
+      </c>
+      <c r="E23" s="108" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F23" s="108" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G23" s="57" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C24" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D24" s="100" t="n">
+        <v>275</v>
+      </c>
+      <c r="E24" s="100" t="n">
+        <v>4.6</v>
+      </c>
+      <c r="F24" s="100" t="n">
+        <v>40.6</v>
+      </c>
+      <c r="G24" s="61" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D25" s="106" t="n">
+        <v>38</v>
+      </c>
+      <c r="E25" s="106" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F25" s="106" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="G25" s="65" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C26" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D26" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="69" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C27" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D27" s="102" t="n">
+        <v>201</v>
+      </c>
+      <c r="E27" s="102" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F27" s="102" t="n">
+        <v>29.7</v>
+      </c>
+      <c r="G27" s="73" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C28" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D28" s="98" t="n">
+        <v>58</v>
+      </c>
+      <c r="E28" s="98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F28" s="98" t="n">
+        <v>8.6</v>
+      </c>
+      <c r="G28" s="77" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C29" s="86" t="inlineStr"/>
+      <c r="D29" s="86" t="n">
+        <v>677</v>
+      </c>
+      <c r="E29" s="86" t="n">
+        <v>11.3</v>
+      </c>
+      <c r="F29" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G29" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B21:G21"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Fix 2026-05-21 end time: 21:32 → 21:53 (83min office work)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11450,8 +11450,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="R3:T3"/>
-    <mergeCell ref="E11:G11"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -12102,7 +12102,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B2:G29"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -12113,12 +12113,18 @@
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
+    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="96" t="inlineStr">
         <is>
           <t>2026年5月21日（木）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -12632,12 +12638,18 @@
         <v>62</v>
       </c>
     </row>
+    <row r="20"/>
     <row r="21">
       <c r="B21" s="52" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C21" s="110" t="n"/>
+      <c r="D21" s="110" t="n"/>
+      <c r="E21" s="110" t="n"/>
+      <c r="F21" s="110" t="n"/>
+      <c r="G21" s="111" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="52" t="inlineStr">
@@ -12685,7 +12697,7 @@
         <v>1.8</v>
       </c>
       <c r="F23" s="108" t="n">
-        <v>15.5</v>
+        <v>15</v>
       </c>
       <c r="G23" s="57" t="n"/>
     </row>
@@ -12707,7 +12719,7 @@
         <v>4.6</v>
       </c>
       <c r="F24" s="100" t="n">
-        <v>40.6</v>
+        <v>39.4</v>
       </c>
       <c r="G24" s="61" t="n"/>
     </row>
@@ -12729,7 +12741,7 @@
         <v>0.6</v>
       </c>
       <c r="F25" s="106" t="n">
-        <v>5.6</v>
+        <v>5.4</v>
       </c>
       <c r="G25" s="65" t="n"/>
     </row>
@@ -12767,13 +12779,13 @@
         </is>
       </c>
       <c r="D27" s="102" t="n">
-        <v>201</v>
+        <v>222</v>
       </c>
       <c r="E27" s="102" t="n">
-        <v>3.4</v>
+        <v>3.7</v>
       </c>
       <c r="F27" s="102" t="n">
-        <v>29.7</v>
+        <v>31.8</v>
       </c>
       <c r="G27" s="73" t="n"/>
     </row>
@@ -12795,7 +12807,7 @@
         <v>1</v>
       </c>
       <c r="F28" s="98" t="n">
-        <v>8.6</v>
+        <v>8.300000000000001</v>
       </c>
       <c r="G28" s="77" t="n"/>
     </row>
@@ -12807,10 +12819,10 @@
       </c>
       <c r="C29" s="86" t="inlineStr"/>
       <c r="D29" s="86" t="n">
-        <v>677</v>
+        <v>698</v>
       </c>
       <c r="E29" s="86" t="n">
-        <v>11.3</v>
+        <v>11.6</v>
       </c>
       <c r="F29" s="86" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add daily task record for 2026-05-22 (出張)
Business trip day: 客先打ち合わせ94min, 移動63%, 電話対応×3件.

https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -17,14 +17,15 @@
     <sheet name="2026-05-19" sheetId="9" state="visible" r:id="rId9"/>
     <sheet name="2026-05-20" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-05-21" sheetId="11" state="visible" r:id="rId11"/>
+    <sheet name="2026-05-22" sheetId="12" state="visible" r:id="rId12"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId12"/>
     <externalReference r:id="rId13"/>
     <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
+    <externalReference r:id="rId18"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -11450,8 +11451,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="R3:T3"/>
     <mergeCell ref="E11:G11"/>
-    <mergeCell ref="R3:T3"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -12102,7 +12103,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="B2:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="2" max="2"/>
@@ -12113,7 +12114,6 @@
     <col width="14" customWidth="1" min="7" max="7"/>
   </cols>
   <sheetData>
-    <row r="1"/>
     <row r="2" ht="26" customHeight="1">
       <c r="B2" s="96" t="inlineStr">
         <is>
@@ -12638,7 +12638,6 @@
         <v>62</v>
       </c>
     </row>
-    <row r="20"/>
     <row r="21">
       <c r="B21" s="52" t="inlineStr">
         <is>
@@ -12823,6 +12822,736 @@
       </c>
       <c r="E29" s="86" t="n">
         <v>11.6</v>
+      </c>
+      <c r="F29" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G29" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B21:G21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet12.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月22日（金）　業務記録　※出張</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>自宅出発・移動（出張・新幹線）</t>
+        </is>
+      </c>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>8:37</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="inlineStr">
+        <is>
+          <t>9:41</t>
+        </is>
+      </c>
+      <c r="G4" s="98" t="n">
+        <v>64</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C5" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D5" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック・返信（新幹線移動中）</t>
+        </is>
+      </c>
+      <c r="E5" s="102" t="inlineStr">
+        <is>
+          <t>9:41</t>
+        </is>
+      </c>
+      <c r="F5" s="102" t="inlineStr">
+        <is>
+          <t>9:44</t>
+        </is>
+      </c>
+      <c r="G5" s="102" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C6" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D6" s="107" t="inlineStr">
+        <is>
+          <t>客先電話対応（新幹線移動中）</t>
+        </is>
+      </c>
+      <c r="E6" s="108" t="inlineStr">
+        <is>
+          <t>9:44</t>
+        </is>
+      </c>
+      <c r="F6" s="108" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="G6" s="108" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D7" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（新幹線移動中）</t>
+        </is>
+      </c>
+      <c r="E7" s="102" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="F7" s="102" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G7" s="102" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C8" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D8" s="97" t="inlineStr">
+        <is>
+          <t>乗り換え待機</t>
+        </is>
+      </c>
+      <c r="E8" s="98" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F8" s="98" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="G8" s="98" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C9" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D9" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（新幹線移動中・再開）</t>
+        </is>
+      </c>
+      <c r="E9" s="102" t="inlineStr">
+        <is>
+          <t>10:27</t>
+        </is>
+      </c>
+      <c r="F9" s="102" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="G9" s="102" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C10" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D10" s="97" t="inlineStr">
+        <is>
+          <t>駅到着・昼食</t>
+        </is>
+      </c>
+      <c r="E10" s="98" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="F10" s="98" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="G10" s="98" t="n">
+        <v>66</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="97" t="inlineStr">
+        <is>
+          <t>客先へ移動（電車・徒歩）</t>
+        </is>
+      </c>
+      <c r="E11" s="98" t="inlineStr">
+        <is>
+          <t>12:01</t>
+        </is>
+      </c>
+      <c r="F11" s="98" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G11" s="98" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C12" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D12" s="107" t="inlineStr">
+        <is>
+          <t>客先打ち合わせ（出張）</t>
+        </is>
+      </c>
+      <c r="E12" s="108" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F12" s="108" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="G12" s="108" t="n">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="97" t="inlineStr">
+        <is>
+          <t>帰路移動（徒歩）</t>
+        </is>
+      </c>
+      <c r="E13" s="98" t="inlineStr">
+        <is>
+          <t>14:34</t>
+        </is>
+      </c>
+      <c r="F13" s="98" t="inlineStr">
+        <is>
+          <t>14:36</t>
+        </is>
+      </c>
+      <c r="G13" s="98" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C14" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D14" s="107" t="inlineStr">
+        <is>
+          <t>客先電話対応（帰路中）</t>
+        </is>
+      </c>
+      <c r="E14" s="108" t="inlineStr">
+        <is>
+          <t>14:36</t>
+        </is>
+      </c>
+      <c r="F14" s="108" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="G14" s="108" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C15" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D15" s="97" t="inlineStr">
+        <is>
+          <t>帰路移動（徒歩→駅）</t>
+        </is>
+      </c>
+      <c r="E15" s="98" t="inlineStr">
+        <is>
+          <t>14:38</t>
+        </is>
+      </c>
+      <c r="F15" s="98" t="inlineStr">
+        <is>
+          <t>15:39</t>
+        </is>
+      </c>
+      <c r="G15" s="98" t="n">
+        <v>61</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C16" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D16" s="101" t="inlineStr">
+        <is>
+          <t>メール確認・返信・電話対応（新幹線移動中）</t>
+        </is>
+      </c>
+      <c r="E16" s="102" t="inlineStr">
+        <is>
+          <t>15:39</t>
+        </is>
+      </c>
+      <c r="F16" s="102" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="G16" s="102" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C17" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
+        <is>
+          <t>乗り換え</t>
+        </is>
+      </c>
+      <c r="E17" s="98" t="inlineStr">
+        <is>
+          <t>16:07</t>
+        </is>
+      </c>
+      <c r="F17" s="98" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="G17" s="98" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C18" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D18" s="97" t="inlineStr">
+        <is>
+          <t>新幹線移動（帰路）</t>
+        </is>
+      </c>
+      <c r="E18" s="98" t="inlineStr">
+        <is>
+          <t>16:10</t>
+        </is>
+      </c>
+      <c r="F18" s="98" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="G18" s="98" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C19" s="54" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D19" s="107" t="inlineStr">
+        <is>
+          <t>客先電話対応</t>
+        </is>
+      </c>
+      <c r="E19" s="108" t="inlineStr">
+        <is>
+          <t>16:51</t>
+        </is>
+      </c>
+      <c r="F19" s="108" t="inlineStr">
+        <is>
+          <t>16:54</t>
+        </is>
+      </c>
+      <c r="G19" s="108" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C22" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D22" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E22" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F22" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G22" s="53" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C23" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D23" s="108" t="n">
+        <v>119</v>
+      </c>
+      <c r="E23" s="108" t="n">
+        <v>2</v>
+      </c>
+      <c r="F23" s="108" t="n">
+        <v>23.9</v>
+      </c>
+      <c r="G23" s="57" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C24" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D24" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E24" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F24" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="G24" s="61" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D25" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="65" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C26" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D26" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="104" t="n">
+        <v>0</v>
+      </c>
+      <c r="G26" s="69" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C27" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D27" s="102" t="n">
+        <v>65</v>
+      </c>
+      <c r="E27" s="102" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F27" s="102" t="n">
+        <v>13.1</v>
+      </c>
+      <c r="G27" s="73" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C28" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D28" s="98" t="n">
+        <v>313</v>
+      </c>
+      <c r="E28" s="98" t="n">
+        <v>5.2</v>
+      </c>
+      <c r="F28" s="98" t="n">
+        <v>63</v>
+      </c>
+      <c r="G28" s="77" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C29" s="86" t="inlineStr"/>
+      <c r="D29" s="86" t="n">
+        <v>497</v>
+      </c>
+      <c r="E29" s="86" t="n">
+        <v>8.300000000000001</v>
       </c>
       <c r="F29" s="86" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add daily task record for 2026-05-25
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -18,14 +18,15 @@
     <sheet name="2026-05-20" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-05-21" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-05-22" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-05-25" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId13"/>
     <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
+    <externalReference r:id="rId19"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -11451,8 +11452,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="R3:T3"/>
-    <mergeCell ref="E11:G11"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -12860,6 +12861,11 @@
           <t>2026年5月22日（金）　業務記録　※出張</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -13379,6 +13385,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C21" s="110" t="n"/>
+      <c r="D21" s="110" t="n"/>
+      <c r="E21" s="110" t="n"/>
+      <c r="F21" s="110" t="n"/>
+      <c r="G21" s="111" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="52" t="inlineStr">
@@ -13552,6 +13563,736 @@
       </c>
       <c r="E29" s="86" t="n">
         <v>8.300000000000001</v>
+      </c>
+      <c r="F29" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G29" s="109" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B2:G2"/>
+    <mergeCell ref="B21:G21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B2:G29"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="2" ht="26" customHeight="1">
+      <c r="B2" s="96" t="inlineStr">
+        <is>
+          <t>2026年5月25日（月）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="22" customHeight="1">
+      <c r="B3" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C3" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D3" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E3" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F3" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G3" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E4" s="98" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F4" s="98" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G4" s="98" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C5" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E5" s="100" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F5" s="100" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G5" s="100" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C6" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D6" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E6" s="106" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F6" s="106" t="inlineStr">
+        <is>
+          <t>8:16</t>
+        </is>
+      </c>
+      <c r="G6" s="106" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C7" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D7" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック・見積回答</t>
+        </is>
+      </c>
+      <c r="E7" s="102" t="inlineStr">
+        <is>
+          <t>8:16</t>
+        </is>
+      </c>
+      <c r="F7" s="102" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="G7" s="102" t="n">
+        <v>44</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1">
+      <c r="B8" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C8" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D8" s="99" t="inlineStr">
+        <is>
+          <t>週初め朝礼</t>
+        </is>
+      </c>
+      <c r="E8" s="100" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="F8" s="100" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="G8" s="100" t="n">
+        <v>40</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1">
+      <c r="B9" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C9" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D9" s="99" t="inlineStr">
+        <is>
+          <t>月次経営者会議</t>
+        </is>
+      </c>
+      <c r="E9" s="100" t="inlineStr">
+        <is>
+          <t>9:40</t>
+        </is>
+      </c>
+      <c r="F9" s="100" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="G9" s="100" t="n">
+        <v>107</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C10" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D10" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E10" s="106" t="inlineStr">
+        <is>
+          <t>11:27</t>
+        </is>
+      </c>
+      <c r="F10" s="106" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="G10" s="106" t="n">
+        <v>13</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C11" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D11" s="101" t="inlineStr">
+        <is>
+          <t>作業時間集計システム構築</t>
+        </is>
+      </c>
+      <c r="E11" s="102" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="F11" s="102" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="G11" s="102" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E12" s="98" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F12" s="98" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="G12" s="98" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C13" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D13" s="99" t="inlineStr">
+        <is>
+          <t>週初め昼礼</t>
+        </is>
+      </c>
+      <c r="E13" s="100" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F13" s="100" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="G13" s="100" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C14" s="62" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D14" s="105" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E14" s="106" t="inlineStr">
+        <is>
+          <t>12:50</t>
+        </is>
+      </c>
+      <c r="F14" s="106" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="G14" s="106" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C15" s="66" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D15" s="103" t="inlineStr">
+        <is>
+          <t>笠取工場 不用品整理</t>
+        </is>
+      </c>
+      <c r="E15" s="104" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="F15" s="104" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="G15" s="104" t="n">
+        <v>105</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C16" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D16" s="101" t="inlineStr">
+        <is>
+          <t>事務作業</t>
+        </is>
+      </c>
+      <c r="E16" s="102" t="inlineStr">
+        <is>
+          <t>14:40</t>
+        </is>
+      </c>
+      <c r="F16" s="102" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="G16" s="102" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C17" s="58" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D17" s="99" t="inlineStr">
+        <is>
+          <t>工程会議</t>
+        </is>
+      </c>
+      <c r="E17" s="100" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="F17" s="100" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="G17" s="100" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C18" s="74" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D18" s="97" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E18" s="98" t="inlineStr">
+        <is>
+          <t>16:45</t>
+        </is>
+      </c>
+      <c r="F18" s="98" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="G18" s="98" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1">
+      <c r="B19" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="70" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="101" t="inlineStr">
+        <is>
+          <t>事務作業（メールチェック・返信・見積もり）</t>
+        </is>
+      </c>
+      <c r="E19" s="102" t="inlineStr">
+        <is>
+          <t>17:00</t>
+        </is>
+      </c>
+      <c r="F19" s="102" t="inlineStr">
+        <is>
+          <t>19:23</t>
+        </is>
+      </c>
+      <c r="G19" s="102" t="n">
+        <v>143</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="52" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C22" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D22" s="52" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E22" s="52" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F22" s="52" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G22" s="53" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="54" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C23" s="55" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D23" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="E23" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="F23" s="108" t="n">
+        <v>0</v>
+      </c>
+      <c r="G23" s="57" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="58" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C24" s="59" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D24" s="100" t="n">
+        <v>250</v>
+      </c>
+      <c r="E24" s="100" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F24" s="100" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="G24" s="61" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="62" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C25" s="63" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D25" s="106" t="n">
+        <v>28</v>
+      </c>
+      <c r="E25" s="106" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F25" s="106" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G25" s="65" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="66" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C26" s="67" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D26" s="104" t="n">
+        <v>105</v>
+      </c>
+      <c r="E26" s="104" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F26" s="104" t="n">
+        <v>15.4</v>
+      </c>
+      <c r="G26" s="69" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="70" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C27" s="71" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D27" s="102" t="n">
+        <v>252</v>
+      </c>
+      <c r="E27" s="102" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F27" s="102" t="n">
+        <v>36.9</v>
+      </c>
+      <c r="G27" s="73" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="74" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C28" s="75" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D28" s="98" t="n">
+        <v>48</v>
+      </c>
+      <c r="E28" s="98" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F28" s="98" t="n">
+        <v>7</v>
+      </c>
+      <c r="G28" s="77" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="86" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C29" s="86" t="inlineStr"/>
+      <c r="D29" s="86" t="n">
+        <v>683</v>
+      </c>
+      <c r="E29" s="86" t="n">
+        <v>11.4</v>
       </c>
       <c r="F29" s="86" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add daily task record for 2026-05-26 (作業中)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -19,14 +19,15 @@
     <sheet name="2026-05-21" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-05-22" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-05-25" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-05-26" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
     <externalReference r:id="rId19"/>
+    <externalReference r:id="rId20"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -1044,7 +1045,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="117">
+  <cellXfs count="125">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center"/>
@@ -1330,6 +1331,30 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="33" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="34" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="41" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="5" fillId="9" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="18" fillId="16" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="14" fillId="12" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="13" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="15" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="13" fillId="11" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="14" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="5" fillId="10" borderId="31" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="right" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -11452,8 +11477,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="R3:T3"/>
     <mergeCell ref="E11:G11"/>
-    <mergeCell ref="R3:T3"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -13601,6 +13626,11 @@
           <t>2026年5月25日（月）　業務記録</t>
         </is>
       </c>
+      <c r="C2" s="110" t="n"/>
+      <c r="D2" s="110" t="n"/>
+      <c r="E2" s="110" t="n"/>
+      <c r="F2" s="110" t="n"/>
+      <c r="G2" s="111" t="n"/>
     </row>
     <row r="3" ht="22" customHeight="1">
       <c r="B3" s="52" t="inlineStr">
@@ -14120,6 +14150,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C21" s="110" t="n"/>
+      <c r="D21" s="110" t="n"/>
+      <c r="E21" s="110" t="n"/>
+      <c r="F21" s="110" t="n"/>
+      <c r="G21" s="111" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="52" t="inlineStr">
@@ -14303,6 +14338,354 @@
   <mergeCells count="2">
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="B21:G21"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" min="1" max="1"/>
+    <col width="6" customWidth="1" min="2" max="2"/>
+    <col width="20" customWidth="1" min="3" max="3"/>
+    <col width="42" customWidth="1" min="4" max="4"/>
+    <col width="8" customWidth="1" min="5" max="5"/>
+    <col width="8" customWidth="1" min="6" max="6"/>
+    <col width="14" customWidth="1" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1">
+      <c r="B1" s="117" t="inlineStr">
+        <is>
+          <t>業務記録　2026-05-26（火）</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1">
+      <c r="B2" s="52" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C2" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D2" s="52" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E2" s="52" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F2" s="52" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G2" s="52" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1">
+      <c r="B3" s="118" t="n">
+        <v>1</v>
+      </c>
+      <c r="C3" s="85" t="inlineStr">
+        <is>
+          <t>⑥ 定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D3" s="85" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E3" s="118" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F3" s="118" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G3" s="118" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1">
+      <c r="B4" s="119" t="n">
+        <v>2</v>
+      </c>
+      <c r="C4" s="81" t="inlineStr">
+        <is>
+          <t>② 社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D4" s="81" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E4" s="119" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F4" s="119" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G4" s="119" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1">
+      <c r="B5" s="120" t="n">
+        <v>3</v>
+      </c>
+      <c r="C5" s="82" t="inlineStr">
+        <is>
+          <t>③ 現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D5" s="82" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E5" s="120" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F5" s="120" t="inlineStr">
+        <is>
+          <t>8:13</t>
+        </is>
+      </c>
+      <c r="G5" s="120" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1">
+      <c r="B6" s="121" t="n">
+        <v>4</v>
+      </c>
+      <c r="C6" s="84" t="inlineStr">
+        <is>
+          <t>⑤ 社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D6" s="84" t="inlineStr">
+        <is>
+          <t>メールチェック・返信</t>
+        </is>
+      </c>
+      <c r="E6" s="121" t="inlineStr">
+        <is>
+          <t>8:13</t>
+        </is>
+      </c>
+      <c r="F6" s="121" t="inlineStr">
+        <is>
+          <t>8:23</t>
+        </is>
+      </c>
+      <c r="G6" s="121" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1">
+      <c r="B7" s="119" t="n">
+        <v>5</v>
+      </c>
+      <c r="C7" s="81" t="inlineStr">
+        <is>
+          <t>② 社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D7" s="81" t="inlineStr">
+        <is>
+          <t>作業時間管理システム構築（進行中）</t>
+        </is>
+      </c>
+      <c r="E7" s="119" t="inlineStr">
+        <is>
+          <t>8:23</t>
+        </is>
+      </c>
+      <c r="F7" s="119" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G7" s="119" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1">
+      <c r="B9" s="52" t="inlineStr">
+        <is>
+          <t>カテゴリ別集計</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1">
+      <c r="B10" s="122" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C10" s="80" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D10" s="80" t="inlineStr"/>
+      <c r="E10" s="122" t="inlineStr"/>
+      <c r="F10" s="122" t="inlineStr"/>
+      <c r="G10" s="122" t="inlineStr">
+        <is>
+          <t>0分 (0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="119" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C11" s="81" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D11" s="81" t="inlineStr"/>
+      <c r="E11" s="119" t="inlineStr"/>
+      <c r="F11" s="119" t="inlineStr"/>
+      <c r="G11" s="119" t="inlineStr">
+        <is>
+          <t>3分 (13.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="120" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C12" s="82" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D12" s="82" t="inlineStr"/>
+      <c r="E12" s="120" t="inlineStr"/>
+      <c r="F12" s="120" t="inlineStr"/>
+      <c r="G12" s="120" t="inlineStr">
+        <is>
+          <t>7分 (30.4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="123" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C13" s="83" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D13" s="83" t="inlineStr"/>
+      <c r="E13" s="123" t="inlineStr"/>
+      <c r="F13" s="123" t="inlineStr"/>
+      <c r="G13" s="123" t="inlineStr">
+        <is>
+          <t>0分 (0.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="121" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C14" s="84" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D14" s="84" t="inlineStr"/>
+      <c r="E14" s="121" t="inlineStr"/>
+      <c r="F14" s="121" t="inlineStr"/>
+      <c r="G14" s="121" t="inlineStr">
+        <is>
+          <t>10分 (43.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="118" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C15" s="85" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D15" s="85" t="inlineStr"/>
+      <c r="E15" s="118" t="inlineStr"/>
+      <c r="F15" s="118" t="inlineStr"/>
+      <c r="G15" s="118" t="inlineStr">
+        <is>
+          <t>3分 (13.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="20" customHeight="1">
+      <c r="B16" s="124" t="inlineStr">
+        <is>
+          <t>記録済み合計</t>
+        </is>
+      </c>
+      <c r="G16" s="52" t="inlineStr">
+        <is>
+          <t>23分 (0時間23分)</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="3">
+    <mergeCell ref="B16:F16"/>
+    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Update 2026-05-26: add consultant meeting (糸ぐち)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11477,8 +11477,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="R3:T3"/>
-    <mergeCell ref="E11:G11"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -14349,7 +14349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G16"/>
+  <dimension ref="B1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -14523,7 +14523,7 @@
       </c>
       <c r="D7" s="81" t="inlineStr">
         <is>
-          <t>作業時間管理システム構築（進行中）</t>
+          <t>作業時間管理システム構築</t>
         </is>
       </c>
       <c r="E7" s="119" t="inlineStr">
@@ -14533,158 +14533,187 @@
       </c>
       <c r="F7" s="119" t="inlineStr">
         <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="G7" s="119" t="n">
+        <v>112</v>
+      </c>
+    </row>
+    <row r="8" ht="30" customHeight="1">
+      <c r="B8" s="122" t="n">
+        <v>6</v>
+      </c>
+      <c r="C8" s="80" t="inlineStr">
+        <is>
+          <t>① 経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D8" s="80" t="inlineStr">
+        <is>
+          <t>コンサルタント来社・業務改善検討
+社内業務・作業の見直し・改善検討　進行中</t>
+        </is>
+      </c>
+      <c r="E8" s="122" t="inlineStr">
+        <is>
+          <t>10:15</t>
+        </is>
+      </c>
+      <c r="F8" s="122" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G7" s="119" t="inlineStr">
+      <c r="G8" s="122" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1">
-      <c r="B9" s="52" t="inlineStr">
+    <row r="10" ht="20" customHeight="1">
+      <c r="B10" s="52" t="inlineStr">
         <is>
           <t>カテゴリ別集計</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1">
-      <c r="B10" s="122" t="inlineStr">
+    <row r="11" ht="18" customHeight="1">
+      <c r="B11" s="122" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C10" s="80" t="inlineStr">
+      <c r="C11" s="80" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D10" s="80" t="inlineStr"/>
-      <c r="E10" s="122" t="inlineStr"/>
-      <c r="F10" s="122" t="inlineStr"/>
-      <c r="G10" s="122" t="inlineStr">
+      <c r="D11" s="80" t="inlineStr"/>
+      <c r="E11" s="122" t="inlineStr"/>
+      <c r="F11" s="122" t="inlineStr"/>
+      <c r="G11" s="122" t="inlineStr">
         <is>
           <t>0分 (0.0%)</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="B11" s="119" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="119" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C11" s="81" t="inlineStr">
+      <c r="C12" s="81" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D11" s="81" t="inlineStr"/>
-      <c r="E11" s="119" t="inlineStr"/>
-      <c r="F11" s="119" t="inlineStr"/>
-      <c r="G11" s="119" t="inlineStr">
-        <is>
-          <t>3分 (13.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="B12" s="120" t="inlineStr">
+      <c r="D12" s="81" t="inlineStr"/>
+      <c r="E12" s="119" t="inlineStr"/>
+      <c r="F12" s="119" t="inlineStr"/>
+      <c r="G12" s="119" t="inlineStr">
+        <is>
+          <t>115分 (85.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="120" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C12" s="82" t="inlineStr">
+      <c r="C13" s="82" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D12" s="82" t="inlineStr"/>
-      <c r="E12" s="120" t="inlineStr"/>
-      <c r="F12" s="120" t="inlineStr"/>
-      <c r="G12" s="120" t="inlineStr">
-        <is>
-          <t>7分 (30.4%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="B13" s="123" t="inlineStr">
+      <c r="D13" s="82" t="inlineStr"/>
+      <c r="E13" s="120" t="inlineStr"/>
+      <c r="F13" s="120" t="inlineStr"/>
+      <c r="G13" s="120" t="inlineStr">
+        <is>
+          <t>7分 (5.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="123" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C13" s="83" t="inlineStr">
+      <c r="C14" s="83" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D13" s="83" t="inlineStr"/>
-      <c r="E13" s="123" t="inlineStr"/>
-      <c r="F13" s="123" t="inlineStr"/>
-      <c r="G13" s="123" t="inlineStr">
+      <c r="D14" s="83" t="inlineStr"/>
+      <c r="E14" s="123" t="inlineStr"/>
+      <c r="F14" s="123" t="inlineStr"/>
+      <c r="G14" s="123" t="inlineStr">
         <is>
           <t>0分 (0.0%)</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="B14" s="121" t="inlineStr">
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="121" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C14" s="84" t="inlineStr">
+      <c r="C15" s="84" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D14" s="84" t="inlineStr"/>
-      <c r="E14" s="121" t="inlineStr"/>
-      <c r="F14" s="121" t="inlineStr"/>
-      <c r="G14" s="121" t="inlineStr">
-        <is>
-          <t>10分 (43.5%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="118" t="inlineStr">
+      <c r="D15" s="84" t="inlineStr"/>
+      <c r="E15" s="121" t="inlineStr"/>
+      <c r="F15" s="121" t="inlineStr"/>
+      <c r="G15" s="121" t="inlineStr">
+        <is>
+          <t>10分 (7.4%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="118" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C15" s="85" t="inlineStr">
+      <c r="C16" s="85" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D15" s="85" t="inlineStr"/>
-      <c r="E15" s="118" t="inlineStr"/>
-      <c r="F15" s="118" t="inlineStr"/>
-      <c r="G15" s="118" t="inlineStr">
-        <is>
-          <t>3分 (13.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="20" customHeight="1">
-      <c r="B16" s="124" t="inlineStr">
+      <c r="D16" s="85" t="inlineStr"/>
+      <c r="E16" s="118" t="inlineStr"/>
+      <c r="F16" s="118" t="inlineStr"/>
+      <c r="G16" s="118" t="inlineStr">
+        <is>
+          <t>3分 (2.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="20" customHeight="1">
+      <c r="B17" s="124" t="inlineStr">
         <is>
           <t>記録済み合計</t>
         </is>
       </c>
-      <c r="G16" s="52" t="inlineStr">
-        <is>
-          <t>23分 (0時間23分)</t>
+      <c r="G17" s="52" t="inlineStr">
+        <is>
+          <t>135分 (2時間15分)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B16:F16"/>
-    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B17:F17"/>
+    <mergeCell ref="B10:G10"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-26: add consultant company name 糸ぐち
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11477,8 +11477,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="R3:T3"/>
     <mergeCell ref="E11:G11"/>
-    <mergeCell ref="R3:T3"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -14552,7 +14552,7 @@
       <c r="D8" s="80" t="inlineStr">
         <is>
           <t>コンサルタント来社・業務改善検討
-社内業務・作業の見直し・改善検討　進行中</t>
+糸ぐち　社内業務・作業の見直し・改善検討　進行中</t>
         </is>
       </c>
       <c r="E8" s="122" t="inlineStr">

</xml_diff>

<commit_message>
Update 2026-05-26: close consultant meeting, add lunch break
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11477,8 +11477,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="E11:G11"/>
     <mergeCell ref="R3:T3"/>
-    <mergeCell ref="E11:G11"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -14349,7 +14349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G17"/>
+  <dimension ref="B1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -14552,7 +14552,7 @@
       <c r="D8" s="80" t="inlineStr">
         <is>
           <t>コンサルタント来社・業務改善検討
-糸ぐち　社内業務・作業の見直し・改善検討　進行中</t>
+糸ぐち　社内業務・作業の見直し・改善検討</t>
         </is>
       </c>
       <c r="E8" s="122" t="inlineStr">
@@ -14562,158 +14562,187 @@
       </c>
       <c r="F8" s="122" t="inlineStr">
         <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="G8" s="122" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" ht="30" customHeight="1">
+      <c r="B9" s="118" t="n">
+        <v>7</v>
+      </c>
+      <c r="C9" s="85" t="inlineStr">
+        <is>
+          <t>⑥ 定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D9" s="85" t="inlineStr">
+        <is>
+          <t>昼休憩
+進行中</t>
+        </is>
+      </c>
+      <c r="E9" s="118" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="F9" s="118" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G8" s="122" t="inlineStr">
+      <c r="G9" s="118" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1">
-      <c r="B10" s="52" t="inlineStr">
+    <row r="11" ht="20" customHeight="1">
+      <c r="B11" s="52" t="inlineStr">
         <is>
           <t>カテゴリ別集計</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1">
-      <c r="B11" s="122" t="inlineStr">
+    <row r="12" ht="18" customHeight="1">
+      <c r="B12" s="122" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C11" s="80" t="inlineStr">
+      <c r="C12" s="80" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D11" s="80" t="inlineStr"/>
-      <c r="E11" s="122" t="inlineStr"/>
-      <c r="F11" s="122" t="inlineStr"/>
-      <c r="G11" s="122" t="inlineStr">
+      <c r="D12" s="80" t="inlineStr"/>
+      <c r="E12" s="122" t="inlineStr"/>
+      <c r="F12" s="122" t="inlineStr"/>
+      <c r="G12" s="122" t="inlineStr">
+        <is>
+          <t>115分 (46.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="119" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C13" s="81" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D13" s="81" t="inlineStr"/>
+      <c r="E13" s="119" t="inlineStr"/>
+      <c r="F13" s="119" t="inlineStr"/>
+      <c r="G13" s="119" t="inlineStr">
+        <is>
+          <t>115分 (46.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="120" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C14" s="82" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D14" s="82" t="inlineStr"/>
+      <c r="E14" s="120" t="inlineStr"/>
+      <c r="F14" s="120" t="inlineStr"/>
+      <c r="G14" s="120" t="inlineStr">
+        <is>
+          <t>7分 (2.8%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="123" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C15" s="83" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D15" s="83" t="inlineStr"/>
+      <c r="E15" s="123" t="inlineStr"/>
+      <c r="F15" s="123" t="inlineStr"/>
+      <c r="G15" s="123" t="inlineStr">
         <is>
           <t>0分 (0.0%)</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="B12" s="119" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
-      <c r="C12" s="81" t="inlineStr">
-        <is>
-          <t>社内マネジメント</t>
-        </is>
-      </c>
-      <c r="D12" s="81" t="inlineStr"/>
-      <c r="E12" s="119" t="inlineStr"/>
-      <c r="F12" s="119" t="inlineStr"/>
-      <c r="G12" s="119" t="inlineStr">
-        <is>
-          <t>115分 (85.2%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="B13" s="120" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C13" s="82" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D13" s="82" t="inlineStr"/>
-      <c r="E13" s="120" t="inlineStr"/>
-      <c r="F13" s="120" t="inlineStr"/>
-      <c r="G13" s="120" t="inlineStr">
-        <is>
-          <t>7分 (5.2%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="B14" s="123" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C14" s="83" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D14" s="83" t="inlineStr"/>
-      <c r="E14" s="123" t="inlineStr"/>
-      <c r="F14" s="123" t="inlineStr"/>
-      <c r="G14" s="123" t="inlineStr">
-        <is>
-          <t>0分 (0.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="121" t="inlineStr">
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="121" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C15" s="84" t="inlineStr">
+      <c r="C16" s="84" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D15" s="84" t="inlineStr"/>
-      <c r="E15" s="121" t="inlineStr"/>
-      <c r="F15" s="121" t="inlineStr"/>
-      <c r="G15" s="121" t="inlineStr">
-        <is>
-          <t>10分 (7.4%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="118" t="inlineStr">
+      <c r="D16" s="84" t="inlineStr"/>
+      <c r="E16" s="121" t="inlineStr"/>
+      <c r="F16" s="121" t="inlineStr"/>
+      <c r="G16" s="121" t="inlineStr">
+        <is>
+          <t>10分 (4.0%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="118" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C16" s="85" t="inlineStr">
+      <c r="C17" s="85" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D16" s="85" t="inlineStr"/>
-      <c r="E16" s="118" t="inlineStr"/>
-      <c r="F16" s="118" t="inlineStr"/>
-      <c r="G16" s="118" t="inlineStr">
-        <is>
-          <t>3分 (2.2%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="20" customHeight="1">
-      <c r="B17" s="124" t="inlineStr">
+      <c r="D17" s="85" t="inlineStr"/>
+      <c r="E17" s="118" t="inlineStr"/>
+      <c r="F17" s="118" t="inlineStr"/>
+      <c r="G17" s="118" t="inlineStr">
+        <is>
+          <t>3分 (1.2%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="20" customHeight="1">
+      <c r="B18" s="124" t="inlineStr">
         <is>
           <t>記録済み合計</t>
         </is>
       </c>
-      <c r="G17" s="52" t="inlineStr">
-        <is>
-          <t>135分 (2時間15分)</t>
+      <c r="G18" s="52" t="inlineStr">
+        <is>
+          <t>250分 (4時間10分)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B17:F17"/>
-    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B18:F18"/>
+    <mergeCell ref="B11:G11"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-26: resume afternoon consultant session (糸ぐち)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11477,8 +11477,8 @@
     <mergeCell ref="B31:B43"/>
     <mergeCell ref="B2:G2"/>
     <mergeCell ref="E10:G10"/>
+    <mergeCell ref="R3:T3"/>
     <mergeCell ref="E11:G11"/>
-    <mergeCell ref="R3:T3"/>
     <mergeCell ref="C46:G46"/>
     <mergeCell ref="B14:G14"/>
     <mergeCell ref="B37:G37"/>
@@ -14349,7 +14349,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G18"/>
+  <dimension ref="B1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" min="1" max="1"/>
@@ -14569,7 +14569,7 @@
         <v>115</v>
       </c>
     </row>
-    <row r="9" ht="30" customHeight="1">
+    <row r="9" ht="18" customHeight="1">
       <c r="B9" s="118" t="n">
         <v>7</v>
       </c>
@@ -14580,8 +14580,7 @@
       </c>
       <c r="D9" s="85" t="inlineStr">
         <is>
-          <t>昼休憩
-進行中</t>
+          <t>昼休憩</t>
         </is>
       </c>
       <c r="E9" s="118" t="inlineStr">
@@ -14591,158 +14590,187 @@
       </c>
       <c r="F9" s="118" t="inlineStr">
         <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="G9" s="118" t="n">
+        <v>33</v>
+      </c>
+    </row>
+    <row r="10" ht="30" customHeight="1">
+      <c r="B10" s="122" t="n">
+        <v>8</v>
+      </c>
+      <c r="C10" s="80" t="inlineStr">
+        <is>
+          <t>① 経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D10" s="80" t="inlineStr">
+        <is>
+          <t>コンサルタント来社・業務改善検討
+糸ぐち　午後の部　進行中</t>
+        </is>
+      </c>
+      <c r="E10" s="122" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="F10" s="122" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G9" s="118" t="inlineStr">
+      <c r="G10" s="122" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1">
-      <c r="B11" s="52" t="inlineStr">
+    <row r="12" ht="20" customHeight="1">
+      <c r="B12" s="52" t="inlineStr">
         <is>
           <t>カテゴリ別集計</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1">
-      <c r="B12" s="122" t="inlineStr">
+    <row r="13" ht="18" customHeight="1">
+      <c r="B13" s="122" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C12" s="80" t="inlineStr">
+      <c r="C13" s="80" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D12" s="80" t="inlineStr"/>
-      <c r="E12" s="122" t="inlineStr"/>
-      <c r="F12" s="122" t="inlineStr"/>
-      <c r="G12" s="122" t="inlineStr">
-        <is>
-          <t>115分 (46.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1">
-      <c r="B13" s="119" t="inlineStr">
+      <c r="D13" s="80" t="inlineStr"/>
+      <c r="E13" s="122" t="inlineStr"/>
+      <c r="F13" s="122" t="inlineStr"/>
+      <c r="G13" s="122" t="inlineStr">
+        <is>
+          <t>115分 (40.6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1">
+      <c r="B14" s="119" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C13" s="81" t="inlineStr">
+      <c r="C14" s="81" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D13" s="81" t="inlineStr"/>
-      <c r="E13" s="119" t="inlineStr"/>
-      <c r="F13" s="119" t="inlineStr"/>
-      <c r="G13" s="119" t="inlineStr">
-        <is>
-          <t>115分 (46.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1">
-      <c r="B14" s="120" t="inlineStr">
+      <c r="D14" s="81" t="inlineStr"/>
+      <c r="E14" s="119" t="inlineStr"/>
+      <c r="F14" s="119" t="inlineStr"/>
+      <c r="G14" s="119" t="inlineStr">
+        <is>
+          <t>115分 (40.6%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1">
+      <c r="B15" s="120" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C14" s="82" t="inlineStr">
+      <c r="C15" s="82" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D14" s="82" t="inlineStr"/>
-      <c r="E14" s="120" t="inlineStr"/>
-      <c r="F14" s="120" t="inlineStr"/>
-      <c r="G14" s="120" t="inlineStr">
-        <is>
-          <t>7分 (2.8%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1">
-      <c r="B15" s="123" t="inlineStr">
+      <c r="D15" s="82" t="inlineStr"/>
+      <c r="E15" s="120" t="inlineStr"/>
+      <c r="F15" s="120" t="inlineStr"/>
+      <c r="G15" s="120" t="inlineStr">
+        <is>
+          <t>7分 (2.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1">
+      <c r="B16" s="123" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C15" s="83" t="inlineStr">
+      <c r="C16" s="83" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D15" s="83" t="inlineStr"/>
-      <c r="E15" s="123" t="inlineStr"/>
-      <c r="F15" s="123" t="inlineStr"/>
-      <c r="G15" s="123" t="inlineStr">
+      <c r="D16" s="83" t="inlineStr"/>
+      <c r="E16" s="123" t="inlineStr"/>
+      <c r="F16" s="123" t="inlineStr"/>
+      <c r="G16" s="123" t="inlineStr">
         <is>
           <t>0分 (0.0%)</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1">
-      <c r="B16" s="121" t="inlineStr">
+    <row r="17" ht="18" customHeight="1">
+      <c r="B17" s="121" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C16" s="84" t="inlineStr">
+      <c r="C17" s="84" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D16" s="84" t="inlineStr"/>
-      <c r="E16" s="121" t="inlineStr"/>
-      <c r="F16" s="121" t="inlineStr"/>
-      <c r="G16" s="121" t="inlineStr">
-        <is>
-          <t>10分 (4.0%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1">
-      <c r="B17" s="118" t="inlineStr">
+      <c r="D17" s="84" t="inlineStr"/>
+      <c r="E17" s="121" t="inlineStr"/>
+      <c r="F17" s="121" t="inlineStr"/>
+      <c r="G17" s="121" t="inlineStr">
+        <is>
+          <t>10分 (3.5%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1">
+      <c r="B18" s="118" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C17" s="85" t="inlineStr">
+      <c r="C18" s="85" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D17" s="85" t="inlineStr"/>
-      <c r="E17" s="118" t="inlineStr"/>
-      <c r="F17" s="118" t="inlineStr"/>
-      <c r="G17" s="118" t="inlineStr">
-        <is>
-          <t>3分 (1.2%)</t>
-        </is>
-      </c>
-    </row>
-    <row r="18" ht="20" customHeight="1">
-      <c r="B18" s="124" t="inlineStr">
+      <c r="D18" s="85" t="inlineStr"/>
+      <c r="E18" s="118" t="inlineStr"/>
+      <c r="F18" s="118" t="inlineStr"/>
+      <c r="G18" s="118" t="inlineStr">
+        <is>
+          <t>36分 (12.7%)</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="20" customHeight="1">
+      <c r="B19" s="124" t="inlineStr">
         <is>
           <t>記録済み合計</t>
         </is>
       </c>
-      <c r="G18" s="52" t="inlineStr">
-        <is>
-          <t>250分 (4時間10分)</t>
+      <c r="G19" s="52" t="inlineStr">
+        <is>
+          <t>283分 (4時間43分)</t>
         </is>
       </c>
     </row>
   </sheetData>
   <mergeCells count="3">
-    <mergeCell ref="B18:F18"/>
-    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B19:F19"/>
+    <mergeCell ref="B12:G12"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Complete 2026-05-26 daily record (end 19:03)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -476,7 +476,7 @@
       </patternFill>
     </fill>
   </fills>
-  <borders count="13">
+  <borders count="17">
     <border>
       <left/>
       <right/>
@@ -610,6 +610,34 @@
       <right style="thin"/>
       <top style="thin"/>
       <bottom style="thin"/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
+    </border>
+    <border>
+      <left/>
+      <right style="thin"/>
+      <top style="thin"/>
+      <bottom style="thin"/>
+      <diagonal/>
     </border>
   </borders>
   <cellStyleXfs count="1">
@@ -10529,7 +10557,7 @@
       </c>
       <c r="D11" s="87" t="inlineStr">
         <is>
-          <t>事務作業（資料作成・事務作業）</t>
+          <t>事務作業（メールチェック・返信・見積もり）</t>
         </is>
       </c>
       <c r="E11" s="86" t="inlineStr">
@@ -10539,13 +10567,11 @@
       </c>
       <c r="F11" s="86" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G11" s="86" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+          <t>19:03</t>
+        </is>
+      </c>
+      <c r="G11" s="86" t="n">
+        <v>168</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" s="64">
@@ -10601,7 +10627,7 @@
         <v>5.5</v>
       </c>
       <c r="F15" s="88" t="n">
-        <v>66.09999999999999</v>
+        <v>49.3</v>
       </c>
       <c r="G15" s="88" t="n"/>
     </row>
@@ -10623,7 +10649,7 @@
         <v>1.9</v>
       </c>
       <c r="F16" s="82" t="n">
-        <v>23.2</v>
+        <v>17.3</v>
       </c>
       <c r="G16" s="82" t="n"/>
     </row>
@@ -10645,7 +10671,7 @@
         <v>0.1</v>
       </c>
       <c r="F17" s="84" t="n">
-        <v>1.4</v>
+        <v>1.1</v>
       </c>
       <c r="G17" s="84" t="n"/>
     </row>
@@ -10683,13 +10709,13 @@
         </is>
       </c>
       <c r="D19" s="86" t="n">
-        <v>10</v>
+        <v>178</v>
       </c>
       <c r="E19" s="86" t="n">
-        <v>0.2</v>
+        <v>3</v>
       </c>
       <c r="F19" s="86" t="n">
-        <v>2</v>
+        <v>26.8</v>
       </c>
       <c r="G19" s="86" t="n"/>
     </row>
@@ -10711,7 +10737,7 @@
         <v>0.6</v>
       </c>
       <c r="F20" s="80" t="n">
-        <v>7.3</v>
+        <v>5.4</v>
       </c>
       <c r="G20" s="80" t="n"/>
     </row>
@@ -10723,10 +10749,10 @@
       </c>
       <c r="C21" s="90" t="n"/>
       <c r="D21" s="79" t="n">
-        <v>495</v>
+        <v>663</v>
       </c>
       <c r="E21" s="79" t="n">
-        <v>8.199999999999999</v>
+        <v>11.1</v>
       </c>
       <c r="F21" s="79" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add daily task record for 2026-05-27 (作業中)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -18,14 +18,15 @@
     <sheet name="2026-05-22" sheetId="10" state="visible" r:id="rId10"/>
     <sheet name="2026-05-25" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-05-26" sheetId="12" state="visible" r:id="rId12"/>
+    <sheet name="2026-05-27" sheetId="13" state="visible" r:id="rId13"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId13"/>
     <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
+    <externalReference r:id="rId19"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -643,7 +644,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="93">
+  <cellXfs count="95">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -869,6 +870,8 @@
     <xf numFmtId="0" fontId="26" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -10271,6 +10274,11 @@
           <t>2026年5月26日（火）　業務記録</t>
         </is>
       </c>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="94" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1" s="64">
       <c r="B2" s="79" t="inlineStr">
@@ -10580,6 +10588,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C13" s="93" t="n"/>
+      <c r="D13" s="93" t="n"/>
+      <c r="E13" s="93" t="n"/>
+      <c r="F13" s="93" t="n"/>
+      <c r="G13" s="94" t="n"/>
     </row>
     <row r="14" ht="18" customHeight="1" s="64">
       <c r="B14" s="79" t="inlineStr">
@@ -10762,6 +10775,499 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet13.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="64" min="1" max="1"/>
+    <col width="6" customWidth="1" style="64" min="2" max="2"/>
+    <col width="20" customWidth="1" style="64" min="3" max="3"/>
+    <col width="44" customWidth="1" style="64" min="4" max="4"/>
+    <col width="8" customWidth="1" style="64" min="5" max="5"/>
+    <col width="8" customWidth="1" style="64" min="6" max="6"/>
+    <col width="14" customWidth="1" style="64" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" s="64">
+      <c r="B1" s="78" t="inlineStr">
+        <is>
+          <t>2026年5月27日（水）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="64">
+      <c r="B2" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C2" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D2" s="79" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E2" s="79" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F2" s="79" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G2" s="79" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="64">
+      <c r="B3" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C3" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D3" s="81" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E3" s="80" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F3" s="80" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G3" s="80" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="64">
+      <c r="B4" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C4" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D4" s="83" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E4" s="82" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F4" s="82" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G4" s="82" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="64">
+      <c r="B5" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C5" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D5" s="85" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E5" s="84" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F5" s="84" t="inlineStr">
+        <is>
+          <t>8:25</t>
+        </is>
+      </c>
+      <c r="G5" s="84" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="64">
+      <c r="B6" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C6" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D6" s="87" t="inlineStr">
+        <is>
+          <t>メールチェック・返信</t>
+        </is>
+      </c>
+      <c r="E6" s="86" t="inlineStr">
+        <is>
+          <t>8:25</t>
+        </is>
+      </c>
+      <c r="F6" s="86" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="G6" s="86" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C7" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D7" s="87" t="inlineStr">
+        <is>
+          <t>見積もり作成</t>
+        </is>
+      </c>
+      <c r="E7" s="86" t="inlineStr">
+        <is>
+          <t>8:40</t>
+        </is>
+      </c>
+      <c r="F7" s="86" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G7" s="86" t="n">
+        <v>90</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C8" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D8" s="83" t="inlineStr">
+        <is>
+          <t>改善提案委員会（社内会議）</t>
+        </is>
+      </c>
+      <c r="E8" s="82" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F8" s="82" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="G8" s="82" t="n">
+        <v>115</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C9" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D9" s="81" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E9" s="80" t="inlineStr">
+        <is>
+          <t>12:05</t>
+        </is>
+      </c>
+      <c r="F9" s="80" t="inlineStr">
+        <is>
+          <t>12:22</t>
+        </is>
+      </c>
+      <c r="G9" s="80" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C10" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D10" s="89" t="inlineStr">
+        <is>
+          <t>客先への見積もり提出・見積もり作成</t>
+        </is>
+      </c>
+      <c r="E10" s="88" t="inlineStr">
+        <is>
+          <t>12:22</t>
+        </is>
+      </c>
+      <c r="F10" s="88" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G10" s="88" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="20" customHeight="1" s="64">
+      <c r="B12" s="90" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C13" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D13" s="79" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E13" s="79" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F13" s="79" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G13" s="79" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C14" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D14" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" s="88" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C15" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D15" s="82" t="n">
+        <v>118</v>
+      </c>
+      <c r="E15" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="F15" s="82" t="n">
+        <v>45</v>
+      </c>
+      <c r="G15" s="82" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C16" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D16" s="84" t="n">
+        <v>19</v>
+      </c>
+      <c r="E16" s="84" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F16" s="84" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="G16" s="84" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C17" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D17" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="91" t="n"/>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C18" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D18" s="86" t="n">
+        <v>105</v>
+      </c>
+      <c r="E18" s="86" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F18" s="86" t="n">
+        <v>40.1</v>
+      </c>
+      <c r="G18" s="86" t="n"/>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C19" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D19" s="80" t="n">
+        <v>20</v>
+      </c>
+      <c r="E19" s="80" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F19" s="80" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="G19" s="80" t="n"/>
+    </row>
+    <row r="20" ht="20" customHeight="1" s="64">
+      <c r="B20" s="79" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C20" s="90" t="n"/>
+      <c r="D20" s="79" t="n">
+        <v>262</v>
+      </c>
+      <c r="E20" s="79" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F20" s="79" t="n">
+        <v>100</v>
+      </c>
+      <c r="G20" s="79" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B12:G12"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-27: add afternoon break
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -10787,7 +10787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G20"/>
+  <dimension ref="B1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11071,203 +11071,233 @@
       </c>
       <c r="F10" s="88" t="inlineStr">
         <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="G10" s="88" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="81" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E11" s="80" t="inlineStr">
+        <is>
+          <t>12:31</t>
+        </is>
+      </c>
+      <c r="F11" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G10" s="88" t="inlineStr">
+      <c r="G11" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1" s="64">
-      <c r="B12" s="90" t="inlineStr">
+    <row r="13" ht="20" customHeight="1" s="64">
+      <c r="B13" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" s="64">
-      <c r="B13" s="79" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C13" s="79" t="inlineStr">
+      <c r="C14" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D13" s="79" t="inlineStr">
+      <c r="D14" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E13" s="79" t="inlineStr">
+      <c r="E14" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F13" s="79" t="inlineStr">
+      <c r="F14" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G13" s="79" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="88" t="inlineStr">
+      <c r="G14" s="79" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C14" s="89" t="inlineStr">
+      <c r="C15" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D14" s="88" t="n">
+      <c r="D15" s="88" t="n">
+        <v>9</v>
+      </c>
+      <c r="E15" s="88" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F15" s="88" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="G15" s="88" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C16" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D16" s="82" t="n">
+        <v>118</v>
+      </c>
+      <c r="E16" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="F16" s="82" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G16" s="82" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C17" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D17" s="84" t="n">
+        <v>19</v>
+      </c>
+      <c r="E17" s="84" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F17" s="84" t="n">
+        <v>7</v>
+      </c>
+      <c r="G17" s="84" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C18" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D18" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="88" t="n">
+      <c r="E18" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="88" t="n">
+      <c r="F18" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="88" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="82" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
-      <c r="C15" s="83" t="inlineStr">
-        <is>
-          <t>社内マネジメント</t>
-        </is>
-      </c>
-      <c r="D15" s="82" t="n">
-        <v>118</v>
-      </c>
-      <c r="E15" s="82" t="n">
-        <v>2</v>
-      </c>
-      <c r="F15" s="82" t="n">
-        <v>45</v>
-      </c>
-      <c r="G15" s="82" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="84" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C16" s="85" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D16" s="84" t="n">
-        <v>19</v>
-      </c>
-      <c r="E16" s="84" t="n">
+      <c r="G18" s="91" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="86" t="n">
+        <v>105</v>
+      </c>
+      <c r="E19" s="86" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F19" s="86" t="n">
+        <v>38.7</v>
+      </c>
+      <c r="G19" s="86" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C20" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D20" s="80" t="n">
+        <v>20</v>
+      </c>
+      <c r="E20" s="80" t="n">
         <v>0.3</v>
       </c>
-      <c r="F16" s="84" t="n">
-        <v>7.3</v>
-      </c>
-      <c r="G16" s="84" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1" s="64">
-      <c r="B17" s="91" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C17" s="92" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D17" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="E17" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F17" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G17" s="91" t="n"/>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="64">
-      <c r="B18" s="86" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C18" s="87" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D18" s="86" t="n">
-        <v>105</v>
-      </c>
-      <c r="E18" s="86" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F18" s="86" t="n">
-        <v>40.1</v>
-      </c>
-      <c r="G18" s="86" t="n"/>
-    </row>
-    <row r="19" ht="18" customHeight="1" s="64">
-      <c r="B19" s="80" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="C19" s="81" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D19" s="80" t="n">
-        <v>20</v>
-      </c>
-      <c r="E19" s="80" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F19" s="80" t="n">
-        <v>7.6</v>
-      </c>
-      <c r="G19" s="80" t="n"/>
-    </row>
-    <row r="20" ht="20" customHeight="1" s="64">
-      <c r="B20" s="79" t="inlineStr">
+      <c r="F20" s="80" t="n">
+        <v>7.4</v>
+      </c>
+      <c r="G20" s="80" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C20" s="90" t="n"/>
-      <c r="D20" s="79" t="n">
-        <v>262</v>
-      </c>
-      <c r="E20" s="79" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F20" s="79" t="n">
+      <c r="C21" s="90" t="n"/>
+      <c r="D21" s="79" t="n">
+        <v>271</v>
+      </c>
+      <c r="E21" s="79" t="n">
+        <v>4.5</v>
+      </c>
+      <c r="F21" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G20" s="79" t="n"/>
+      <c r="G21" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:G13"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-27: add cleaning and floor patrol
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -10787,7 +10787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G21"/>
+  <dimension ref="B1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11101,203 +11101,263 @@
       </c>
       <c r="F11" s="80" t="inlineStr">
         <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="G11" s="80" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="81" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E12" s="80" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F12" s="80" t="inlineStr">
+        <is>
+          <t>12:51</t>
+        </is>
+      </c>
+      <c r="G12" s="80" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C13" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D13" s="85" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E13" s="84" t="inlineStr">
+        <is>
+          <t>12:51</t>
+        </is>
+      </c>
+      <c r="F13" s="84" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G11" s="80" t="inlineStr">
+      <c r="G13" s="84" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1" s="64">
-      <c r="B13" s="90" t="inlineStr">
+    <row r="15" ht="20" customHeight="1" s="64">
+      <c r="B15" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="79" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C14" s="79" t="inlineStr">
+      <c r="C16" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D14" s="79" t="inlineStr">
+      <c r="D16" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E14" s="79" t="inlineStr">
+      <c r="E16" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F14" s="79" t="inlineStr">
+      <c r="F16" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G14" s="79" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="88" t="inlineStr">
+      <c r="G16" s="79" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C15" s="89" t="inlineStr">
+      <c r="C17" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D15" s="88" t="n">
+      <c r="D17" s="88" t="n">
         <v>9</v>
       </c>
-      <c r="E15" s="88" t="n">
+      <c r="E17" s="88" t="n">
         <v>0.1</v>
       </c>
-      <c r="F15" s="88" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="G15" s="88" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="82" t="inlineStr">
+      <c r="F17" s="88" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="G17" s="88" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C16" s="83" t="inlineStr">
+      <c r="C18" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D16" s="82" t="n">
+      <c r="D18" s="82" t="n">
         <v>118</v>
       </c>
-      <c r="E16" s="82" t="n">
+      <c r="E18" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="F16" s="82" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="G16" s="82" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="84" t="inlineStr">
+      <c r="F18" s="82" t="n">
+        <v>40.5</v>
+      </c>
+      <c r="G18" s="82" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C17" s="85" t="inlineStr">
+      <c r="C19" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D17" s="84" t="n">
+      <c r="D19" s="84" t="n">
         <v>19</v>
       </c>
-      <c r="E17" s="84" t="n">
+      <c r="E19" s="84" t="n">
         <v>0.3</v>
       </c>
-      <c r="F17" s="84" t="n">
-        <v>7</v>
-      </c>
-      <c r="G17" s="84" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="91" t="inlineStr">
+      <c r="F19" s="84" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="G19" s="84" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C18" s="92" t="inlineStr">
+      <c r="C20" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D18" s="91" t="n">
+      <c r="D20" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="91" t="n">
+      <c r="E20" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="91" t="n">
+      <c r="F20" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="91" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="86" t="inlineStr">
+      <c r="G20" s="91" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C19" s="87" t="inlineStr">
+      <c r="C21" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D19" s="86" t="n">
+      <c r="D21" s="86" t="n">
         <v>105</v>
       </c>
-      <c r="E19" s="86" t="n">
+      <c r="E21" s="86" t="n">
         <v>1.8</v>
       </c>
-      <c r="F19" s="86" t="n">
-        <v>38.7</v>
-      </c>
-      <c r="G19" s="86" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="80" t="inlineStr">
+      <c r="F21" s="86" t="n">
+        <v>36.1</v>
+      </c>
+      <c r="G21" s="86" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C20" s="81" t="inlineStr">
+      <c r="C22" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D20" s="80" t="n">
-        <v>20</v>
-      </c>
-      <c r="E20" s="80" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F20" s="80" t="n">
-        <v>7.4</v>
-      </c>
-      <c r="G20" s="80" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="79" t="inlineStr">
+      <c r="D22" s="80" t="n">
+        <v>40</v>
+      </c>
+      <c r="E22" s="80" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F22" s="80" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G22" s="80" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C21" s="90" t="n"/>
-      <c r="D21" s="79" t="n">
-        <v>271</v>
-      </c>
-      <c r="E21" s="79" t="n">
-        <v>4.5</v>
-      </c>
-      <c r="F21" s="79" t="n">
+      <c r="C23" s="90" t="n"/>
+      <c r="D23" s="79" t="n">
+        <v>291</v>
+      </c>
+      <c r="E23" s="79" t="n">
+        <v>4.8</v>
+      </c>
+      <c r="F23" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G21" s="79" t="n"/>
+      <c r="G23" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B15:G15"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-27: close floor patrol, start email check
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -10787,7 +10787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G23"/>
+  <dimension ref="B1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11161,203 +11161,233 @@
       </c>
       <c r="F13" s="84" t="inlineStr">
         <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="G13" s="84" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C14" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D14" s="87" t="inlineStr">
+        <is>
+          <t>メールチェック</t>
+        </is>
+      </c>
+      <c r="E14" s="86" t="inlineStr">
+        <is>
+          <t>13:22</t>
+        </is>
+      </c>
+      <c r="F14" s="86" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G13" s="84" t="inlineStr">
+      <c r="G14" s="86" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1" s="64">
-      <c r="B15" s="90" t="inlineStr">
+    <row r="16" ht="20" customHeight="1" s="64">
+      <c r="B16" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="79" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C16" s="79" t="inlineStr">
+      <c r="C17" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D16" s="79" t="inlineStr">
+      <c r="D17" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E16" s="79" t="inlineStr">
+      <c r="E17" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F16" s="79" t="inlineStr">
+      <c r="F17" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G16" s="79" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="88" t="inlineStr">
+      <c r="G17" s="79" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C17" s="89" t="inlineStr">
+      <c r="C18" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D17" s="88" t="n">
+      <c r="D18" s="88" t="n">
         <v>9</v>
       </c>
-      <c r="E17" s="88" t="n">
+      <c r="E18" s="88" t="n">
         <v>0.1</v>
       </c>
-      <c r="F17" s="88" t="n">
-        <v>3.1</v>
-      </c>
-      <c r="G17" s="88" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="82" t="inlineStr">
+      <c r="F18" s="88" t="n">
+        <v>2.8</v>
+      </c>
+      <c r="G18" s="88" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C18" s="83" t="inlineStr">
+      <c r="C19" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D18" s="82" t="n">
+      <c r="D19" s="82" t="n">
         <v>118</v>
       </c>
-      <c r="E18" s="82" t="n">
+      <c r="E19" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="F18" s="82" t="n">
-        <v>40.5</v>
-      </c>
-      <c r="G18" s="82" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="84" t="inlineStr">
+      <c r="F19" s="82" t="n">
+        <v>36.6</v>
+      </c>
+      <c r="G19" s="82" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C19" s="85" t="inlineStr">
+      <c r="C20" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D19" s="84" t="n">
-        <v>19</v>
-      </c>
-      <c r="E19" s="84" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F19" s="84" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="G19" s="84" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="91" t="inlineStr">
+      <c r="D20" s="84" t="n">
+        <v>50</v>
+      </c>
+      <c r="E20" s="84" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F20" s="84" t="n">
+        <v>15.5</v>
+      </c>
+      <c r="G20" s="84" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C20" s="92" t="inlineStr">
+      <c r="C21" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D20" s="91" t="n">
+      <c r="D21" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="91" t="n">
+      <c r="E21" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="91" t="n">
+      <c r="F21" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="91" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="86" t="inlineStr">
+      <c r="G21" s="91" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C21" s="87" t="inlineStr">
+      <c r="C22" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D21" s="86" t="n">
+      <c r="D22" s="86" t="n">
         <v>105</v>
       </c>
-      <c r="E21" s="86" t="n">
+      <c r="E22" s="86" t="n">
         <v>1.8</v>
       </c>
-      <c r="F21" s="86" t="n">
-        <v>36.1</v>
-      </c>
-      <c r="G21" s="86" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="80" t="inlineStr">
+      <c r="F22" s="86" t="n">
+        <v>32.6</v>
+      </c>
+      <c r="G22" s="86" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C22" s="81" t="inlineStr">
+      <c r="C23" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D22" s="80" t="n">
+      <c r="D23" s="80" t="n">
         <v>40</v>
       </c>
-      <c r="E22" s="80" t="n">
+      <c r="E23" s="80" t="n">
         <v>0.7</v>
       </c>
-      <c r="F22" s="80" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="G22" s="80" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="79" t="inlineStr">
+      <c r="F23" s="80" t="n">
+        <v>12.4</v>
+      </c>
+      <c r="G23" s="80" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C23" s="90" t="n"/>
-      <c r="D23" s="79" t="n">
-        <v>291</v>
-      </c>
-      <c r="E23" s="79" t="n">
-        <v>4.8</v>
-      </c>
-      <c r="F23" s="79" t="n">
+      <c r="C24" s="90" t="n"/>
+      <c r="D24" s="79" t="n">
+        <v>322</v>
+      </c>
+      <c r="E24" s="79" t="n">
+        <v>5.4</v>
+      </c>
+      <c r="F24" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G23" s="79" t="n"/>
+      <c r="G24" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B16:G16"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-27: depart for 兵庫県中央会 交流会
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -10787,7 +10787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G24"/>
+  <dimension ref="B1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11191,203 +11191,233 @@
       </c>
       <c r="F14" s="86" t="inlineStr">
         <is>
+          <t>13:48</t>
+        </is>
+      </c>
+      <c r="G14" s="86" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C15" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D15" s="81" t="inlineStr">
+        <is>
+          <t>着替え・移動（兵庫県中央会 交流会へ）</t>
+        </is>
+      </c>
+      <c r="E15" s="80" t="inlineStr">
+        <is>
+          <t>13:48</t>
+        </is>
+      </c>
+      <c r="F15" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G14" s="86" t="inlineStr">
+      <c r="G15" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1" s="64">
-      <c r="B16" s="90" t="inlineStr">
+    <row r="17" ht="20" customHeight="1" s="64">
+      <c r="B17" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="79" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C17" s="79" t="inlineStr">
+      <c r="C18" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D17" s="79" t="inlineStr">
+      <c r="D18" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E17" s="79" t="inlineStr">
+      <c r="E18" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F17" s="79" t="inlineStr">
+      <c r="F18" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G17" s="79" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="88" t="inlineStr">
+      <c r="G18" s="79" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C18" s="89" t="inlineStr">
+      <c r="C19" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D18" s="88" t="n">
+      <c r="D19" s="88" t="n">
         <v>9</v>
       </c>
-      <c r="E18" s="88" t="n">
+      <c r="E19" s="88" t="n">
         <v>0.1</v>
       </c>
-      <c r="F18" s="88" t="n">
-        <v>2.8</v>
-      </c>
-      <c r="G18" s="88" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="82" t="inlineStr">
+      <c r="F19" s="88" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="G19" s="88" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C19" s="83" t="inlineStr">
+      <c r="C20" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D19" s="82" t="n">
+      <c r="D20" s="82" t="n">
         <v>118</v>
       </c>
-      <c r="E19" s="82" t="n">
+      <c r="E20" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="F19" s="82" t="n">
-        <v>36.6</v>
-      </c>
-      <c r="G19" s="82" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="84" t="inlineStr">
+      <c r="F20" s="82" t="n">
+        <v>33.9</v>
+      </c>
+      <c r="G20" s="82" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C20" s="85" t="inlineStr">
+      <c r="C21" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D20" s="84" t="n">
+      <c r="D21" s="84" t="n">
         <v>50</v>
       </c>
-      <c r="E20" s="84" t="n">
+      <c r="E21" s="84" t="n">
         <v>0.8</v>
       </c>
-      <c r="F20" s="84" t="n">
-        <v>15.5</v>
-      </c>
-      <c r="G20" s="84" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="91" t="inlineStr">
+      <c r="F21" s="84" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="G21" s="84" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C21" s="92" t="inlineStr">
+      <c r="C22" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D21" s="91" t="n">
+      <c r="D22" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="91" t="n">
+      <c r="E22" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="91" t="n">
+      <c r="F22" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G21" s="91" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="86" t="inlineStr">
+      <c r="G22" s="91" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C22" s="87" t="inlineStr">
+      <c r="C23" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D22" s="86" t="n">
-        <v>105</v>
-      </c>
-      <c r="E22" s="86" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F22" s="86" t="n">
-        <v>32.6</v>
-      </c>
-      <c r="G22" s="86" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="80" t="inlineStr">
+      <c r="D23" s="86" t="n">
+        <v>131</v>
+      </c>
+      <c r="E23" s="86" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F23" s="86" t="n">
+        <v>37.6</v>
+      </c>
+      <c r="G23" s="86" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C23" s="81" t="inlineStr">
+      <c r="C24" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D23" s="80" t="n">
+      <c r="D24" s="80" t="n">
         <v>40</v>
       </c>
-      <c r="E23" s="80" t="n">
+      <c r="E24" s="80" t="n">
         <v>0.7</v>
       </c>
-      <c r="F23" s="80" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="G23" s="80" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="79" t="inlineStr">
+      <c r="F24" s="80" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G24" s="80" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C24" s="90" t="n"/>
-      <c r="D24" s="79" t="n">
-        <v>322</v>
-      </c>
-      <c r="E24" s="79" t="n">
-        <v>5.4</v>
-      </c>
-      <c r="F24" s="79" t="n">
+      <c r="C25" s="90" t="n"/>
+      <c r="D25" s="79" t="n">
+        <v>348</v>
+      </c>
+      <c r="E25" s="79" t="n">
+        <v>5.8</v>
+      </c>
+      <c r="F25" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G24" s="79" t="n"/>
+      <c r="G25" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B17:G17"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-27: start 兵庫県中央会 総会 at 15:00
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -10787,7 +10787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G25"/>
+  <dimension ref="B1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11221,203 +11221,233 @@
       </c>
       <c r="F15" s="80" t="inlineStr">
         <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="G15" s="80" t="n">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C16" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D16" s="89" t="inlineStr">
+        <is>
+          <t>兵庫県中央会 総会</t>
+        </is>
+      </c>
+      <c r="E16" s="88" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="F16" s="88" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G15" s="80" t="inlineStr">
+      <c r="G16" s="88" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="20" customHeight="1" s="64">
-      <c r="B17" s="90" t="inlineStr">
+    <row r="18" ht="20" customHeight="1" s="64">
+      <c r="B18" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="79" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C18" s="79" t="inlineStr">
+      <c r="C19" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D18" s="79" t="inlineStr">
+      <c r="D19" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E18" s="79" t="inlineStr">
+      <c r="E19" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F18" s="79" t="inlineStr">
+      <c r="F19" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G18" s="79" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="88" t="inlineStr">
+      <c r="G19" s="79" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C19" s="89" t="inlineStr">
+      <c r="C20" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D19" s="88" t="n">
+      <c r="D20" s="88" t="n">
         <v>9</v>
       </c>
-      <c r="E19" s="88" t="n">
+      <c r="E20" s="88" t="n">
         <v>0.1</v>
       </c>
-      <c r="F19" s="88" t="n">
-        <v>2.6</v>
-      </c>
-      <c r="G19" s="88" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="82" t="inlineStr">
+      <c r="F20" s="88" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="G20" s="88" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C20" s="83" t="inlineStr">
+      <c r="C21" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D20" s="82" t="n">
+      <c r="D21" s="82" t="n">
         <v>118</v>
       </c>
-      <c r="E20" s="82" t="n">
+      <c r="E21" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="F20" s="82" t="n">
-        <v>33.9</v>
-      </c>
-      <c r="G20" s="82" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="84" t="inlineStr">
+      <c r="F21" s="82" t="n">
+        <v>28.1</v>
+      </c>
+      <c r="G21" s="82" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C21" s="85" t="inlineStr">
+      <c r="C22" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D21" s="84" t="n">
+      <c r="D22" s="84" t="n">
         <v>50</v>
       </c>
-      <c r="E21" s="84" t="n">
+      <c r="E22" s="84" t="n">
         <v>0.8</v>
       </c>
-      <c r="F21" s="84" t="n">
-        <v>14.4</v>
-      </c>
-      <c r="G21" s="84" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="91" t="inlineStr">
+      <c r="F22" s="84" t="n">
+        <v>11.9</v>
+      </c>
+      <c r="G22" s="84" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C22" s="92" t="inlineStr">
+      <c r="C23" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D22" s="91" t="n">
+      <c r="D23" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E22" s="91" t="n">
+      <c r="E23" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F22" s="91" t="n">
+      <c r="F23" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G22" s="91" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="86" t="inlineStr">
+      <c r="G23" s="91" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C23" s="87" t="inlineStr">
+      <c r="C24" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D23" s="86" t="n">
+      <c r="D24" s="86" t="n">
         <v>131</v>
       </c>
-      <c r="E23" s="86" t="n">
+      <c r="E24" s="86" t="n">
         <v>2.2</v>
       </c>
-      <c r="F23" s="86" t="n">
-        <v>37.6</v>
-      </c>
-      <c r="G23" s="86" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="80" t="inlineStr">
+      <c r="F24" s="86" t="n">
+        <v>31.2</v>
+      </c>
+      <c r="G24" s="86" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C24" s="81" t="inlineStr">
+      <c r="C25" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D24" s="80" t="n">
-        <v>40</v>
-      </c>
-      <c r="E24" s="80" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F24" s="80" t="n">
-        <v>11.5</v>
-      </c>
-      <c r="G24" s="80" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="79" t="inlineStr">
+      <c r="D25" s="80" t="n">
+        <v>112</v>
+      </c>
+      <c r="E25" s="80" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F25" s="80" t="n">
+        <v>26.7</v>
+      </c>
+      <c r="G25" s="80" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C25" s="90" t="n"/>
-      <c r="D25" s="79" t="n">
-        <v>348</v>
-      </c>
-      <c r="E25" s="79" t="n">
-        <v>5.8</v>
-      </c>
-      <c r="F25" s="79" t="n">
+      <c r="C26" s="90" t="n"/>
+      <c r="D26" s="79" t="n">
+        <v>420</v>
+      </c>
+      <c r="E26" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G25" s="79" t="n"/>
+      <c r="G26" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B17:G17"/>
+    <mergeCell ref="B18:G18"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-27: add partner company phone calls during travel
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -10787,7 +10787,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G26"/>
+  <dimension ref="B1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11221,11 +11221,11 @@
       </c>
       <c r="F15" s="80" t="inlineStr">
         <is>
-          <t>15:00</t>
+          <t>14:20</t>
         </is>
       </c>
       <c r="G15" s="80" t="n">
-        <v>72</v>
+        <v>32</v>
       </c>
     </row>
     <row r="16" ht="18" customHeight="1" s="64">
@@ -11241,213 +11241,333 @@
       </c>
       <c r="D16" s="89" t="inlineStr">
         <is>
+          <t>協力会社 電話対応</t>
+        </is>
+      </c>
+      <c r="E16" s="88" t="inlineStr">
+        <is>
+          <t>14:20</t>
+        </is>
+      </c>
+      <c r="F16" s="88" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="G16" s="88" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C17" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D17" s="81" t="inlineStr">
+        <is>
+          <t>移動・待機</t>
+        </is>
+      </c>
+      <c r="E17" s="80" t="inlineStr">
+        <is>
+          <t>14:32</t>
+        </is>
+      </c>
+      <c r="F17" s="80" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="G17" s="80" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C18" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D18" s="89" t="inlineStr">
+        <is>
+          <t>協力会社 電話対応</t>
+        </is>
+      </c>
+      <c r="E18" s="88" t="inlineStr">
+        <is>
+          <t>14:46</t>
+        </is>
+      </c>
+      <c r="F18" s="88" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="G18" s="88" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C19" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D19" s="81" t="inlineStr">
+        <is>
+          <t>移動・待機</t>
+        </is>
+      </c>
+      <c r="E19" s="80" t="inlineStr">
+        <is>
+          <t>14:48</t>
+        </is>
+      </c>
+      <c r="F19" s="80" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="G19" s="80" t="n">
+        <v>12</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C20" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D20" s="89" t="inlineStr">
+        <is>
           <t>兵庫県中央会 総会</t>
         </is>
       </c>
-      <c r="E16" s="88" t="inlineStr">
+      <c r="E20" s="88" t="inlineStr">
         <is>
           <t>15:00</t>
         </is>
       </c>
-      <c r="F16" s="88" t="inlineStr">
+      <c r="F20" s="88" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G16" s="88" t="inlineStr">
+      <c r="G20" s="88" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1" s="64">
-      <c r="B18" s="90" t="inlineStr">
+    <row r="22" ht="20" customHeight="1" s="64">
+      <c r="B22" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="79" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C19" s="79" t="inlineStr">
+      <c r="C23" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D19" s="79" t="inlineStr">
+      <c r="D23" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E19" s="79" t="inlineStr">
+      <c r="E23" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F19" s="79" t="inlineStr">
+      <c r="F23" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G19" s="79" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="88" t="inlineStr">
+      <c r="G23" s="79" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C20" s="89" t="inlineStr">
+      <c r="C24" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D20" s="88" t="n">
-        <v>9</v>
-      </c>
-      <c r="E20" s="88" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F20" s="88" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="G20" s="88" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="82" t="inlineStr">
+      <c r="D24" s="88" t="n">
+        <v>23</v>
+      </c>
+      <c r="E24" s="88" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F24" s="88" t="n">
+        <v>5.5</v>
+      </c>
+      <c r="G24" s="88" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C21" s="83" t="inlineStr">
+      <c r="C25" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D21" s="82" t="n">
+      <c r="D25" s="82" t="n">
         <v>118</v>
       </c>
-      <c r="E21" s="82" t="n">
+      <c r="E25" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="F21" s="82" t="n">
+      <c r="F25" s="82" t="n">
         <v>28.1</v>
       </c>
-      <c r="G21" s="82" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="84" t="inlineStr">
+      <c r="G25" s="82" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C22" s="85" t="inlineStr">
+      <c r="C26" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D22" s="84" t="n">
+      <c r="D26" s="84" t="n">
         <v>50</v>
       </c>
-      <c r="E22" s="84" t="n">
+      <c r="E26" s="84" t="n">
         <v>0.8</v>
       </c>
-      <c r="F22" s="84" t="n">
+      <c r="F26" s="84" t="n">
         <v>11.9</v>
       </c>
-      <c r="G22" s="84" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="91" t="inlineStr">
+      <c r="G26" s="84" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C23" s="92" t="inlineStr">
+      <c r="C27" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D23" s="91" t="n">
+      <c r="D27" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="91" t="n">
+      <c r="E27" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="91" t="n">
+      <c r="F27" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="91" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="86" t="inlineStr">
+      <c r="G27" s="91" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C24" s="87" t="inlineStr">
+      <c r="C28" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D24" s="86" t="n">
+      <c r="D28" s="86" t="n">
         <v>131</v>
       </c>
-      <c r="E24" s="86" t="n">
+      <c r="E28" s="86" t="n">
         <v>2.2</v>
       </c>
-      <c r="F24" s="86" t="n">
+      <c r="F28" s="86" t="n">
         <v>31.2</v>
       </c>
-      <c r="G24" s="86" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="80" t="inlineStr">
+      <c r="G28" s="86" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C25" s="81" t="inlineStr">
+      <c r="C29" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D25" s="80" t="n">
-        <v>112</v>
-      </c>
-      <c r="E25" s="80" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="F25" s="80" t="n">
-        <v>26.7</v>
-      </c>
-      <c r="G25" s="80" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="79" t="inlineStr">
+      <c r="D29" s="80" t="n">
+        <v>98</v>
+      </c>
+      <c r="E29" s="80" t="n">
+        <v>1.6</v>
+      </c>
+      <c r="F29" s="80" t="n">
+        <v>23.3</v>
+      </c>
+      <c r="G29" s="80" t="n"/>
+    </row>
+    <row r="30">
+      <c r="B30" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C26" s="90" t="n"/>
-      <c r="D26" s="79" t="n">
+      <c r="C30" s="90" t="n"/>
+      <c r="D30" s="79" t="n">
         <v>420</v>
       </c>
-      <c r="E26" s="79" t="n">
+      <c r="E30" s="79" t="n">
         <v>7</v>
       </c>
-      <c r="F26" s="79" t="n">
+      <c r="F30" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G26" s="79" t="n"/>
+      <c r="G30" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B22:G22"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Complete 2026-05-27 daily record (end 20:20)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11361,7 +11361,7 @@
       </c>
       <c r="D20" s="89" t="inlineStr">
         <is>
-          <t>兵庫県中央会 総会</t>
+          <t>兵庫県中央会 総会・交流会</t>
         </is>
       </c>
       <c r="E20" s="88" t="inlineStr">
@@ -11371,13 +11371,11 @@
       </c>
       <c r="F20" s="88" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G20" s="88" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+          <t>20:20</t>
+        </is>
+      </c>
+      <c r="G20" s="88" t="n">
+        <v>320</v>
       </c>
     </row>
     <row r="22" ht="20" customHeight="1" s="64">
@@ -11427,13 +11425,13 @@
         </is>
       </c>
       <c r="D24" s="88" t="n">
-        <v>23</v>
+        <v>343</v>
       </c>
       <c r="E24" s="88" t="n">
-        <v>0.4</v>
+        <v>5.7</v>
       </c>
       <c r="F24" s="88" t="n">
-        <v>5.5</v>
+        <v>46.4</v>
       </c>
       <c r="G24" s="88" t="n"/>
     </row>
@@ -11455,7 +11453,7 @@
         <v>2</v>
       </c>
       <c r="F25" s="82" t="n">
-        <v>28.1</v>
+        <v>15.9</v>
       </c>
       <c r="G25" s="82" t="n"/>
     </row>
@@ -11477,7 +11475,7 @@
         <v>0.8</v>
       </c>
       <c r="F26" s="84" t="n">
-        <v>11.9</v>
+        <v>6.8</v>
       </c>
       <c r="G26" s="84" t="n"/>
     </row>
@@ -11521,7 +11519,7 @@
         <v>2.2</v>
       </c>
       <c r="F28" s="86" t="n">
-        <v>31.2</v>
+        <v>17.7</v>
       </c>
       <c r="G28" s="86" t="n"/>
     </row>
@@ -11543,7 +11541,7 @@
         <v>1.6</v>
       </c>
       <c r="F29" s="80" t="n">
-        <v>23.3</v>
+        <v>13.2</v>
       </c>
       <c r="G29" s="80" t="n"/>
     </row>
@@ -11555,10 +11553,10 @@
       </c>
       <c r="C30" s="90" t="n"/>
       <c r="D30" s="79" t="n">
-        <v>420</v>
+        <v>740</v>
       </c>
       <c r="E30" s="79" t="n">
-        <v>7</v>
+        <v>12.3</v>
       </c>
       <c r="F30" s="79" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add daily task record for 2026-05-28 (作業中)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -19,14 +19,15 @@
     <sheet name="2026-05-25" sheetId="11" state="visible" r:id="rId11"/>
     <sheet name="2026-05-26" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-05-27" sheetId="13" state="visible" r:id="rId13"/>
+    <sheet name="2026-05-28" sheetId="14" state="visible" r:id="rId14"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId14"/>
     <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
     <externalReference r:id="rId19"/>
+    <externalReference r:id="rId20"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -10805,6 +10806,11 @@
           <t>2026年5月27日（水）　業務記録</t>
         </is>
       </c>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="94" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1" s="64">
       <c r="B2" s="79" t="inlineStr">
@@ -11384,6 +11390,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C22" s="93" t="n"/>
+      <c r="D22" s="93" t="n"/>
+      <c r="E22" s="93" t="n"/>
+      <c r="F22" s="93" t="n"/>
+      <c r="G22" s="94" t="n"/>
     </row>
     <row r="23">
       <c r="B23" s="79" t="inlineStr">
@@ -11566,6 +11577,289 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B22:G22"/>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet14.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G13"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="64" min="1" max="1"/>
+    <col width="6" customWidth="1" style="64" min="2" max="2"/>
+    <col width="20" customWidth="1" style="64" min="3" max="3"/>
+    <col width="44" customWidth="1" style="64" min="4" max="4"/>
+    <col width="8" customWidth="1" style="64" min="5" max="5"/>
+    <col width="8" customWidth="1" style="64" min="6" max="6"/>
+    <col width="14" customWidth="1" style="64" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" s="64">
+      <c r="B1" s="78" t="inlineStr">
+        <is>
+          <t>2026年5月28日（木）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="64">
+      <c r="B2" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C2" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D2" s="79" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E2" s="79" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F2" s="79" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G2" s="79" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="64">
+      <c r="B3" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C3" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D3" s="87" t="inlineStr">
+        <is>
+          <t>事務作業</t>
+        </is>
+      </c>
+      <c r="E3" s="86" t="inlineStr">
+        <is>
+          <t>7:36</t>
+        </is>
+      </c>
+      <c r="F3" s="86" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G3" s="86" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" ht="20" customHeight="1" s="64">
+      <c r="B5" s="90" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C6" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D6" s="79" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E6" s="79" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F6" s="79" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G6" s="79" t="n"/>
+    </row>
+    <row r="7">
+      <c r="B7" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C7" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D7" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" s="88" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C8" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D8" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="82" t="n">
+        <v>0</v>
+      </c>
+      <c r="G8" s="82" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C9" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D9" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="84" t="n">
+        <v>0</v>
+      </c>
+      <c r="G9" s="84" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C10" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D10" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G10" s="91" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C11" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D11" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="86" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="80" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" s="80" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="79" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C13" s="90" t="n"/>
+      <c r="D13" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="79" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" s="79" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B5:G5"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: close office work, start break
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G13"/>
+  <dimension ref="B1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11663,203 +11663,233 @@
       </c>
       <c r="F3" s="86" t="inlineStr">
         <is>
+          <t>7:53</t>
+        </is>
+      </c>
+      <c r="G3" s="86" t="n">
+        <v>17</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="64">
+      <c r="B4" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="81" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E4" s="80" t="inlineStr">
+        <is>
+          <t>7:53</t>
+        </is>
+      </c>
+      <c r="F4" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G3" s="86" t="inlineStr">
+      <c r="G4" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="5" ht="20" customHeight="1" s="64">
-      <c r="B5" s="90" t="inlineStr">
+    <row r="6" ht="20" customHeight="1" s="64">
+      <c r="B6" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="6">
-      <c r="B6" s="79" t="inlineStr">
+    <row r="7">
+      <c r="B7" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C6" s="79" t="inlineStr">
+      <c r="C7" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D6" s="79" t="inlineStr">
+      <c r="D7" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E6" s="79" t="inlineStr">
+      <c r="E7" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F6" s="79" t="inlineStr">
+      <c r="F7" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G6" s="79" t="n"/>
-    </row>
-    <row r="7">
-      <c r="B7" s="88" t="inlineStr">
+      <c r="G7" s="79" t="n"/>
+    </row>
+    <row r="8">
+      <c r="B8" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C7" s="89" t="inlineStr">
+      <c r="C8" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D7" s="88" t="n">
+      <c r="D8" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="88" t="n">
+      <c r="E8" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="88" t="n">
+      <c r="F8" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G7" s="88" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="82" t="inlineStr">
+      <c r="G8" s="88" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C8" s="83" t="inlineStr">
+      <c r="C9" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D8" s="82" t="n">
+      <c r="D9" s="82" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="82" t="n">
+      <c r="E9" s="82" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="82" t="n">
+      <c r="F9" s="82" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="82" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="84" t="inlineStr">
+      <c r="G9" s="82" t="n"/>
+    </row>
+    <row r="10">
+      <c r="B10" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C9" s="85" t="inlineStr">
+      <c r="C10" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D9" s="84" t="n">
+      <c r="D10" s="84" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="84" t="n">
+      <c r="E10" s="84" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="84" t="n">
+      <c r="F10" s="84" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="84" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="91" t="inlineStr">
+      <c r="G10" s="84" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C10" s="92" t="inlineStr">
+      <c r="C11" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D10" s="91" t="n">
+      <c r="D11" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="91" t="n">
+      <c r="E11" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="91" t="n">
+      <c r="F11" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="91" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="86" t="inlineStr">
+      <c r="G11" s="91" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C11" s="87" t="inlineStr">
+      <c r="C12" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D11" s="86" t="n">
+      <c r="D12" s="86" t="n">
+        <v>17</v>
+      </c>
+      <c r="E12" s="86" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F12" s="86" t="n">
+        <v>100</v>
+      </c>
+      <c r="G12" s="86" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="80" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="86" t="n">
+      <c r="E13" s="80" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="86" t="n">
+      <c r="F13" s="80" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="86" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="80" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="C12" s="81" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D12" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="G12" s="80" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="79" t="inlineStr">
+      <c r="G13" s="80" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C13" s="90" t="n"/>
-      <c r="D13" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="79" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="79" t="n"/>
+      <c r="C14" s="90" t="n"/>
+      <c r="D14" s="79" t="n">
+        <v>17</v>
+      </c>
+      <c r="E14" s="79" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F14" s="79" t="n">
+        <v>100</v>
+      </c>
+      <c r="G14" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B5:G5"/>
+    <mergeCell ref="B6:G6"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: radio exercises, morning meetings, floor patrol
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G14"/>
+  <dimension ref="B1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11693,203 +11693,293 @@
       </c>
       <c r="F4" s="80" t="inlineStr">
         <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="G4" s="80" t="n">
+        <v>7</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="64">
+      <c r="B5" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C5" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D5" s="81" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E5" s="80" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F5" s="80" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G5" s="80" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="64">
+      <c r="B6" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C6" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D6" s="83" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E6" s="82" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F6" s="82" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="G6" s="82" t="n">
+        <v>2</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C7" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D7" s="85" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E7" s="84" t="inlineStr">
+        <is>
+          <t>8:05</t>
+        </is>
+      </c>
+      <c r="F7" s="84" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G4" s="80" t="inlineStr">
+      <c r="G7" s="84" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="20" customHeight="1" s="64">
-      <c r="B6" s="90" t="inlineStr">
+    <row r="9" ht="20" customHeight="1" s="64">
+      <c r="B9" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="7">
-      <c r="B7" s="79" t="inlineStr">
+    <row r="10">
+      <c r="B10" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C7" s="79" t="inlineStr">
+      <c r="C10" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D7" s="79" t="inlineStr">
+      <c r="D10" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E7" s="79" t="inlineStr">
+      <c r="E10" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F7" s="79" t="inlineStr">
+      <c r="F10" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G7" s="79" t="n"/>
-    </row>
-    <row r="8">
-      <c r="B8" s="88" t="inlineStr">
+      <c r="G10" s="79" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C8" s="89" t="inlineStr">
+      <c r="C11" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D8" s="88" t="n">
+      <c r="D11" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="88" t="n">
+      <c r="E11" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="88" t="n">
+      <c r="F11" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G8" s="88" t="n"/>
-    </row>
-    <row r="9">
-      <c r="B9" s="82" t="inlineStr">
+      <c r="G11" s="88" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C9" s="83" t="inlineStr">
+      <c r="C12" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D9" s="82" t="n">
+      <c r="D12" s="82" t="n">
+        <v>2</v>
+      </c>
+      <c r="E12" s="82" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="82" t="n">
+      <c r="F12" s="82" t="n">
+        <v>6.9</v>
+      </c>
+      <c r="G12" s="82" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C13" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D13" s="84" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="82" t="n">
+      <c r="E13" s="84" t="n">
         <v>0</v>
       </c>
-      <c r="G9" s="82" t="n"/>
-    </row>
-    <row r="10">
-      <c r="B10" s="84" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C10" s="85" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D10" s="84" t="n">
+      <c r="F13" s="84" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="84" t="n">
+      <c r="G13" s="84" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C14" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D14" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="84" t="n">
+      <c r="E14" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G10" s="84" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="91" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C11" s="92" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D11" s="91" t="n">
+      <c r="F14" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G11" s="91" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="86" t="inlineStr">
+      <c r="G14" s="91" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C12" s="87" t="inlineStr">
+      <c r="C15" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D12" s="86" t="n">
+      <c r="D15" s="86" t="n">
         <v>17</v>
       </c>
-      <c r="E12" s="86" t="n">
+      <c r="E15" s="86" t="n">
         <v>0.3</v>
       </c>
-      <c r="F12" s="86" t="n">
+      <c r="F15" s="86" t="n">
+        <v>58.6</v>
+      </c>
+      <c r="G15" s="86" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C16" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D16" s="80" t="n">
+        <v>10</v>
+      </c>
+      <c r="E16" s="80" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F16" s="80" t="n">
+        <v>34.5</v>
+      </c>
+      <c r="G16" s="80" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="79" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C17" s="90" t="n"/>
+      <c r="D17" s="79" t="n">
+        <v>29</v>
+      </c>
+      <c r="E17" s="79" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F17" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G12" s="86" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="80" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="C13" s="81" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D13" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="80" t="n">
-        <v>0</v>
-      </c>
-      <c r="G13" s="80" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="79" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="C14" s="90" t="n"/>
-      <c r="D14" s="79" t="n">
-        <v>17</v>
-      </c>
-      <c r="E14" s="79" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F14" s="79" t="n">
-        <v>100</v>
-      </c>
-      <c r="G14" s="79" t="n"/>
+      <c r="G17" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B6:G6"/>
+    <mergeCell ref="B9:G9"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: close floor patrol, start office work
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G17"/>
+  <dimension ref="B1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11783,203 +11783,233 @@
       </c>
       <c r="F7" s="84" t="inlineStr">
         <is>
+          <t>8:35</t>
+        </is>
+      </c>
+      <c r="G7" s="84" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C8" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D8" s="87" t="inlineStr">
+        <is>
+          <t>事務作業</t>
+        </is>
+      </c>
+      <c r="E8" s="86" t="inlineStr">
+        <is>
+          <t>8:35</t>
+        </is>
+      </c>
+      <c r="F8" s="86" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G7" s="84" t="inlineStr">
+      <c r="G8" s="86" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1" s="64">
-      <c r="B9" s="90" t="inlineStr">
+    <row r="10" ht="20" customHeight="1" s="64">
+      <c r="B10" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="79" t="inlineStr">
+    <row r="11">
+      <c r="B11" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C10" s="79" t="inlineStr">
+      <c r="C11" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D10" s="79" t="inlineStr">
+      <c r="D11" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E10" s="79" t="inlineStr">
+      <c r="E11" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F10" s="79" t="inlineStr">
+      <c r="F11" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G10" s="79" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="88" t="inlineStr">
+      <c r="G11" s="79" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C11" s="89" t="inlineStr">
+      <c r="C12" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D11" s="88" t="n">
+      <c r="D12" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="88" t="n">
+      <c r="E12" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="88" t="n">
+      <c r="F12" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="88" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="82" t="inlineStr">
+      <c r="G12" s="88" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C12" s="83" t="inlineStr">
+      <c r="C13" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D12" s="82" t="n">
+      <c r="D13" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="E12" s="82" t="n">
+      <c r="E13" s="82" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="82" t="n">
-        <v>6.9</v>
-      </c>
-      <c r="G12" s="82" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="84" t="inlineStr">
+      <c r="F13" s="82" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="G13" s="82" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C13" s="85" t="inlineStr">
+      <c r="C14" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D13" s="84" t="n">
+      <c r="D14" s="84" t="n">
+        <v>30</v>
+      </c>
+      <c r="E14" s="84" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F14" s="84" t="n">
+        <v>50.8</v>
+      </c>
+      <c r="G14" s="84" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C15" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D15" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="84" t="n">
+      <c r="E15" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="84" t="n">
+      <c r="F15" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="84" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="91" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C14" s="92" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D14" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G14" s="91" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="86" t="inlineStr">
+      <c r="G15" s="91" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C15" s="87" t="inlineStr">
+      <c r="C16" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D15" s="86" t="n">
+      <c r="D16" s="86" t="n">
         <v>17</v>
       </c>
-      <c r="E15" s="86" t="n">
+      <c r="E16" s="86" t="n">
         <v>0.3</v>
       </c>
-      <c r="F15" s="86" t="n">
-        <v>58.6</v>
-      </c>
-      <c r="G15" s="86" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="80" t="inlineStr">
+      <c r="F16" s="86" t="n">
+        <v>28.8</v>
+      </c>
+      <c r="G16" s="86" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C16" s="81" t="inlineStr">
+      <c r="C17" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D16" s="80" t="n">
+      <c r="D17" s="80" t="n">
         <v>10</v>
       </c>
-      <c r="E16" s="80" t="n">
+      <c r="E17" s="80" t="n">
         <v>0.2</v>
       </c>
-      <c r="F16" s="80" t="n">
-        <v>34.5</v>
-      </c>
-      <c r="G16" s="80" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="79" t="inlineStr">
+      <c r="F17" s="80" t="n">
+        <v>16.9</v>
+      </c>
+      <c r="G17" s="80" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C17" s="90" t="n"/>
-      <c r="D17" s="79" t="n">
-        <v>29</v>
-      </c>
-      <c r="E17" s="79" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F17" s="79" t="n">
+      <c r="C18" s="90" t="n"/>
+      <c r="D18" s="79" t="n">
+        <v>59</v>
+      </c>
+      <c r="E18" s="79" t="n">
+        <v>1</v>
+      </c>
+      <c r="F18" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G17" s="79" t="n"/>
+      <c r="G18" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B10:G10"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: on-site item check for estimate
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G18"/>
+  <dimension ref="B1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11813,203 +11813,233 @@
       </c>
       <c r="F8" s="86" t="inlineStr">
         <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="G8" s="86" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C9" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D9" s="85" t="inlineStr">
+        <is>
+          <t>現場 現物確認（見積もり対応）</t>
+        </is>
+      </c>
+      <c r="E9" s="84" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="F9" s="84" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G8" s="86" t="inlineStr">
+      <c r="G9" s="84" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="20" customHeight="1" s="64">
-      <c r="B10" s="90" t="inlineStr">
+    <row r="11" ht="20" customHeight="1" s="64">
+      <c r="B11" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="B11" s="79" t="inlineStr">
+    <row r="12">
+      <c r="B12" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C11" s="79" t="inlineStr">
+      <c r="C12" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D11" s="79" t="inlineStr">
+      <c r="D12" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E11" s="79" t="inlineStr">
+      <c r="E12" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F11" s="79" t="inlineStr">
+      <c r="F12" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G11" s="79" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="88" t="inlineStr">
+      <c r="G12" s="79" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C12" s="89" t="inlineStr">
+      <c r="C13" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D12" s="88" t="n">
+      <c r="D13" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="88" t="n">
+      <c r="E13" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="88" t="n">
+      <c r="F13" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G12" s="88" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="82" t="inlineStr">
+      <c r="G13" s="88" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C13" s="83" t="inlineStr">
+      <c r="C14" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D13" s="82" t="n">
+      <c r="D14" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="E13" s="82" t="n">
+      <c r="E14" s="82" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="82" t="n">
-        <v>3.4</v>
-      </c>
-      <c r="G13" s="82" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="84" t="inlineStr">
+      <c r="F14" s="82" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="G14" s="82" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C14" s="85" t="inlineStr">
+      <c r="C15" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D14" s="84" t="n">
+      <c r="D15" s="84" t="n">
         <v>30</v>
       </c>
-      <c r="E14" s="84" t="n">
+      <c r="E15" s="84" t="n">
         <v>0.5</v>
       </c>
-      <c r="F14" s="84" t="n">
-        <v>50.8</v>
-      </c>
-      <c r="G14" s="84" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="91" t="inlineStr">
+      <c r="F15" s="84" t="n">
+        <v>43.5</v>
+      </c>
+      <c r="G15" s="84" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C15" s="92" t="inlineStr">
+      <c r="C16" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D15" s="91" t="n">
+      <c r="D16" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="91" t="n">
+      <c r="E16" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="91" t="n">
+      <c r="F16" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="91" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="86" t="inlineStr">
+      <c r="G16" s="91" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C16" s="87" t="inlineStr">
+      <c r="C17" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D16" s="86" t="n">
-        <v>17</v>
-      </c>
-      <c r="E16" s="86" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F16" s="86" t="n">
-        <v>28.8</v>
-      </c>
-      <c r="G16" s="86" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="80" t="inlineStr">
+      <c r="D17" s="86" t="n">
+        <v>27</v>
+      </c>
+      <c r="E17" s="86" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F17" s="86" t="n">
+        <v>39.1</v>
+      </c>
+      <c r="G17" s="86" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C17" s="81" t="inlineStr">
+      <c r="C18" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D17" s="80" t="n">
+      <c r="D18" s="80" t="n">
         <v>10</v>
       </c>
-      <c r="E17" s="80" t="n">
+      <c r="E18" s="80" t="n">
         <v>0.2</v>
       </c>
-      <c r="F17" s="80" t="n">
-        <v>16.9</v>
-      </c>
-      <c r="G17" s="80" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="79" t="inlineStr">
+      <c r="F18" s="80" t="n">
+        <v>14.5</v>
+      </c>
+      <c r="G18" s="80" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C18" s="90" t="n"/>
-      <c r="D18" s="79" t="n">
-        <v>59</v>
-      </c>
-      <c r="E18" s="79" t="n">
-        <v>1</v>
-      </c>
-      <c r="F18" s="79" t="n">
+      <c r="C19" s="90" t="n"/>
+      <c r="D19" s="79" t="n">
+        <v>69</v>
+      </c>
+      <c r="E19" s="79" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F19" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G18" s="79" t="n"/>
+      <c r="G19" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B10:G10"/>
+    <mergeCell ref="B11:G11"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: close item check, start break
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G19"/>
+  <dimension ref="B1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11843,203 +11843,233 @@
       </c>
       <c r="F9" s="84" t="inlineStr">
         <is>
+          <t>10:02</t>
+        </is>
+      </c>
+      <c r="G9" s="84" t="n">
+        <v>77</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C10" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D10" s="81" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E10" s="80" t="inlineStr">
+        <is>
+          <t>10:02</t>
+        </is>
+      </c>
+      <c r="F10" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G9" s="84" t="inlineStr">
+      <c r="G10" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="20" customHeight="1" s="64">
-      <c r="B11" s="90" t="inlineStr">
+    <row r="12" ht="20" customHeight="1" s="64">
+      <c r="B12" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="B12" s="79" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C12" s="79" t="inlineStr">
+      <c r="C13" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D12" s="79" t="inlineStr">
+      <c r="D13" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E12" s="79" t="inlineStr">
+      <c r="E13" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F12" s="79" t="inlineStr">
+      <c r="F13" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G12" s="79" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="88" t="inlineStr">
+      <c r="G13" s="79" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C13" s="89" t="inlineStr">
+      <c r="C14" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D13" s="88" t="n">
+      <c r="D14" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="88" t="n">
+      <c r="E14" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="88" t="n">
+      <c r="F14" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G13" s="88" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="82" t="inlineStr">
+      <c r="G14" s="88" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C14" s="83" t="inlineStr">
+      <c r="C15" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D14" s="82" t="n">
+      <c r="D15" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="E14" s="82" t="n">
+      <c r="E15" s="82" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="82" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="G14" s="82" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="84" t="inlineStr">
+      <c r="F15" s="82" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="G15" s="82" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C15" s="85" t="inlineStr">
+      <c r="C16" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D15" s="84" t="n">
-        <v>30</v>
-      </c>
-      <c r="E15" s="84" t="n">
+      <c r="D16" s="84" t="n">
+        <v>107</v>
+      </c>
+      <c r="E16" s="84" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F16" s="84" t="n">
+        <v>73.3</v>
+      </c>
+      <c r="G16" s="84" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C17" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D17" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G17" s="91" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C18" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D18" s="86" t="n">
+        <v>27</v>
+      </c>
+      <c r="E18" s="86" t="n">
         <v>0.5</v>
       </c>
-      <c r="F15" s="84" t="n">
-        <v>43.5</v>
-      </c>
-      <c r="G15" s="84" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="91" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C16" s="92" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D16" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G16" s="91" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="86" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C17" s="87" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D17" s="86" t="n">
-        <v>27</v>
-      </c>
-      <c r="E17" s="86" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F17" s="86" t="n">
-        <v>39.1</v>
-      </c>
-      <c r="G17" s="86" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="80" t="inlineStr">
+      <c r="F18" s="86" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G18" s="86" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C18" s="81" t="inlineStr">
+      <c r="C19" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D18" s="80" t="n">
+      <c r="D19" s="80" t="n">
         <v>10</v>
       </c>
-      <c r="E18" s="80" t="n">
+      <c r="E19" s="80" t="n">
         <v>0.2</v>
       </c>
-      <c r="F18" s="80" t="n">
-        <v>14.5</v>
-      </c>
-      <c r="G18" s="80" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="79" t="inlineStr">
+      <c r="F19" s="80" t="n">
+        <v>6.8</v>
+      </c>
+      <c r="G19" s="80" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C19" s="90" t="n"/>
-      <c r="D19" s="79" t="n">
-        <v>69</v>
-      </c>
-      <c r="E19" s="79" t="n">
-        <v>1.1</v>
-      </c>
-      <c r="F19" s="79" t="n">
+      <c r="C20" s="90" t="n"/>
+      <c r="D20" s="79" t="n">
+        <v>146</v>
+      </c>
+      <c r="E20" s="79" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F20" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G19" s="79" t="n"/>
+      <c r="G20" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B11:G11"/>
+    <mergeCell ref="B12:G12"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: close break, start accounting meeting
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G20"/>
+  <dimension ref="B1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11873,203 +11873,233 @@
       </c>
       <c r="F10" s="80" t="inlineStr">
         <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="G10" s="80" t="n">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C11" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D11" s="83" t="inlineStr">
+        <is>
+          <t>会計会議</t>
+        </is>
+      </c>
+      <c r="E11" s="82" t="inlineStr">
+        <is>
+          <t>10:13</t>
+        </is>
+      </c>
+      <c r="F11" s="82" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G10" s="80" t="inlineStr">
+      <c r="G11" s="82" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1" s="64">
-      <c r="B12" s="90" t="inlineStr">
+    <row r="13" ht="20" customHeight="1" s="64">
+      <c r="B13" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="79" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C13" s="79" t="inlineStr">
+      <c r="C14" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D13" s="79" t="inlineStr">
+      <c r="D14" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E13" s="79" t="inlineStr">
+      <c r="E14" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F13" s="79" t="inlineStr">
+      <c r="F14" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G13" s="79" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="88" t="inlineStr">
+      <c r="G14" s="79" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C14" s="89" t="inlineStr">
+      <c r="C15" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D14" s="88" t="n">
+      <c r="D15" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="88" t="n">
+      <c r="E15" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="88" t="n">
+      <c r="F15" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="88" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="82" t="inlineStr">
+      <c r="G15" s="88" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C15" s="83" t="inlineStr">
+      <c r="C16" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D15" s="82" t="n">
+      <c r="D16" s="82" t="n">
         <v>2</v>
       </c>
-      <c r="E15" s="82" t="n">
+      <c r="E16" s="82" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="82" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="G15" s="82" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="84" t="inlineStr">
+      <c r="F16" s="82" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="G16" s="82" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C16" s="85" t="inlineStr">
+      <c r="C17" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D16" s="84" t="n">
+      <c r="D17" s="84" t="n">
         <v>107</v>
       </c>
-      <c r="E16" s="84" t="n">
+      <c r="E17" s="84" t="n">
         <v>1.8</v>
       </c>
-      <c r="F16" s="84" t="n">
-        <v>73.3</v>
-      </c>
-      <c r="G16" s="84" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="91" t="inlineStr">
+      <c r="F17" s="84" t="n">
+        <v>68.2</v>
+      </c>
+      <c r="G17" s="84" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C17" s="92" t="inlineStr">
+      <c r="C18" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D17" s="91" t="n">
+      <c r="D18" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="91" t="n">
+      <c r="E18" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="91" t="n">
+      <c r="F18" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="91" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="86" t="inlineStr">
+      <c r="G18" s="91" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C18" s="87" t="inlineStr">
+      <c r="C19" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D18" s="86" t="n">
+      <c r="D19" s="86" t="n">
         <v>27</v>
       </c>
-      <c r="E18" s="86" t="n">
+      <c r="E19" s="86" t="n">
         <v>0.5</v>
       </c>
-      <c r="F18" s="86" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="G18" s="86" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="80" t="inlineStr">
+      <c r="F19" s="86" t="n">
+        <v>17.2</v>
+      </c>
+      <c r="G19" s="86" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C19" s="81" t="inlineStr">
+      <c r="C20" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D19" s="80" t="n">
-        <v>10</v>
-      </c>
-      <c r="E19" s="80" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F19" s="80" t="n">
-        <v>6.8</v>
-      </c>
-      <c r="G19" s="80" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="79" t="inlineStr">
+      <c r="D20" s="80" t="n">
+        <v>21</v>
+      </c>
+      <c r="E20" s="80" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F20" s="80" t="n">
+        <v>13.4</v>
+      </c>
+      <c r="G20" s="80" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C20" s="90" t="n"/>
-      <c r="D20" s="79" t="n">
-        <v>146</v>
-      </c>
-      <c r="E20" s="79" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="F20" s="79" t="n">
+      <c r="C21" s="90" t="n"/>
+      <c r="D21" s="79" t="n">
+        <v>157</v>
+      </c>
+      <c r="E21" s="79" t="n">
+        <v>2.6</v>
+      </c>
+      <c r="F21" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G20" s="79" t="n"/>
+      <c r="G21" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B13:G13"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: close accounting meeting at 11:13
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11903,13 +11903,11 @@
       </c>
       <c r="F11" s="82" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G11" s="82" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="G11" s="82" t="n">
+        <v>60</v>
       </c>
     </row>
     <row r="13" ht="20" customHeight="1" s="64">
@@ -11981,13 +11979,13 @@
         </is>
       </c>
       <c r="D16" s="82" t="n">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="E16" s="82" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="F16" s="82" t="n">
-        <v>1.3</v>
+        <v>28.6</v>
       </c>
       <c r="G16" s="82" t="n"/>
     </row>
@@ -12009,7 +12007,7 @@
         <v>1.8</v>
       </c>
       <c r="F17" s="84" t="n">
-        <v>68.2</v>
+        <v>49.3</v>
       </c>
       <c r="G17" s="84" t="n"/>
     </row>
@@ -12053,7 +12051,7 @@
         <v>0.5</v>
       </c>
       <c r="F19" s="86" t="n">
-        <v>17.2</v>
+        <v>12.4</v>
       </c>
       <c r="G19" s="86" t="n"/>
     </row>
@@ -12075,7 +12073,7 @@
         <v>0.3</v>
       </c>
       <c r="F20" s="80" t="n">
-        <v>13.4</v>
+        <v>9.699999999999999</v>
       </c>
       <c r="G20" s="80" t="n"/>
     </row>
@@ -12087,10 +12085,10 @@
       </c>
       <c r="C21" s="90" t="n"/>
       <c r="D21" s="79" t="n">
-        <v>157</v>
+        <v>217</v>
       </c>
       <c r="E21" s="79" t="n">
-        <v>2.6</v>
+        <v>3.6</v>
       </c>
       <c r="F21" s="79" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Update 2026-05-28: early lunch break at 11:29
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G21"/>
+  <dimension ref="B1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11910,194 +11910,226 @@
         <v>60</v>
       </c>
     </row>
-    <row r="13" ht="20" customHeight="1" s="64">
-      <c r="B13" s="90" t="inlineStr">
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="81" t="inlineStr">
+        <is>
+          <t>昼休憩（早め）</t>
+        </is>
+      </c>
+      <c r="E12" s="80" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="F12" s="80" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G12" s="80" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="20" customHeight="1" s="64">
+      <c r="B14" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="79" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C14" s="79" t="inlineStr">
+      <c r="C15" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D14" s="79" t="inlineStr">
+      <c r="D15" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E14" s="79" t="inlineStr">
+      <c r="E15" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F14" s="79" t="inlineStr">
+      <c r="F15" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G14" s="79" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="88" t="inlineStr">
+      <c r="G15" s="79" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C15" s="89" t="inlineStr">
+      <c r="C16" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D15" s="88" t="n">
+      <c r="D16" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="88" t="n">
+      <c r="E16" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="88" t="n">
+      <c r="F16" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G15" s="88" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="82" t="inlineStr">
+      <c r="G16" s="88" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C16" s="83" t="inlineStr">
+      <c r="C17" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D16" s="82" t="n">
+      <c r="D17" s="82" t="n">
         <v>62</v>
       </c>
-      <c r="E16" s="82" t="n">
+      <c r="E17" s="82" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="82" t="n">
+      <c r="F17" s="82" t="n">
         <v>28.6</v>
       </c>
-      <c r="G16" s="82" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="84" t="inlineStr">
+      <c r="G17" s="82" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C17" s="85" t="inlineStr">
+      <c r="C18" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D17" s="84" t="n">
+      <c r="D18" s="84" t="n">
         <v>107</v>
       </c>
-      <c r="E17" s="84" t="n">
+      <c r="E18" s="84" t="n">
         <v>1.8</v>
       </c>
-      <c r="F17" s="84" t="n">
+      <c r="F18" s="84" t="n">
         <v>49.3</v>
       </c>
-      <c r="G17" s="84" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="91" t="inlineStr">
+      <c r="G18" s="84" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C18" s="92" t="inlineStr">
+      <c r="C19" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D18" s="91" t="n">
+      <c r="D19" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="91" t="n">
+      <c r="E19" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="91" t="n">
+      <c r="F19" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="91" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="86" t="inlineStr">
+      <c r="G19" s="91" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C19" s="87" t="inlineStr">
+      <c r="C20" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D19" s="86" t="n">
+      <c r="D20" s="86" t="n">
         <v>27</v>
       </c>
-      <c r="E19" s="86" t="n">
+      <c r="E20" s="86" t="n">
         <v>0.5</v>
       </c>
-      <c r="F19" s="86" t="n">
+      <c r="F20" s="86" t="n">
         <v>12.4</v>
       </c>
-      <c r="G19" s="86" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="80" t="inlineStr">
+      <c r="G20" s="86" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C20" s="81" t="inlineStr">
+      <c r="C21" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D20" s="80" t="n">
+      <c r="D21" s="80" t="n">
         <v>21</v>
       </c>
-      <c r="E20" s="80" t="n">
+      <c r="E21" s="80" t="n">
         <v>0.3</v>
       </c>
-      <c r="F20" s="80" t="n">
+      <c r="F21" s="80" t="n">
         <v>9.699999999999999</v>
       </c>
-      <c r="G20" s="80" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="79" t="inlineStr">
+      <c r="G21" s="80" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C21" s="90" t="n"/>
-      <c r="D21" s="79" t="n">
+      <c r="C22" s="90" t="n"/>
+      <c r="D22" s="79" t="n">
         <v>217</v>
       </c>
-      <c r="E21" s="79" t="n">
+      <c r="E22" s="79" t="n">
         <v>3.6</v>
       </c>
-      <c r="F21" s="79" t="n">
+      <c r="F22" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G21" s="79" t="n"/>
+      <c r="G22" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B14:G14"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: insert office work after accounting meeting
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G22"/>
+  <dimension ref="B1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11911,225 +11911,255 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="80" t="inlineStr">
+      <c r="B12" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C12" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D12" s="87" t="inlineStr">
+        <is>
+          <t>事務作業</t>
+        </is>
+      </c>
+      <c r="E12" s="86" t="inlineStr">
+        <is>
+          <t>11:13</t>
+        </is>
+      </c>
+      <c r="F12" s="86" t="inlineStr">
+        <is>
+          <t>11:29</t>
+        </is>
+      </c>
+      <c r="G12" s="86" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C12" s="81" t="inlineStr">
+      <c r="C13" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D12" s="81" t="inlineStr">
+      <c r="D13" s="81" t="inlineStr">
         <is>
           <t>昼休憩（早め）</t>
         </is>
       </c>
-      <c r="E12" s="80" t="inlineStr">
+      <c r="E13" s="80" t="inlineStr">
         <is>
           <t>11:29</t>
         </is>
       </c>
-      <c r="F12" s="80" t="inlineStr">
+      <c r="F13" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G12" s="80" t="inlineStr">
+      <c r="G13" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="20" customHeight="1" s="64">
-      <c r="B14" s="90" t="inlineStr">
+    <row r="15" ht="20" customHeight="1" s="64">
+      <c r="B15" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="79" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C15" s="79" t="inlineStr">
+      <c r="C16" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D15" s="79" t="inlineStr">
+      <c r="D16" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E15" s="79" t="inlineStr">
+      <c r="E16" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F15" s="79" t="inlineStr">
+      <c r="F16" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G15" s="79" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="88" t="inlineStr">
+      <c r="G16" s="79" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C16" s="89" t="inlineStr">
+      <c r="C17" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D16" s="88" t="n">
+      <c r="D17" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="88" t="n">
+      <c r="E17" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="88" t="n">
+      <c r="F17" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G16" s="88" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="82" t="inlineStr">
+      <c r="G17" s="88" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C17" s="83" t="inlineStr">
+      <c r="C18" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D17" s="82" t="n">
+      <c r="D18" s="82" t="n">
         <v>62</v>
       </c>
-      <c r="E17" s="82" t="n">
+      <c r="E18" s="82" t="n">
         <v>1</v>
       </c>
-      <c r="F17" s="82" t="n">
-        <v>28.6</v>
-      </c>
-      <c r="G17" s="82" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="84" t="inlineStr">
+      <c r="F18" s="82" t="n">
+        <v>26.6</v>
+      </c>
+      <c r="G18" s="82" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C18" s="85" t="inlineStr">
+      <c r="C19" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D18" s="84" t="n">
+      <c r="D19" s="84" t="n">
         <v>107</v>
       </c>
-      <c r="E18" s="84" t="n">
+      <c r="E19" s="84" t="n">
         <v>1.8</v>
       </c>
-      <c r="F18" s="84" t="n">
-        <v>49.3</v>
-      </c>
-      <c r="G18" s="84" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="91" t="inlineStr">
+      <c r="F19" s="84" t="n">
+        <v>45.9</v>
+      </c>
+      <c r="G19" s="84" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C19" s="92" t="inlineStr">
+      <c r="C20" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D19" s="91" t="n">
+      <c r="D20" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="91" t="n">
+      <c r="E20" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="91" t="n">
+      <c r="F20" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G19" s="91" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="86" t="inlineStr">
+      <c r="G20" s="91" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C20" s="87" t="inlineStr">
+      <c r="C21" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D20" s="86" t="n">
-        <v>27</v>
-      </c>
-      <c r="E20" s="86" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F20" s="86" t="n">
-        <v>12.4</v>
-      </c>
-      <c r="G20" s="86" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="80" t="inlineStr">
+      <c r="D21" s="86" t="n">
+        <v>43</v>
+      </c>
+      <c r="E21" s="86" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F21" s="86" t="n">
+        <v>18.5</v>
+      </c>
+      <c r="G21" s="86" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C21" s="81" t="inlineStr">
+      <c r="C22" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D21" s="80" t="n">
+      <c r="D22" s="80" t="n">
         <v>21</v>
       </c>
-      <c r="E21" s="80" t="n">
+      <c r="E22" s="80" t="n">
         <v>0.3</v>
       </c>
-      <c r="F21" s="80" t="n">
-        <v>9.699999999999999</v>
-      </c>
-      <c r="G21" s="80" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="79" t="inlineStr">
+      <c r="F22" s="80" t="n">
+        <v>9</v>
+      </c>
+      <c r="G22" s="80" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C22" s="90" t="n"/>
-      <c r="D22" s="79" t="n">
-        <v>217</v>
-      </c>
-      <c r="E22" s="79" t="n">
-        <v>3.6</v>
-      </c>
-      <c r="F22" s="79" t="n">
+      <c r="C23" s="90" t="n"/>
+      <c r="D23" s="79" t="n">
+        <v>233</v>
+      </c>
+      <c r="E23" s="79" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F23" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G22" s="79" t="n"/>
+      <c r="G23" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B14:G14"/>
+    <mergeCell ref="B15:G15"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: close lunch, depart for client visit
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G23"/>
+  <dimension ref="B1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11953,7 +11953,7 @@
       </c>
       <c r="D13" s="81" t="inlineStr">
         <is>
-          <t>昼休憩（早め）</t>
+          <t>昼休憩</t>
         </is>
       </c>
       <c r="E13" s="80" t="inlineStr">
@@ -11963,203 +11963,233 @@
       </c>
       <c r="F13" s="80" t="inlineStr">
         <is>
+          <t>11:59</t>
+        </is>
+      </c>
+      <c r="G13" s="80" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C14" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D14" s="81" t="inlineStr">
+        <is>
+          <t>客先へ移動</t>
+        </is>
+      </c>
+      <c r="E14" s="80" t="inlineStr">
+        <is>
+          <t>11:59</t>
+        </is>
+      </c>
+      <c r="F14" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G13" s="80" t="inlineStr">
+      <c r="G14" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="20" customHeight="1" s="64">
-      <c r="B15" s="90" t="inlineStr">
+    <row r="16" ht="20" customHeight="1" s="64">
+      <c r="B16" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="79" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C16" s="79" t="inlineStr">
+      <c r="C17" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D16" s="79" t="inlineStr">
+      <c r="D17" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E16" s="79" t="inlineStr">
+      <c r="E17" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F16" s="79" t="inlineStr">
+      <c r="F17" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G16" s="79" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="88" t="inlineStr">
+      <c r="G17" s="79" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C17" s="89" t="inlineStr">
+      <c r="C18" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D17" s="88" t="n">
+      <c r="D18" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="88" t="n">
+      <c r="E18" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="88" t="n">
+      <c r="F18" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G17" s="88" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="82" t="inlineStr">
+      <c r="G18" s="88" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C18" s="83" t="inlineStr">
+      <c r="C19" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D18" s="82" t="n">
+      <c r="D19" s="82" t="n">
         <v>62</v>
       </c>
-      <c r="E18" s="82" t="n">
+      <c r="E19" s="82" t="n">
         <v>1</v>
       </c>
-      <c r="F18" s="82" t="n">
-        <v>26.6</v>
-      </c>
-      <c r="G18" s="82" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="84" t="inlineStr">
+      <c r="F19" s="82" t="n">
+        <v>23.6</v>
+      </c>
+      <c r="G19" s="82" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C19" s="85" t="inlineStr">
+      <c r="C20" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D19" s="84" t="n">
+      <c r="D20" s="84" t="n">
         <v>107</v>
       </c>
-      <c r="E19" s="84" t="n">
+      <c r="E20" s="84" t="n">
         <v>1.8</v>
       </c>
-      <c r="F19" s="84" t="n">
-        <v>45.9</v>
-      </c>
-      <c r="G19" s="84" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="91" t="inlineStr">
+      <c r="F20" s="84" t="n">
+        <v>40.7</v>
+      </c>
+      <c r="G20" s="84" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C20" s="92" t="inlineStr">
+      <c r="C21" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D20" s="91" t="n">
+      <c r="D21" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="91" t="n">
+      <c r="E21" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="91" t="n">
+      <c r="F21" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="91" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="86" t="inlineStr">
+      <c r="G21" s="91" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C21" s="87" t="inlineStr">
+      <c r="C22" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D21" s="86" t="n">
+      <c r="D22" s="86" t="n">
         <v>43</v>
       </c>
-      <c r="E21" s="86" t="n">
+      <c r="E22" s="86" t="n">
         <v>0.7</v>
       </c>
-      <c r="F21" s="86" t="n">
-        <v>18.5</v>
-      </c>
-      <c r="G21" s="86" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="80" t="inlineStr">
+      <c r="F22" s="86" t="n">
+        <v>16.3</v>
+      </c>
+      <c r="G22" s="86" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C22" s="81" t="inlineStr">
+      <c r="C23" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D22" s="80" t="n">
-        <v>21</v>
-      </c>
-      <c r="E22" s="80" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F22" s="80" t="n">
-        <v>9</v>
-      </c>
-      <c r="G22" s="80" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="79" t="inlineStr">
+      <c r="D23" s="80" t="n">
+        <v>51</v>
+      </c>
+      <c r="E23" s="80" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F23" s="80" t="n">
+        <v>19.4</v>
+      </c>
+      <c r="G23" s="80" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C23" s="90" t="n"/>
-      <c r="D23" s="79" t="n">
-        <v>233</v>
-      </c>
-      <c r="E23" s="79" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F23" s="79" t="n">
+      <c r="C24" s="90" t="n"/>
+      <c r="D24" s="79" t="n">
+        <v>263</v>
+      </c>
+      <c r="E24" s="79" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F24" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G23" s="79" t="n"/>
+      <c r="G24" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B15:G15"/>
+    <mergeCell ref="B16:G16"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: client meeting done, heading to 鉄道技術展
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G24"/>
+  <dimension ref="B1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -11993,203 +11993,263 @@
       </c>
       <c r="F14" s="80" t="inlineStr">
         <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="G14" s="80" t="n">
+        <v>41</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C15" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D15" s="89" t="inlineStr">
+        <is>
+          <t>客先打ち合わせ</t>
+        </is>
+      </c>
+      <c r="E15" s="88" t="inlineStr">
+        <is>
+          <t>12:40</t>
+        </is>
+      </c>
+      <c r="F15" s="88" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="G15" s="88" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C16" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D16" s="81" t="inlineStr">
+        <is>
+          <t>鉄道技術展へ移動（市場調査）</t>
+        </is>
+      </c>
+      <c r="E16" s="80" t="inlineStr">
+        <is>
+          <t>13:10</t>
+        </is>
+      </c>
+      <c r="F16" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G14" s="80" t="inlineStr">
+      <c r="G16" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="20" customHeight="1" s="64">
-      <c r="B16" s="90" t="inlineStr">
+    <row r="18" ht="20" customHeight="1" s="64">
+      <c r="B18" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="79" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C17" s="79" t="inlineStr">
+      <c r="C19" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D17" s="79" t="inlineStr">
+      <c r="D19" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E17" s="79" t="inlineStr">
+      <c r="E19" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F17" s="79" t="inlineStr">
+      <c r="F19" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G17" s="79" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="88" t="inlineStr">
+      <c r="G19" s="79" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C18" s="89" t="inlineStr">
+      <c r="C20" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D18" s="88" t="n">
+      <c r="D20" s="88" t="n">
+        <v>30</v>
+      </c>
+      <c r="E20" s="88" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F20" s="88" t="n">
+        <v>9</v>
+      </c>
+      <c r="G20" s="88" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C21" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D21" s="82" t="n">
+        <v>62</v>
+      </c>
+      <c r="E21" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="82" t="n">
+        <v>18.6</v>
+      </c>
+      <c r="G21" s="82" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C22" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D22" s="84" t="n">
+        <v>107</v>
+      </c>
+      <c r="E22" s="84" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F22" s="84" t="n">
+        <v>32</v>
+      </c>
+      <c r="G22" s="84" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C23" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D23" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="88" t="n">
+      <c r="E23" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="88" t="n">
+      <c r="F23" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G18" s="88" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="82" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
-      <c r="C19" s="83" t="inlineStr">
-        <is>
-          <t>社内マネジメント</t>
-        </is>
-      </c>
-      <c r="D19" s="82" t="n">
-        <v>62</v>
-      </c>
-      <c r="E19" s="82" t="n">
-        <v>1</v>
-      </c>
-      <c r="F19" s="82" t="n">
-        <v>23.6</v>
-      </c>
-      <c r="G19" s="82" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="84" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C20" s="85" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D20" s="84" t="n">
-        <v>107</v>
-      </c>
-      <c r="E20" s="84" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F20" s="84" t="n">
-        <v>40.7</v>
-      </c>
-      <c r="G20" s="84" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="91" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C21" s="92" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D21" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="E21" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F21" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G21" s="91" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="86" t="inlineStr">
+      <c r="G23" s="91" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C22" s="87" t="inlineStr">
+      <c r="C24" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D22" s="86" t="n">
+      <c r="D24" s="86" t="n">
         <v>43</v>
       </c>
-      <c r="E22" s="86" t="n">
+      <c r="E24" s="86" t="n">
         <v>0.7</v>
       </c>
-      <c r="F22" s="86" t="n">
-        <v>16.3</v>
-      </c>
-      <c r="G22" s="86" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="80" t="inlineStr">
+      <c r="F24" s="86" t="n">
+        <v>12.9</v>
+      </c>
+      <c r="G24" s="86" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C23" s="81" t="inlineStr">
+      <c r="C25" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D23" s="80" t="n">
-        <v>51</v>
-      </c>
-      <c r="E23" s="80" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F23" s="80" t="n">
-        <v>19.4</v>
-      </c>
-      <c r="G23" s="80" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="79" t="inlineStr">
+      <c r="D25" s="80" t="n">
+        <v>92</v>
+      </c>
+      <c r="E25" s="80" t="n">
+        <v>1.5</v>
+      </c>
+      <c r="F25" s="80" t="n">
+        <v>27.5</v>
+      </c>
+      <c r="G25" s="80" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C24" s="90" t="n"/>
-      <c r="D24" s="79" t="n">
-        <v>263</v>
-      </c>
-      <c r="E24" s="79" t="n">
-        <v>4.4</v>
-      </c>
-      <c r="F24" s="79" t="n">
+      <c r="C26" s="90" t="n"/>
+      <c r="D26" s="79" t="n">
+        <v>334</v>
+      </c>
+      <c r="E26" s="79" t="n">
+        <v>5.6</v>
+      </c>
+      <c r="F26" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G24" s="79" t="n"/>
+      <c r="G26" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B16:G16"/>
+    <mergeCell ref="B18:G18"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: arrive at 鉄道技術展, start market research
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G26"/>
+  <dimension ref="B1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -12043,7 +12043,7 @@
       </c>
       <c r="D16" s="81" t="inlineStr">
         <is>
-          <t>鉄道技術展へ移動（市場調査）</t>
+          <t>鉄道技術展へ移動</t>
         </is>
       </c>
       <c r="E16" s="80" t="inlineStr">
@@ -12053,203 +12053,233 @@
       </c>
       <c r="F16" s="80" t="inlineStr">
         <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="G16" s="80" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C17" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D17" s="89" t="inlineStr">
+        <is>
+          <t>鉄道技術展 市場調査</t>
+        </is>
+      </c>
+      <c r="E17" s="88" t="inlineStr">
+        <is>
+          <t>14:03</t>
+        </is>
+      </c>
+      <c r="F17" s="88" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G16" s="80" t="inlineStr">
+      <c r="G17" s="88" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="20" customHeight="1" s="64">
-      <c r="B18" s="90" t="inlineStr">
+    <row r="19" ht="20" customHeight="1" s="64">
+      <c r="B19" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="79" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C19" s="79" t="inlineStr">
+      <c r="C20" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D19" s="79" t="inlineStr">
+      <c r="D20" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E19" s="79" t="inlineStr">
+      <c r="E20" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F19" s="79" t="inlineStr">
+      <c r="F20" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G19" s="79" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="88" t="inlineStr">
+      <c r="G20" s="79" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C20" s="89" t="inlineStr">
+      <c r="C21" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D20" s="88" t="n">
+      <c r="D21" s="88" t="n">
         <v>30</v>
       </c>
-      <c r="E20" s="88" t="n">
+      <c r="E21" s="88" t="n">
         <v>0.5</v>
       </c>
-      <c r="F20" s="88" t="n">
-        <v>9</v>
-      </c>
-      <c r="G20" s="88" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="82" t="inlineStr">
+      <c r="F21" s="88" t="n">
+        <v>7.8</v>
+      </c>
+      <c r="G21" s="88" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C21" s="83" t="inlineStr">
+      <c r="C22" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D21" s="82" t="n">
+      <c r="D22" s="82" t="n">
         <v>62</v>
       </c>
-      <c r="E21" s="82" t="n">
+      <c r="E22" s="82" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="82" t="n">
-        <v>18.6</v>
-      </c>
-      <c r="G21" s="82" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="84" t="inlineStr">
+      <c r="F22" s="82" t="n">
+        <v>16</v>
+      </c>
+      <c r="G22" s="82" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C22" s="85" t="inlineStr">
+      <c r="C23" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D22" s="84" t="n">
+      <c r="D23" s="84" t="n">
         <v>107</v>
       </c>
-      <c r="E22" s="84" t="n">
+      <c r="E23" s="84" t="n">
         <v>1.8</v>
       </c>
-      <c r="F22" s="84" t="n">
-        <v>32</v>
-      </c>
-      <c r="G22" s="84" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="91" t="inlineStr">
+      <c r="F23" s="84" t="n">
+        <v>27.6</v>
+      </c>
+      <c r="G23" s="84" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C23" s="92" t="inlineStr">
+      <c r="C24" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D23" s="91" t="n">
+      <c r="D24" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="91" t="n">
+      <c r="E24" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="91" t="n">
+      <c r="F24" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G23" s="91" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="86" t="inlineStr">
+      <c r="G24" s="91" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C24" s="87" t="inlineStr">
+      <c r="C25" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D24" s="86" t="n">
+      <c r="D25" s="86" t="n">
         <v>43</v>
       </c>
-      <c r="E24" s="86" t="n">
+      <c r="E25" s="86" t="n">
         <v>0.7</v>
       </c>
-      <c r="F24" s="86" t="n">
-        <v>12.9</v>
-      </c>
-      <c r="G24" s="86" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="80" t="inlineStr">
+      <c r="F25" s="86" t="n">
+        <v>11.1</v>
+      </c>
+      <c r="G25" s="86" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C25" s="81" t="inlineStr">
+      <c r="C26" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D25" s="80" t="n">
-        <v>92</v>
-      </c>
-      <c r="E25" s="80" t="n">
-        <v>1.5</v>
-      </c>
-      <c r="F25" s="80" t="n">
-        <v>27.5</v>
-      </c>
-      <c r="G25" s="80" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="79" t="inlineStr">
+      <c r="D26" s="80" t="n">
+        <v>145</v>
+      </c>
+      <c r="E26" s="80" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F26" s="80" t="n">
+        <v>37.5</v>
+      </c>
+      <c r="G26" s="80" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C26" s="90" t="n"/>
-      <c r="D26" s="79" t="n">
-        <v>334</v>
-      </c>
-      <c r="E26" s="79" t="n">
-        <v>5.6</v>
-      </c>
-      <c r="F26" s="79" t="n">
+      <c r="C27" s="90" t="n"/>
+      <c r="D27" s="79" t="n">
+        <v>387</v>
+      </c>
+      <c r="E27" s="79" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F27" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G26" s="79" t="n"/>
+      <c r="G27" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B19:G19"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: close market research, return to office
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G27"/>
+  <dimension ref="B1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -12083,203 +12083,233 @@
       </c>
       <c r="F17" s="88" t="inlineStr">
         <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="G17" s="88" t="n">
+        <v>83</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C18" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D18" s="81" t="inlineStr">
+        <is>
+          <t>帰社移動</t>
+        </is>
+      </c>
+      <c r="E18" s="80" t="inlineStr">
+        <is>
+          <t>15:26</t>
+        </is>
+      </c>
+      <c r="F18" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G17" s="88" t="inlineStr">
+      <c r="G18" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="19" ht="20" customHeight="1" s="64">
-      <c r="B19" s="90" t="inlineStr">
+    <row r="20" ht="20" customHeight="1" s="64">
+      <c r="B20" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="79" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C20" s="79" t="inlineStr">
+      <c r="C21" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D20" s="79" t="inlineStr">
+      <c r="D21" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E20" s="79" t="inlineStr">
+      <c r="E21" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F20" s="79" t="inlineStr">
+      <c r="F21" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G20" s="79" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="88" t="inlineStr">
+      <c r="G21" s="79" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C21" s="89" t="inlineStr">
+      <c r="C22" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D21" s="88" t="n">
-        <v>30</v>
-      </c>
-      <c r="E21" s="88" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F21" s="88" t="n">
+      <c r="D22" s="88" t="n">
+        <v>113</v>
+      </c>
+      <c r="E22" s="88" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F22" s="88" t="n">
+        <v>24</v>
+      </c>
+      <c r="G22" s="88" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C23" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D23" s="82" t="n">
+        <v>62</v>
+      </c>
+      <c r="E23" s="82" t="n">
+        <v>1</v>
+      </c>
+      <c r="F23" s="82" t="n">
+        <v>13.2</v>
+      </c>
+      <c r="G23" s="82" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C24" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D24" s="84" t="n">
+        <v>107</v>
+      </c>
+      <c r="E24" s="84" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F24" s="84" t="n">
+        <v>22.8</v>
+      </c>
+      <c r="G24" s="84" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C25" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D25" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="E25" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="F25" s="91" t="n">
+        <v>0</v>
+      </c>
+      <c r="G25" s="91" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C26" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D26" s="86" t="n">
+        <v>43</v>
+      </c>
+      <c r="E26" s="86" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F26" s="86" t="n">
+        <v>9.1</v>
+      </c>
+      <c r="G26" s="86" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C27" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D27" s="80" t="n">
+        <v>145</v>
+      </c>
+      <c r="E27" s="80" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F27" s="80" t="n">
+        <v>30.9</v>
+      </c>
+      <c r="G27" s="80" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="79" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C28" s="90" t="n"/>
+      <c r="D28" s="79" t="n">
+        <v>470</v>
+      </c>
+      <c r="E28" s="79" t="n">
         <v>7.8</v>
       </c>
-      <c r="G21" s="88" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="82" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
-      <c r="C22" s="83" t="inlineStr">
-        <is>
-          <t>社内マネジメント</t>
-        </is>
-      </c>
-      <c r="D22" s="82" t="n">
-        <v>62</v>
-      </c>
-      <c r="E22" s="82" t="n">
-        <v>1</v>
-      </c>
-      <c r="F22" s="82" t="n">
-        <v>16</v>
-      </c>
-      <c r="G22" s="82" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="84" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C23" s="85" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D23" s="84" t="n">
-        <v>107</v>
-      </c>
-      <c r="E23" s="84" t="n">
-        <v>1.8</v>
-      </c>
-      <c r="F23" s="84" t="n">
-        <v>27.6</v>
-      </c>
-      <c r="G23" s="84" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="91" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C24" s="92" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D24" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="E24" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="F24" s="91" t="n">
-        <v>0</v>
-      </c>
-      <c r="G24" s="91" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="86" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C25" s="87" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D25" s="86" t="n">
-        <v>43</v>
-      </c>
-      <c r="E25" s="86" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F25" s="86" t="n">
-        <v>11.1</v>
-      </c>
-      <c r="G25" s="86" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="80" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="C26" s="81" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D26" s="80" t="n">
-        <v>145</v>
-      </c>
-      <c r="E26" s="80" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="F26" s="80" t="n">
-        <v>37.5</v>
-      </c>
-      <c r="G26" s="80" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="79" t="inlineStr">
-        <is>
-          <t>合計</t>
-        </is>
-      </c>
-      <c r="C27" s="90" t="n"/>
-      <c r="D27" s="79" t="n">
-        <v>387</v>
-      </c>
-      <c r="E27" s="79" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F27" s="79" t="n">
+      <c r="F28" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G27" s="79" t="n"/>
+      <c r="G28" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B19:G19"/>
+    <mergeCell ref="B20:G20"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-28: return to office at 17:01
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -12113,13 +12113,11 @@
       </c>
       <c r="F18" s="80" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G18" s="80" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="G18" s="80" t="n">
+        <v>95</v>
       </c>
     </row>
     <row r="20" ht="20" customHeight="1" s="64">
@@ -12175,7 +12173,7 @@
         <v>1.9</v>
       </c>
       <c r="F22" s="88" t="n">
-        <v>24</v>
+        <v>20</v>
       </c>
       <c r="G22" s="88" t="n"/>
     </row>
@@ -12197,7 +12195,7 @@
         <v>1</v>
       </c>
       <c r="F23" s="82" t="n">
-        <v>13.2</v>
+        <v>11</v>
       </c>
       <c r="G23" s="82" t="n"/>
     </row>
@@ -12219,7 +12217,7 @@
         <v>1.8</v>
       </c>
       <c r="F24" s="84" t="n">
-        <v>22.8</v>
+        <v>18.9</v>
       </c>
       <c r="G24" s="84" t="n"/>
     </row>
@@ -12263,7 +12261,7 @@
         <v>0.7</v>
       </c>
       <c r="F26" s="86" t="n">
-        <v>9.1</v>
+        <v>7.6</v>
       </c>
       <c r="G26" s="86" t="n"/>
     </row>
@@ -12279,13 +12277,13 @@
         </is>
       </c>
       <c r="D27" s="80" t="n">
-        <v>145</v>
+        <v>240</v>
       </c>
       <c r="E27" s="80" t="n">
-        <v>2.4</v>
+        <v>4</v>
       </c>
       <c r="F27" s="80" t="n">
-        <v>30.9</v>
+        <v>42.5</v>
       </c>
       <c r="G27" s="80" t="n"/>
     </row>
@@ -12297,10 +12295,10 @@
       </c>
       <c r="C28" s="90" t="n"/>
       <c r="D28" s="79" t="n">
-        <v>470</v>
+        <v>565</v>
       </c>
       <c r="E28" s="79" t="n">
-        <v>7.8</v>
+        <v>9.4</v>
       </c>
       <c r="F28" s="79" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Update 2026-05-28: start email check after return
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -11589,7 +11589,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G28"/>
+  <dimension ref="B1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -12120,194 +12120,226 @@
         <v>95</v>
       </c>
     </row>
-    <row r="20" ht="20" customHeight="1" s="64">
-      <c r="B20" s="90" t="inlineStr">
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="87" t="inlineStr">
+        <is>
+          <t>メールチェック</t>
+        </is>
+      </c>
+      <c r="E19" s="86" t="inlineStr">
+        <is>
+          <t>17:01</t>
+        </is>
+      </c>
+      <c r="F19" s="86" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G19" s="86" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="20" customHeight="1" s="64">
+      <c r="B21" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="79" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C21" s="79" t="inlineStr">
+      <c r="C22" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D21" s="79" t="inlineStr">
+      <c r="D22" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E21" s="79" t="inlineStr">
+      <c r="E22" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F21" s="79" t="inlineStr">
+      <c r="F22" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G21" s="79" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="88" t="inlineStr">
+      <c r="G22" s="79" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C22" s="89" t="inlineStr">
+      <c r="C23" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D22" s="88" t="n">
+      <c r="D23" s="88" t="n">
         <v>113</v>
       </c>
-      <c r="E22" s="88" t="n">
+      <c r="E23" s="88" t="n">
         <v>1.9</v>
       </c>
-      <c r="F22" s="88" t="n">
+      <c r="F23" s="88" t="n">
         <v>20</v>
       </c>
-      <c r="G22" s="88" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="82" t="inlineStr">
+      <c r="G23" s="88" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C23" s="83" t="inlineStr">
+      <c r="C24" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D23" s="82" t="n">
+      <c r="D24" s="82" t="n">
         <v>62</v>
       </c>
-      <c r="E23" s="82" t="n">
+      <c r="E24" s="82" t="n">
         <v>1</v>
       </c>
-      <c r="F23" s="82" t="n">
+      <c r="F24" s="82" t="n">
         <v>11</v>
       </c>
-      <c r="G23" s="82" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="84" t="inlineStr">
+      <c r="G24" s="82" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C24" s="85" t="inlineStr">
+      <c r="C25" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D24" s="84" t="n">
+      <c r="D25" s="84" t="n">
         <v>107</v>
       </c>
-      <c r="E24" s="84" t="n">
+      <c r="E25" s="84" t="n">
         <v>1.8</v>
       </c>
-      <c r="F24" s="84" t="n">
+      <c r="F25" s="84" t="n">
         <v>18.9</v>
       </c>
-      <c r="G24" s="84" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="91" t="inlineStr">
+      <c r="G25" s="84" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C25" s="92" t="inlineStr">
+      <c r="C26" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D25" s="91" t="n">
+      <c r="D26" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="91" t="n">
+      <c r="E26" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="91" t="n">
+      <c r="F26" s="91" t="n">
         <v>0</v>
       </c>
-      <c r="G25" s="91" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="86" t="inlineStr">
+      <c r="G26" s="91" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C26" s="87" t="inlineStr">
+      <c r="C27" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D26" s="86" t="n">
+      <c r="D27" s="86" t="n">
         <v>43</v>
       </c>
-      <c r="E26" s="86" t="n">
+      <c r="E27" s="86" t="n">
         <v>0.7</v>
       </c>
-      <c r="F26" s="86" t="n">
+      <c r="F27" s="86" t="n">
         <v>7.6</v>
       </c>
-      <c r="G26" s="86" t="n"/>
-    </row>
-    <row r="27">
-      <c r="B27" s="80" t="inlineStr">
+      <c r="G27" s="86" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C27" s="81" t="inlineStr">
+      <c r="C28" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D27" s="80" t="n">
+      <c r="D28" s="80" t="n">
         <v>240</v>
       </c>
-      <c r="E27" s="80" t="n">
+      <c r="E28" s="80" t="n">
         <v>4</v>
       </c>
-      <c r="F27" s="80" t="n">
+      <c r="F28" s="80" t="n">
         <v>42.5</v>
       </c>
-      <c r="G27" s="80" t="n"/>
-    </row>
-    <row r="28">
-      <c r="B28" s="79" t="inlineStr">
+      <c r="G28" s="80" t="n"/>
+    </row>
+    <row r="29">
+      <c r="B29" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C28" s="90" t="n"/>
-      <c r="D28" s="79" t="n">
+      <c r="C29" s="90" t="n"/>
+      <c r="D29" s="79" t="n">
         <v>565</v>
       </c>
-      <c r="E28" s="79" t="n">
+      <c r="E29" s="79" t="n">
         <v>9.4</v>
       </c>
-      <c r="F28" s="79" t="n">
+      <c r="F29" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G28" s="79" t="n"/>
+      <c r="G29" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B20:G20"/>
+    <mergeCell ref="B21:G21"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Complete 2026-05-28 daily record (end 18:45)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -12133,7 +12133,7 @@
       </c>
       <c r="D19" s="87" t="inlineStr">
         <is>
-          <t>メールチェック</t>
+          <t>メールチェック・返信</t>
         </is>
       </c>
       <c r="E19" s="86" t="inlineStr">
@@ -12143,13 +12143,11 @@
       </c>
       <c r="F19" s="86" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G19" s="86" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
+          <t>18:45</t>
+        </is>
+      </c>
+      <c r="G19" s="86" t="n">
+        <v>104</v>
       </c>
     </row>
     <row r="21" ht="20" customHeight="1" s="64">
@@ -12205,7 +12203,7 @@
         <v>1.9</v>
       </c>
       <c r="F23" s="88" t="n">
-        <v>20</v>
+        <v>16.9</v>
       </c>
       <c r="G23" s="88" t="n"/>
     </row>
@@ -12227,7 +12225,7 @@
         <v>1</v>
       </c>
       <c r="F24" s="82" t="n">
-        <v>11</v>
+        <v>9.300000000000001</v>
       </c>
       <c r="G24" s="82" t="n"/>
     </row>
@@ -12249,7 +12247,7 @@
         <v>1.8</v>
       </c>
       <c r="F25" s="84" t="n">
-        <v>18.9</v>
+        <v>16</v>
       </c>
       <c r="G25" s="84" t="n"/>
     </row>
@@ -12287,13 +12285,13 @@
         </is>
       </c>
       <c r="D27" s="86" t="n">
-        <v>43</v>
+        <v>147</v>
       </c>
       <c r="E27" s="86" t="n">
-        <v>0.7</v>
+        <v>2.5</v>
       </c>
       <c r="F27" s="86" t="n">
-        <v>7.6</v>
+        <v>22</v>
       </c>
       <c r="G27" s="86" t="n"/>
     </row>
@@ -12315,7 +12313,7 @@
         <v>4</v>
       </c>
       <c r="F28" s="80" t="n">
-        <v>42.5</v>
+        <v>35.9</v>
       </c>
       <c r="G28" s="80" t="n"/>
     </row>
@@ -12327,10 +12325,10 @@
       </c>
       <c r="C29" s="90" t="n"/>
       <c r="D29" s="79" t="n">
-        <v>565</v>
+        <v>669</v>
       </c>
       <c r="E29" s="79" t="n">
-        <v>9.4</v>
+        <v>11.2</v>
       </c>
       <c r="F29" s="79" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add daily task record for 2026-05-29 (作業中)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -20,14 +20,15 @@
     <sheet name="2026-05-26" sheetId="12" state="visible" r:id="rId12"/>
     <sheet name="2026-05-27" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-05-28" sheetId="14" state="visible" r:id="rId14"/>
+    <sheet name="2026-05-29" sheetId="15" state="visible" r:id="rId15"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId15"/>
     <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
     <externalReference r:id="rId19"/>
     <externalReference r:id="rId20"/>
+    <externalReference r:id="rId21"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -11607,6 +11608,11 @@
           <t>2026年5月28日（木）　業務記録</t>
         </is>
       </c>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="94" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1" s="64">
       <c r="B2" s="79" t="inlineStr">
@@ -12156,6 +12162,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C21" s="93" t="n"/>
+      <c r="D21" s="93" t="n"/>
+      <c r="E21" s="93" t="n"/>
+      <c r="F21" s="93" t="n"/>
+      <c r="G21" s="94" t="n"/>
     </row>
     <row r="22">
       <c r="B22" s="79" t="inlineStr">
@@ -12338,6 +12349,409 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B21:G21"/>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet15.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G17"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="2" customWidth="1" style="64" min="1" max="1"/>
+    <col width="6" customWidth="1" style="64" min="2" max="2"/>
+    <col width="20" customWidth="1" style="64" min="3" max="3"/>
+    <col width="44" customWidth="1" style="64" min="4" max="4"/>
+    <col width="8" customWidth="1" style="64" min="5" max="5"/>
+    <col width="8" customWidth="1" style="64" min="6" max="6"/>
+    <col width="14" customWidth="1" style="64" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="28" customHeight="1" s="64">
+      <c r="B1" s="78" t="inlineStr">
+        <is>
+          <t>2026年5月29日（金）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="64">
+      <c r="B2" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C2" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D2" s="79" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E2" s="79" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F2" s="79" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G2" s="79" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="64">
+      <c r="B3" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C3" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D3" s="81" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E3" s="80" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F3" s="80" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G3" s="80" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="64">
+      <c r="B4" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C4" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D4" s="83" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E4" s="82" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F4" s="82" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G4" s="82" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="64">
+      <c r="B5" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C5" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D5" s="85" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E5" s="84" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F5" s="84" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="G5" s="84" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="64">
+      <c r="B6" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C6" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D6" s="92" t="inlineStr">
+        <is>
+          <t>出荷梱包 手伝い</t>
+        </is>
+      </c>
+      <c r="E6" s="91" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="F6" s="91" t="inlineStr">
+        <is>
+          <t>9:14</t>
+        </is>
+      </c>
+      <c r="G6" s="91" t="n">
+        <v>59</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C7" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D7" s="85" t="inlineStr">
+        <is>
+          <t>製品検査 立ち会い確認</t>
+        </is>
+      </c>
+      <c r="E7" s="84" t="inlineStr">
+        <is>
+          <t>9:14</t>
+        </is>
+      </c>
+      <c r="F7" s="84" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G7" s="84" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="20" customHeight="1" s="64">
+      <c r="B9" s="90" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="B10" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C10" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D10" s="79" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E10" s="79" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F10" s="79" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+      <c r="G10" s="79" t="n"/>
+    </row>
+    <row r="11">
+      <c r="B11" s="88" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C11" s="89" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D11" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="88" t="n">
+        <v>0</v>
+      </c>
+      <c r="G11" s="88" t="n"/>
+    </row>
+    <row r="12">
+      <c r="B12" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C12" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D12" s="82" t="n">
+        <v>3</v>
+      </c>
+      <c r="E12" s="82" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F12" s="82" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G12" s="82" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C13" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D13" s="84" t="n">
+        <v>9</v>
+      </c>
+      <c r="E13" s="84" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F13" s="84" t="n">
+        <v>12.2</v>
+      </c>
+      <c r="G13" s="84" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C14" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D14" s="91" t="n">
+        <v>59</v>
+      </c>
+      <c r="E14" s="91" t="n">
+        <v>1</v>
+      </c>
+      <c r="F14" s="91" t="n">
+        <v>79.7</v>
+      </c>
+      <c r="G14" s="91" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C15" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D15" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" s="86" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C16" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D16" s="80" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" s="80" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F16" s="80" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="G16" s="80" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="79" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="C17" s="90" t="n"/>
+      <c r="D17" s="79" t="n">
+        <v>74</v>
+      </c>
+      <c r="E17" s="79" t="n">
+        <v>1.2</v>
+      </c>
+      <c r="F17" s="79" t="n">
+        <v>100</v>
+      </c>
+      <c r="G17" s="79" t="n"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B9:G9"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-29: inspection, loading, cleanup/consultation, break
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -12361,7 +12361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G17"/>
+  <dimension ref="B1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -12555,203 +12555,293 @@
       </c>
       <c r="F7" s="84" t="inlineStr">
         <is>
+          <t>9:30</t>
+        </is>
+      </c>
+      <c r="G7" s="84" t="n">
+        <v>16</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C8" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D8" s="92" t="inlineStr">
+        <is>
+          <t>荷下ろし・荷積み</t>
+        </is>
+      </c>
+      <c r="E8" s="91" t="inlineStr">
+        <is>
+          <t>9:30</t>
+        </is>
+      </c>
+      <c r="F8" s="91" t="inlineStr">
+        <is>
+          <t>9:50</t>
+        </is>
+      </c>
+      <c r="G8" s="91" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="82" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C9" s="83" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D9" s="83" t="inlineStr">
+        <is>
+          <t>現場掃除・廃棄方法相談（副リーダー）</t>
+        </is>
+      </c>
+      <c r="E9" s="82" t="inlineStr">
+        <is>
+          <t>9:50</t>
+        </is>
+      </c>
+      <c r="F9" s="82" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="G9" s="82" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C10" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D10" s="81" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E10" s="80" t="inlineStr">
+        <is>
+          <t>10:04</t>
+        </is>
+      </c>
+      <c r="F10" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G7" s="84" t="inlineStr">
+      <c r="G10" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="20" customHeight="1" s="64">
-      <c r="B9" s="90" t="inlineStr">
+    <row r="12" ht="20" customHeight="1" s="64">
+      <c r="B12" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="B10" s="79" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C10" s="79" t="inlineStr">
+      <c r="C13" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D10" s="79" t="inlineStr">
+      <c r="D13" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E10" s="79" t="inlineStr">
+      <c r="E13" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F10" s="79" t="inlineStr">
+      <c r="F13" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G10" s="79" t="n"/>
-    </row>
-    <row r="11">
-      <c r="B11" s="88" t="inlineStr">
+      <c r="G13" s="79" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C11" s="89" t="inlineStr">
+      <c r="C14" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D11" s="88" t="n">
+      <c r="D14" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="88" t="n">
+      <c r="E14" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="88" t="n">
+      <c r="F14" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G11" s="88" t="n"/>
-    </row>
-    <row r="12">
-      <c r="B12" s="82" t="inlineStr">
+      <c r="G14" s="88" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C12" s="83" t="inlineStr">
+      <c r="C15" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D12" s="82" t="n">
+      <c r="D15" s="82" t="n">
+        <v>17</v>
+      </c>
+      <c r="E15" s="82" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F15" s="82" t="n">
+        <v>13.7</v>
+      </c>
+      <c r="G15" s="82" t="n"/>
+    </row>
+    <row r="16">
+      <c r="B16" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C16" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D16" s="84" t="n">
+        <v>25</v>
+      </c>
+      <c r="E16" s="84" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F16" s="84" t="n">
+        <v>20.2</v>
+      </c>
+      <c r="G16" s="84" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="91" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C17" s="92" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D17" s="91" t="n">
+        <v>79</v>
+      </c>
+      <c r="E17" s="91" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F17" s="91" t="n">
+        <v>63.7</v>
+      </c>
+      <c r="G17" s="91" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C18" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D18" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="86" t="n">
+        <v>0</v>
+      </c>
+      <c r="G18" s="86" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C19" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D19" s="80" t="n">
         <v>3</v>
       </c>
-      <c r="E12" s="82" t="n">
+      <c r="E19" s="80" t="n">
         <v>0.1</v>
       </c>
-      <c r="F12" s="82" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="G12" s="82" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="84" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C13" s="85" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D13" s="84" t="n">
-        <v>9</v>
-      </c>
-      <c r="E13" s="84" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F13" s="84" t="n">
-        <v>12.2</v>
-      </c>
-      <c r="G13" s="84" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="91" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C14" s="92" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D14" s="91" t="n">
-        <v>59</v>
-      </c>
-      <c r="E14" s="91" t="n">
-        <v>1</v>
-      </c>
-      <c r="F14" s="91" t="n">
-        <v>79.7</v>
-      </c>
-      <c r="G14" s="91" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="86" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C15" s="87" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D15" s="86" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" s="86" t="n">
-        <v>0</v>
-      </c>
-      <c r="F15" s="86" t="n">
-        <v>0</v>
-      </c>
-      <c r="G15" s="86" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="80" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="C16" s="81" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D16" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="E16" s="80" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F16" s="80" t="n">
-        <v>4.1</v>
-      </c>
-      <c r="G16" s="80" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="79" t="inlineStr">
+      <c r="F19" s="80" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="G19" s="80" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C17" s="90" t="n"/>
-      <c r="D17" s="79" t="n">
-        <v>74</v>
-      </c>
-      <c r="E17" s="79" t="n">
-        <v>1.2</v>
-      </c>
-      <c r="F17" s="79" t="n">
+      <c r="C20" s="90" t="n"/>
+      <c r="D20" s="79" t="n">
+        <v>124</v>
+      </c>
+      <c r="E20" s="79" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F20" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G17" s="79" t="n"/>
+      <c r="G20" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B9:G9"/>
+    <mergeCell ref="B12:G12"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-29: add tasks through 15:01 break
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -12361,7 +12361,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G20"/>
+  <dimension ref="B1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -12645,203 +12645,383 @@
       </c>
       <c r="F10" s="80" t="inlineStr">
         <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G10" s="80" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C11" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D11" s="87" t="inlineStr">
+        <is>
+          <t>見積もり業務</t>
+        </is>
+      </c>
+      <c r="E11" s="86" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F11" s="86" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="G11" s="86" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="81" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E12" s="80" t="inlineStr">
+        <is>
+          <t>12:10</t>
+        </is>
+      </c>
+      <c r="F12" s="80" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="G12" s="80" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="81" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E13" s="80" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F13" s="80" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="G13" s="80" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="84" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C14" s="85" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D14" s="85" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E14" s="84" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="F14" s="84" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="G14" s="84" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="86" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C15" s="87" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D15" s="87" t="inlineStr">
+        <is>
+          <t>メールチェック・見積もり確認・治具データ整理</t>
+        </is>
+      </c>
+      <c r="E15" s="86" t="inlineStr">
+        <is>
+          <t>13:05</t>
+        </is>
+      </c>
+      <c r="F15" s="86" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="G15" s="86" t="n">
+        <v>116</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="80" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C16" s="81" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D16" s="81" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E16" s="80" t="inlineStr">
+        <is>
+          <t>15:01</t>
+        </is>
+      </c>
+      <c r="F16" s="80" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G10" s="80" t="inlineStr">
+      <c r="G16" s="80" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="20" customHeight="1" s="64">
-      <c r="B12" s="90" t="inlineStr">
+    <row r="18" ht="20" customHeight="1" s="64">
+      <c r="B18" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="79" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C13" s="79" t="inlineStr">
+      <c r="C19" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D13" s="79" t="inlineStr">
+      <c r="D19" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E13" s="79" t="inlineStr">
+      <c r="E19" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F13" s="79" t="inlineStr">
+      <c r="F19" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G13" s="79" t="n"/>
-    </row>
-    <row r="14">
-      <c r="B14" s="88" t="inlineStr">
+      <c r="G19" s="79" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C14" s="89" t="inlineStr">
+      <c r="C20" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D14" s="88" t="n">
+      <c r="D20" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="88" t="n">
+      <c r="E20" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="88" t="n">
+      <c r="F20" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G14" s="88" t="n"/>
-    </row>
-    <row r="15">
-      <c r="B15" s="82" t="inlineStr">
+      <c r="G20" s="88" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C15" s="83" t="inlineStr">
+      <c r="C21" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D15" s="82" t="n">
+      <c r="D21" s="82" t="n">
         <v>17</v>
       </c>
-      <c r="E15" s="82" t="n">
+      <c r="E21" s="82" t="n">
         <v>0.3</v>
       </c>
-      <c r="F15" s="82" t="n">
-        <v>13.7</v>
-      </c>
-      <c r="G15" s="82" t="n"/>
-    </row>
-    <row r="16">
-      <c r="B16" s="84" t="inlineStr">
+      <c r="F21" s="82" t="n">
+        <v>4</v>
+      </c>
+      <c r="G21" s="82" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C16" s="85" t="inlineStr">
+      <c r="C22" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D16" s="84" t="n">
-        <v>25</v>
-      </c>
-      <c r="E16" s="84" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F16" s="84" t="n">
-        <v>20.2</v>
-      </c>
-      <c r="G16" s="84" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="91" t="inlineStr">
+      <c r="D22" s="84" t="n">
+        <v>35</v>
+      </c>
+      <c r="E22" s="84" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F22" s="84" t="n">
+        <v>8.300000000000001</v>
+      </c>
+      <c r="G22" s="84" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C17" s="92" t="inlineStr">
+      <c r="C23" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D17" s="91" t="n">
+      <c r="D23" s="91" t="n">
         <v>79</v>
       </c>
-      <c r="E17" s="91" t="n">
+      <c r="E23" s="91" t="n">
         <v>1.3</v>
       </c>
-      <c r="F17" s="91" t="n">
-        <v>63.7</v>
-      </c>
-      <c r="G17" s="91" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="86" t="inlineStr">
+      <c r="F23" s="91" t="n">
+        <v>18.8</v>
+      </c>
+      <c r="G23" s="91" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C18" s="87" t="inlineStr">
+      <c r="C24" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D18" s="86" t="n">
-        <v>0</v>
-      </c>
-      <c r="E18" s="86" t="n">
-        <v>0</v>
-      </c>
-      <c r="F18" s="86" t="n">
-        <v>0</v>
-      </c>
-      <c r="G18" s="86" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="80" t="inlineStr">
+      <c r="D24" s="86" t="n">
+        <v>236</v>
+      </c>
+      <c r="E24" s="86" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F24" s="86" t="n">
+        <v>56.1</v>
+      </c>
+      <c r="G24" s="86" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C19" s="81" t="inlineStr">
+      <c r="C25" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D19" s="80" t="n">
-        <v>3</v>
-      </c>
-      <c r="E19" s="80" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F19" s="80" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="G19" s="80" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="79" t="inlineStr">
+      <c r="D25" s="80" t="n">
+        <v>54</v>
+      </c>
+      <c r="E25" s="80" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F25" s="80" t="n">
+        <v>12.8</v>
+      </c>
+      <c r="G25" s="80" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C20" s="90" t="n"/>
-      <c r="D20" s="79" t="n">
-        <v>124</v>
-      </c>
-      <c r="E20" s="79" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="F20" s="79" t="n">
+      <c r="C26" s="90" t="n"/>
+      <c r="D26" s="79" t="n">
+        <v>421</v>
+      </c>
+      <c r="E26" s="79" t="n">
+        <v>7</v>
+      </c>
+      <c r="F26" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G20" s="79" t="n"/>
+      <c r="G26" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">
-    <mergeCell ref="B12:G12"/>
+    <mergeCell ref="B18:G18"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-05-29: close break 15:01-15:10, start 品質会議 15:10
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -176,7 +176,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="27">
+  <fonts count="28">
     <font>
       <name val="游ゴシック"/>
       <family val="2"/>
@@ -354,6 +354,10 @@
     </font>
     <font>
       <color rgb="00C55A11"/>
+      <sz val="11"/>
+    </font>
+    <font>
+      <color rgb="00000000"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -646,7 +650,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="95">
+  <cellXfs count="98">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -874,6 +878,15 @@
     </xf>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="15" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="0" borderId="16" pivotButton="0" quotePrefix="0" xfId="0"/>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="標準" xfId="0" builtinId="0"/>
@@ -12361,7 +12374,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G26"/>
+  <dimension ref="A1:G26"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -12379,6 +12392,11 @@
           <t>2026年5月29日（金）　業務記録</t>
         </is>
       </c>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="94" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1" s="64">
       <c r="B2" s="79" t="inlineStr">
@@ -12823,16 +12841,42 @@
           <t>15:01</t>
         </is>
       </c>
-      <c r="F16" s="80" t="inlineStr">
+      <c r="F16" s="95" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="G16" s="95" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C17" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
+        <is>
+          <t>品質会議</t>
+        </is>
+      </c>
+      <c r="E17" s="96" t="inlineStr">
+        <is>
+          <t>15:10</t>
+        </is>
+      </c>
+      <c r="F17" s="96" t="inlineStr">
         <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G16" s="80" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
+      <c r="G17" s="96" t="n"/>
     </row>
     <row r="18" ht="20" customHeight="1" s="64">
       <c r="B18" s="90" t="inlineStr">
@@ -12840,6 +12884,11 @@
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
+      <c r="C18" s="93" t="n"/>
+      <c r="D18" s="93" t="n"/>
+      <c r="E18" s="93" t="n"/>
+      <c r="F18" s="93" t="n"/>
+      <c r="G18" s="94" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="79" t="inlineStr">

</xml_diff>

<commit_message>
Update 2026-05-29: close 品質会議 15:10-16:40 (90分)
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -12873,10 +12873,12 @@
       </c>
       <c r="F17" s="96" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G17" s="96" t="n"/>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="G17" s="96" t="n">
+        <v>90</v>
+      </c>
     </row>
     <row r="18" ht="20" customHeight="1" s="64">
       <c r="B18" s="90" t="inlineStr">

</xml_diff>

<commit_message>
Update 2026-05-29: 現場周り 16:40-17:10, start メールチェック 17:10
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -650,7 +650,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="98">
+  <cellXfs count="102">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -885,6 +885,18 @@
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="0" fontId="27" fillId="16" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="17" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="18" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
@@ -12374,7 +12386,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G26"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -12881,194 +12893,252 @@
       </c>
     </row>
     <row r="18" ht="20" customHeight="1" s="64">
-      <c r="B18" s="90" t="inlineStr">
+      <c r="B18" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C18" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D18" s="99" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E18" s="98" t="inlineStr">
+        <is>
+          <t>16:40</t>
+        </is>
+      </c>
+      <c r="F18" s="98" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="G18" s="98" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック</t>
+        </is>
+      </c>
+      <c r="E19" s="100" t="inlineStr">
+        <is>
+          <t>17:10</t>
+        </is>
+      </c>
+      <c r="F19" s="100" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G19" s="100" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="90" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C18" s="93" t="n"/>
-      <c r="D18" s="93" t="n"/>
-      <c r="E18" s="93" t="n"/>
-      <c r="F18" s="93" t="n"/>
-      <c r="G18" s="94" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="79" t="inlineStr">
+      <c r="C20" s="93" t="n"/>
+      <c r="D20" s="93" t="n"/>
+      <c r="E20" s="93" t="n"/>
+      <c r="F20" s="93" t="n"/>
+      <c r="G20" s="94" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C19" s="79" t="inlineStr">
+      <c r="C21" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D19" s="79" t="inlineStr">
+      <c r="D21" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E19" s="79" t="inlineStr">
+      <c r="E21" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F19" s="79" t="inlineStr">
+      <c r="F21" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
-      <c r="G19" s="79" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="88" t="inlineStr">
+      <c r="G21" s="79" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="88" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C20" s="89" t="inlineStr">
+      <c r="C22" s="89" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D20" s="88" t="n">
+      <c r="D22" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="88" t="n">
+      <c r="E22" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="88" t="n">
+      <c r="F22" s="88" t="n">
         <v>0</v>
       </c>
-      <c r="G20" s="88" t="n"/>
-    </row>
-    <row r="21">
-      <c r="B21" s="82" t="inlineStr">
+      <c r="G22" s="88" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="82" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C21" s="83" t="inlineStr">
+      <c r="C23" s="83" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D21" s="82" t="n">
-        <v>17</v>
-      </c>
-      <c r="E21" s="82" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F21" s="82" t="n">
-        <v>4</v>
-      </c>
-      <c r="G21" s="82" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="84" t="inlineStr">
+      <c r="D23" s="82" t="n">
+        <v>107</v>
+      </c>
+      <c r="E23" s="82" t="n">
+        <v>1.8</v>
+      </c>
+      <c r="F23" s="82" t="n">
+        <v>19.5</v>
+      </c>
+      <c r="G23" s="82" t="n"/>
+    </row>
+    <row r="24">
+      <c r="B24" s="84" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C22" s="85" t="inlineStr">
+      <c r="C24" s="85" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D22" s="84" t="n">
-        <v>35</v>
-      </c>
-      <c r="E22" s="84" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F22" s="84" t="n">
-        <v>8.300000000000001</v>
-      </c>
-      <c r="G22" s="84" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="91" t="inlineStr">
+      <c r="D24" s="84" t="n">
+        <v>65</v>
+      </c>
+      <c r="E24" s="84" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F24" s="84" t="n">
+        <v>11.8</v>
+      </c>
+      <c r="G24" s="84" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="91" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C23" s="92" t="inlineStr">
+      <c r="C25" s="92" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D23" s="91" t="n">
+      <c r="D25" s="91" t="n">
         <v>79</v>
       </c>
-      <c r="E23" s="91" t="n">
+      <c r="E25" s="91" t="n">
         <v>1.3</v>
       </c>
-      <c r="F23" s="91" t="n">
-        <v>18.8</v>
-      </c>
-      <c r="G23" s="91" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="86" t="inlineStr">
+      <c r="F25" s="91" t="n">
+        <v>14.4</v>
+      </c>
+      <c r="G25" s="91" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="86" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C24" s="87" t="inlineStr">
+      <c r="C26" s="87" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D24" s="86" t="n">
+      <c r="D26" s="86" t="n">
         <v>236</v>
       </c>
-      <c r="E24" s="86" t="n">
+      <c r="E26" s="86" t="n">
         <v>3.9</v>
       </c>
-      <c r="F24" s="86" t="n">
-        <v>56.1</v>
-      </c>
-      <c r="G24" s="86" t="n"/>
-    </row>
-    <row r="25">
-      <c r="B25" s="80" t="inlineStr">
+      <c r="F26" s="86" t="n">
+        <v>42.9</v>
+      </c>
+      <c r="G26" s="86" t="n"/>
+    </row>
+    <row r="27">
+      <c r="B27" s="80" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C25" s="81" t="inlineStr">
+      <c r="C27" s="81" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D25" s="80" t="n">
-        <v>54</v>
-      </c>
-      <c r="E25" s="80" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="F25" s="80" t="n">
-        <v>12.8</v>
-      </c>
-      <c r="G25" s="80" t="n"/>
-    </row>
-    <row r="26">
-      <c r="B26" s="79" t="inlineStr">
+      <c r="D27" s="80" t="n">
+        <v>63</v>
+      </c>
+      <c r="E27" s="80" t="n">
+        <v>1.1</v>
+      </c>
+      <c r="F27" s="80" t="n">
+        <v>11.5</v>
+      </c>
+      <c r="G27" s="80" t="n"/>
+    </row>
+    <row r="28">
+      <c r="B28" s="79" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="C26" s="90" t="n"/>
-      <c r="D26" s="79" t="n">
-        <v>421</v>
-      </c>
-      <c r="E26" s="79" t="n">
-        <v>7</v>
-      </c>
-      <c r="F26" s="79" t="n">
+      <c r="C28" s="90" t="n"/>
+      <c r="D28" s="79" t="n">
+        <v>550</v>
+      </c>
+      <c r="E28" s="79" t="n">
+        <v>9.199999999999999</v>
+      </c>
+      <c r="F28" s="79" t="n">
         <v>100</v>
       </c>
-      <c r="G26" s="79" t="n"/>
+      <c r="G28" s="79" t="n"/>
     </row>
   </sheetData>
   <mergeCells count="2">

</xml_diff>

<commit_message>
Add 2026-06-01: new sheet, tasks 8:00-10:25, PCデータ整理 in progress
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -21,14 +21,15 @@
     <sheet name="2026-05-27" sheetId="13" state="visible" r:id="rId13"/>
     <sheet name="2026-05-28" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-05-29" sheetId="15" state="visible" r:id="rId15"/>
+    <sheet name="2026-06-01" sheetId="16" state="visible" r:id="rId16"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId16"/>
     <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
     <externalReference r:id="rId19"/>
     <externalReference r:id="rId20"/>
     <externalReference r:id="rId21"/>
+    <externalReference r:id="rId22"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -176,7 +177,7 @@
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <numFmts count="0"/>
-  <fonts count="28">
+  <fonts count="30">
     <font>
       <name val="游ゴシック"/>
       <family val="2"/>
@@ -360,8 +361,18 @@
       <color rgb="00000000"/>
       <sz val="11"/>
     </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00FFFFFF"/>
+      <sz val="13"/>
+    </font>
+    <font>
+      <b val="1"/>
+      <color rgb="00000000"/>
+      <sz val="11"/>
+    </font>
   </fonts>
-  <fills count="21">
+  <fills count="22">
     <fill>
       <patternFill/>
     </fill>
@@ -480,6 +491,12 @@
       <patternFill patternType="solid">
         <fgColor rgb="00FCE4D6"/>
         <bgColor rgb="00FCE4D6"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="00D9E1F2"/>
+        <bgColor rgb="00D9E1F2"/>
       </patternFill>
     </fill>
   </fills>
@@ -650,7 +667,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="102">
+  <cellXfs count="108">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -898,6 +915,24 @@
     </xf>
     <xf numFmtId="0" fontId="27" fillId="18" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="28" fillId="13" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="15" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="20" fillId="13" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="19" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="29" fillId="21" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -12386,7 +12421,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="B1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="2" customWidth="1" style="64" min="1" max="1"/>
@@ -12898,29 +12933,11 @@
           <t>③</t>
         </is>
       </c>
-      <c r="C18" s="98" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D18" s="99" t="inlineStr">
-        <is>
-          <t>現場周り</t>
-        </is>
-      </c>
-      <c r="E18" s="98" t="inlineStr">
-        <is>
-          <t>16:40</t>
-        </is>
-      </c>
-      <c r="F18" s="98" t="inlineStr">
-        <is>
-          <t>17:10</t>
-        </is>
-      </c>
-      <c r="G18" s="98" t="n">
-        <v>30</v>
-      </c>
+      <c r="C18" s="93" t="n"/>
+      <c r="D18" s="93" t="n"/>
+      <c r="E18" s="93" t="n"/>
+      <c r="F18" s="93" t="n"/>
+      <c r="G18" s="94" t="n"/>
     </row>
     <row r="19">
       <c r="B19" s="100" t="inlineStr">
@@ -13143,6 +13160,515 @@
   </sheetData>
   <mergeCells count="2">
     <mergeCell ref="B18:G18"/>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet16.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G20"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="64" min="2" max="2"/>
+    <col width="18" customWidth="1" style="64" min="3" max="3"/>
+    <col width="42" customWidth="1" style="64" min="4" max="4"/>
+    <col width="8" customWidth="1" style="64" min="5" max="5"/>
+    <col width="8" customWidth="1" style="64" min="6" max="6"/>
+    <col width="12" customWidth="1" style="64" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" s="64">
+      <c r="B1" s="102" t="inlineStr">
+        <is>
+          <t>2026年6月1日（月）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="64">
+      <c r="B2" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C2" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D2" s="79" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E2" s="79" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F2" s="79" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G2" s="79" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="64">
+      <c r="B3" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C3" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D3" s="97" t="inlineStr">
+        <is>
+          <t>全体朝礼</t>
+        </is>
+      </c>
+      <c r="E3" s="96" t="inlineStr">
+        <is>
+          <t>8:00</t>
+        </is>
+      </c>
+      <c r="F3" s="96" t="inlineStr">
+        <is>
+          <t>8:20</t>
+        </is>
+      </c>
+      <c r="G3" s="96" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="64">
+      <c r="B4" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C4" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D4" s="103" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E4" s="95" t="inlineStr">
+        <is>
+          <t>8:20</t>
+        </is>
+      </c>
+      <c r="F4" s="95" t="inlineStr">
+        <is>
+          <t>8:23</t>
+        </is>
+      </c>
+      <c r="G4" s="95" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="64">
+      <c r="B5" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C5" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D5" s="97" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E5" s="96" t="inlineStr">
+        <is>
+          <t>8:23</t>
+        </is>
+      </c>
+      <c r="F5" s="96" t="inlineStr">
+        <is>
+          <t>8:26</t>
+        </is>
+      </c>
+      <c r="G5" s="96" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="64">
+      <c r="B6" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C6" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D6" s="99" t="inlineStr">
+        <is>
+          <t>工場周り</t>
+        </is>
+      </c>
+      <c r="E6" s="98" t="inlineStr">
+        <is>
+          <t>8:26</t>
+        </is>
+      </c>
+      <c r="F6" s="98" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="G6" s="98" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C7" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D7" s="101" t="inlineStr">
+        <is>
+          <t>事務処理</t>
+        </is>
+      </c>
+      <c r="E7" s="100" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="F7" s="100" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="G7" s="100" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C8" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D8" s="97" t="inlineStr">
+        <is>
+          <t>朝礼（月次全体会議）</t>
+        </is>
+      </c>
+      <c r="E8" s="96" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="F8" s="96" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="G8" s="96" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C9" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D9" s="103" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E9" s="95" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F9" s="95" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G9" s="95" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C10" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D10" s="101" t="inlineStr">
+        <is>
+          <t>事務処理（改善提案コメント記入）</t>
+        </is>
+      </c>
+      <c r="E10" s="100" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F10" s="100" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="G10" s="100" t="n">
+        <v>15</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C11" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D11" s="101" t="inlineStr">
+        <is>
+          <t>PCデータ整理</t>
+        </is>
+      </c>
+      <c r="E11" s="100" t="inlineStr">
+        <is>
+          <t>10:25</t>
+        </is>
+      </c>
+      <c r="F11" s="100" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G11" s="100" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="104" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C13" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D13" s="79" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E13" s="79" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F13" s="79" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="105" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C14" s="105" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D14" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C15" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D15" s="96" t="n">
+        <v>83</v>
+      </c>
+      <c r="E15" s="96" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F15" s="96" t="n">
+        <v>57.2</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C16" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D16" s="98" t="n">
+        <v>19</v>
+      </c>
+      <c r="E16" s="98" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F16" s="98" t="n">
+        <v>13.1</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C17" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D17" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F17" s="106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C18" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D18" s="100" t="n">
+        <v>30</v>
+      </c>
+      <c r="E18" s="100" t="n">
+        <v>0.5</v>
+      </c>
+      <c r="F18" s="100" t="n">
+        <v>20.7</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C19" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D19" s="95" t="n">
+        <v>13</v>
+      </c>
+      <c r="E19" s="95" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F19" s="95" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="107" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="D20" s="107" t="n">
+        <v>145</v>
+      </c>
+      <c r="E20" s="107" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F20" s="107" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B12:G12"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-06-01: close PCデータ整理 10:25-10:29, start 治具確認 10:29
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -13172,7 +13172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G20"/>
+  <dimension ref="A1:G21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -13189,6 +13189,11 @@
           <t>2026年6月1日（月）　業務記録</t>
         </is>
       </c>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="94" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1" s="64">
       <c r="B2" s="79" t="inlineStr">
@@ -13485,184 +13490,219 @@
       </c>
       <c r="F11" s="100" t="inlineStr">
         <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="G11" s="100" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C12" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D12" s="99" t="inlineStr">
+        <is>
+          <t>治具確認</t>
+        </is>
+      </c>
+      <c r="E12" s="98" t="inlineStr">
+        <is>
+          <t>10:29</t>
+        </is>
+      </c>
+      <c r="F12" s="98" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G11" s="100" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="104" t="inlineStr">
+      <c r="G12" s="98" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="79" t="inlineStr">
+      <c r="C13" s="93" t="n"/>
+      <c r="D13" s="93" t="n"/>
+      <c r="E13" s="93" t="n"/>
+      <c r="F13" s="93" t="n"/>
+      <c r="G13" s="94" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C13" s="79" t="inlineStr">
+      <c r="C14" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D13" s="79" t="inlineStr">
+      <c r="D14" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E13" s="79" t="inlineStr">
+      <c r="E14" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F13" s="79" t="inlineStr">
+      <c r="F14" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="105" t="inlineStr">
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C14" s="105" t="inlineStr">
+      <c r="C15" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D14" s="105" t="n">
+      <c r="D15" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="105" t="n">
+      <c r="E15" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="105" t="n">
+      <c r="F15" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="96" t="inlineStr">
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C15" s="96" t="inlineStr">
+      <c r="C16" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D15" s="96" t="n">
+      <c r="D16" s="96" t="n">
         <v>83</v>
       </c>
-      <c r="E15" s="96" t="n">
+      <c r="E16" s="96" t="n">
         <v>1.4</v>
       </c>
-      <c r="F15" s="96" t="n">
+      <c r="F16" s="96" t="n">
         <v>57.2</v>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="98" t="inlineStr">
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C16" s="98" t="inlineStr">
+      <c r="C17" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D16" s="98" t="n">
+      <c r="D17" s="98" t="n">
         <v>19</v>
       </c>
-      <c r="E16" s="98" t="n">
+      <c r="E17" s="98" t="n">
         <v>0.3</v>
       </c>
-      <c r="F16" s="98" t="n">
+      <c r="F17" s="98" t="n">
         <v>13.1</v>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" s="64">
-      <c r="B17" s="106" t="inlineStr">
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C17" s="106" t="inlineStr">
+      <c r="C18" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D17" s="106" t="n">
+      <c r="D18" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="106" t="n">
+      <c r="E18" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="106" t="n">
+      <c r="F18" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" s="64">
-      <c r="B18" s="100" t="inlineStr">
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C18" s="100" t="inlineStr">
+      <c r="C19" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D18" s="100" t="n">
+      <c r="D19" s="100" t="n">
         <v>30</v>
       </c>
-      <c r="E18" s="100" t="n">
+      <c r="E19" s="100" t="n">
         <v>0.5</v>
       </c>
-      <c r="F18" s="100" t="n">
+      <c r="F19" s="100" t="n">
         <v>20.7</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" s="64">
-      <c r="B19" s="95" t="inlineStr">
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C19" s="95" t="inlineStr">
+      <c r="C20" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D19" s="95" t="n">
+      <c r="D20" s="95" t="n">
         <v>13</v>
       </c>
-      <c r="E19" s="95" t="n">
+      <c r="E20" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F19" s="95" t="n">
+      <c r="F20" s="95" t="n">
         <v>9</v>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1" s="64">
-      <c r="B20" s="107" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D20" s="107" t="n">
+      <c r="D21" s="107" t="n">
         <v>145</v>
       </c>
-      <c r="E20" s="107" t="n">
+      <c r="E21" s="107" t="n">
         <v>2.4</v>
       </c>
-      <c r="F20" s="107" t="n">
+      <c r="F21" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-01: fix 治具確認 10:29-10:55, restart PCデータ整理 10:55
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -13172,7 +13172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -13520,195 +13520,224 @@
       </c>
       <c r="F12" s="98" t="inlineStr">
         <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="G12" s="98" t="n">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C13" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D13" s="101" t="inlineStr">
+        <is>
+          <t>PCデータ整理</t>
+        </is>
+      </c>
+      <c r="E13" s="100" t="inlineStr">
+        <is>
+          <t>10:55</t>
+        </is>
+      </c>
+      <c r="F13" s="100" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G12" s="98" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="104" t="inlineStr">
+      <c r="G13" s="100" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C13" s="93" t="n"/>
-      <c r="D13" s="93" t="n"/>
-      <c r="E13" s="93" t="n"/>
-      <c r="F13" s="93" t="n"/>
-      <c r="G13" s="94" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="79" t="inlineStr">
+      <c r="C14" s="93" t="n"/>
+      <c r="D14" s="93" t="n"/>
+      <c r="E14" s="93" t="n"/>
+      <c r="F14" s="93" t="n"/>
+      <c r="G14" s="94" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C14" s="79" t="inlineStr">
+      <c r="C15" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D14" s="79" t="inlineStr">
+      <c r="D15" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E14" s="79" t="inlineStr">
+      <c r="E15" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F14" s="79" t="inlineStr">
+      <c r="F15" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="105" t="inlineStr">
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C15" s="105" t="inlineStr">
+      <c r="C16" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D15" s="105" t="n">
+      <c r="D16" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="105" t="n">
+      <c r="E16" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="105" t="n">
+      <c r="F16" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="96" t="inlineStr">
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C16" s="96" t="inlineStr">
+      <c r="C17" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D16" s="96" t="n">
+      <c r="D17" s="96" t="n">
         <v>83</v>
       </c>
-      <c r="E16" s="96" t="n">
+      <c r="E17" s="96" t="n">
         <v>1.4</v>
       </c>
-      <c r="F16" s="96" t="n">
-        <v>57.2</v>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1" s="64">
-      <c r="B17" s="98" t="inlineStr">
+      <c r="F17" s="96" t="n">
+        <v>47.4</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C17" s="98" t="inlineStr">
+      <c r="C18" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D17" s="98" t="n">
-        <v>19</v>
-      </c>
-      <c r="E17" s="98" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F17" s="98" t="n">
-        <v>13.1</v>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="64">
-      <c r="B18" s="106" t="inlineStr">
+      <c r="D18" s="98" t="n">
+        <v>45</v>
+      </c>
+      <c r="E18" s="98" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F18" s="98" t="n">
+        <v>25.7</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C18" s="106" t="inlineStr">
+      <c r="C19" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D18" s="106" t="n">
+      <c r="D19" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="106" t="n">
+      <c r="E19" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="106" t="n">
+      <c r="F19" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" s="64">
-      <c r="B19" s="100" t="inlineStr">
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C19" s="100" t="inlineStr">
+      <c r="C20" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D19" s="100" t="n">
-        <v>30</v>
-      </c>
-      <c r="E19" s="100" t="n">
-        <v>0.5</v>
-      </c>
-      <c r="F19" s="100" t="n">
-        <v>20.7</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" s="64">
-      <c r="B20" s="95" t="inlineStr">
+      <c r="D20" s="100" t="n">
+        <v>34</v>
+      </c>
+      <c r="E20" s="100" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F20" s="100" t="n">
+        <v>19.4</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C20" s="95" t="inlineStr">
+      <c r="C21" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D20" s="95" t="n">
+      <c r="D21" s="95" t="n">
         <v>13</v>
       </c>
-      <c r="E20" s="95" t="n">
+      <c r="E21" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F20" s="95" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="107" t="inlineStr">
+      <c r="F21" s="95" t="n">
+        <v>7.4</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D21" s="107" t="n">
-        <v>145</v>
-      </c>
-      <c r="E21" s="107" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="F21" s="107" t="n">
+      <c r="D22" s="107" t="n">
+        <v>175</v>
+      </c>
+      <c r="E22" s="107" t="n">
+        <v>2.9</v>
+      </c>
+      <c r="F22" s="107" t="n">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B12:G12"/>
+  <mergeCells count="1">
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-06-01: close PCデータ整理 10:55-11:20, start 新人社員教育資料準備 11:20
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -13172,7 +13172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -13550,189 +13550,219 @@
       </c>
       <c r="F13" s="100" t="inlineStr">
         <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="G13" s="100" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C14" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D14" s="97" t="inlineStr">
+        <is>
+          <t>新人社員教育 資料準備</t>
+        </is>
+      </c>
+      <c r="E14" s="96" t="inlineStr">
+        <is>
+          <t>11:20</t>
+        </is>
+      </c>
+      <c r="F14" s="96" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G13" s="100" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="104" t="inlineStr">
+      <c r="G14" s="96" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C14" s="93" t="n"/>
-      <c r="D14" s="93" t="n"/>
-      <c r="E14" s="93" t="n"/>
-      <c r="F14" s="93" t="n"/>
-      <c r="G14" s="94" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="79" t="inlineStr">
+      <c r="C15" s="93" t="n"/>
+      <c r="D15" s="93" t="n"/>
+      <c r="E15" s="93" t="n"/>
+      <c r="F15" s="93" t="n"/>
+      <c r="G15" s="94" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C15" s="79" t="inlineStr">
+      <c r="C16" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D15" s="79" t="inlineStr">
+      <c r="D16" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E15" s="79" t="inlineStr">
+      <c r="E16" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F15" s="79" t="inlineStr">
+      <c r="F16" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="105" t="inlineStr">
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C16" s="105" t="inlineStr">
+      <c r="C17" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D16" s="105" t="n">
+      <c r="D17" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="105" t="n">
+      <c r="E17" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="105" t="n">
+      <c r="F17" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" s="64">
-      <c r="B17" s="96" t="inlineStr">
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C17" s="96" t="inlineStr">
+      <c r="C18" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D17" s="96" t="n">
+      <c r="D18" s="96" t="n">
         <v>83</v>
       </c>
-      <c r="E17" s="96" t="n">
+      <c r="E18" s="96" t="n">
         <v>1.4</v>
       </c>
-      <c r="F17" s="96" t="n">
-        <v>47.4</v>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="64">
-      <c r="B18" s="98" t="inlineStr">
+      <c r="F18" s="96" t="n">
+        <v>41.5</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C18" s="98" t="inlineStr">
+      <c r="C19" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D18" s="98" t="n">
+      <c r="D19" s="98" t="n">
         <v>45</v>
       </c>
-      <c r="E18" s="98" t="n">
+      <c r="E19" s="98" t="n">
         <v>0.8</v>
       </c>
-      <c r="F18" s="98" t="n">
-        <v>25.7</v>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1" s="64">
-      <c r="B19" s="106" t="inlineStr">
+      <c r="F19" s="98" t="n">
+        <v>22.5</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C19" s="106" t="inlineStr">
+      <c r="C20" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D19" s="106" t="n">
+      <c r="D20" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="106" t="n">
+      <c r="E20" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="106" t="n">
+      <c r="F20" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="20" ht="18" customHeight="1" s="64">
-      <c r="B20" s="100" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C20" s="100" t="inlineStr">
+      <c r="C21" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D20" s="100" t="n">
-        <v>34</v>
-      </c>
-      <c r="E20" s="100" t="n">
-        <v>0.6</v>
-      </c>
-      <c r="F20" s="100" t="n">
-        <v>19.4</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="95" t="inlineStr">
+      <c r="D21" s="100" t="n">
+        <v>59</v>
+      </c>
+      <c r="E21" s="100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F21" s="100" t="n">
+        <v>29.5</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C21" s="95" t="inlineStr">
+      <c r="C22" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D21" s="95" t="n">
+      <c r="D22" s="95" t="n">
         <v>13</v>
       </c>
-      <c r="E21" s="95" t="n">
+      <c r="E22" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F21" s="95" t="n">
-        <v>7.4</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="107" t="inlineStr">
+      <c r="F22" s="95" t="n">
+        <v>6.5</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D22" s="107" t="n">
-        <v>175</v>
-      </c>
-      <c r="E22" s="107" t="n">
-        <v>2.9</v>
-      </c>
-      <c r="F22" s="107" t="n">
+      <c r="D23" s="107" t="n">
+        <v>200</v>
+      </c>
+      <c r="E23" s="107" t="n">
+        <v>3.3</v>
+      </c>
+      <c r="F23" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-01: close 資料準備 11:20-12:15, start 昼休憩 12:15
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -13172,7 +13172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G24"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -13580,189 +13580,219 @@
       </c>
       <c r="F14" s="96" t="inlineStr">
         <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="G14" s="96" t="n">
+        <v>55</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C15" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D15" s="103" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E15" s="95" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F15" s="95" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G14" s="96" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="104" t="inlineStr">
+      <c r="G15" s="95" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C15" s="93" t="n"/>
-      <c r="D15" s="93" t="n"/>
-      <c r="E15" s="93" t="n"/>
-      <c r="F15" s="93" t="n"/>
-      <c r="G15" s="94" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="79" t="inlineStr">
+      <c r="C16" s="93" t="n"/>
+      <c r="D16" s="93" t="n"/>
+      <c r="E16" s="93" t="n"/>
+      <c r="F16" s="93" t="n"/>
+      <c r="G16" s="94" t="n"/>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C16" s="79" t="inlineStr">
+      <c r="C17" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D16" s="79" t="inlineStr">
+      <c r="D17" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E16" s="79" t="inlineStr">
+      <c r="E17" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F16" s="79" t="inlineStr">
+      <c r="F17" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="18" customHeight="1" s="64">
-      <c r="B17" s="105" t="inlineStr">
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C17" s="105" t="inlineStr">
+      <c r="C18" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D17" s="105" t="n">
+      <c r="D18" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="105" t="n">
+      <c r="E18" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="105" t="n">
+      <c r="F18" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" s="64">
-      <c r="B18" s="96" t="inlineStr">
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C18" s="96" t="inlineStr">
+      <c r="C19" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D18" s="96" t="n">
-        <v>83</v>
-      </c>
-      <c r="E18" s="96" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F18" s="96" t="n">
-        <v>41.5</v>
-      </c>
-    </row>
-    <row r="19" ht="18" customHeight="1" s="64">
-      <c r="B19" s="98" t="inlineStr">
+      <c r="D19" s="96" t="n">
+        <v>138</v>
+      </c>
+      <c r="E19" s="96" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F19" s="96" t="n">
+        <v>54.1</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C19" s="98" t="inlineStr">
+      <c r="C20" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D19" s="98" t="n">
+      <c r="D20" s="98" t="n">
         <v>45</v>
       </c>
-      <c r="E19" s="98" t="n">
+      <c r="E20" s="98" t="n">
         <v>0.8</v>
       </c>
-      <c r="F19" s="98" t="n">
-        <v>22.5</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" s="64">
-      <c r="B20" s="106" t="inlineStr">
+      <c r="F20" s="98" t="n">
+        <v>17.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C20" s="106" t="inlineStr">
+      <c r="C21" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D20" s="106" t="n">
+      <c r="D21" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="106" t="n">
+      <c r="E21" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="106" t="n">
+      <c r="F21" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="100" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C21" s="100" t="inlineStr">
+      <c r="C22" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D21" s="100" t="n">
+      <c r="D22" s="100" t="n">
         <v>59</v>
       </c>
-      <c r="E21" s="100" t="n">
+      <c r="E22" s="100" t="n">
         <v>1</v>
       </c>
-      <c r="F21" s="100" t="n">
-        <v>29.5</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="95" t="inlineStr">
+      <c r="F22" s="100" t="n">
+        <v>23.1</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C22" s="95" t="inlineStr">
+      <c r="C23" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D22" s="95" t="n">
+      <c r="D23" s="95" t="n">
         <v>13</v>
       </c>
-      <c r="E22" s="95" t="n">
+      <c r="E23" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F22" s="95" t="n">
-        <v>6.5</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="107" t="inlineStr">
+      <c r="F23" s="95" t="n">
+        <v>5.1</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D23" s="107" t="n">
-        <v>200</v>
-      </c>
-      <c r="E23" s="107" t="n">
-        <v>3.3</v>
-      </c>
-      <c r="F23" s="107" t="n">
+      <c r="D24" s="107" t="n">
+        <v>255</v>
+      </c>
+      <c r="E24" s="107" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F24" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-01: 昼休憩close, 掃除/資料準備/新人教育/休憩 12:45-15:00+
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -13172,7 +13172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G24"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -13610,189 +13610,309 @@
       </c>
       <c r="F15" s="95" t="inlineStr">
         <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="G15" s="95" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C16" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D16" s="103" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E16" s="95" t="inlineStr">
+        <is>
+          <t>12:45</t>
+        </is>
+      </c>
+      <c r="F16" s="95" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="G16" s="95" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C17" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
+        <is>
+          <t>新人社員教育 資料準備</t>
+        </is>
+      </c>
+      <c r="E17" s="96" t="inlineStr">
+        <is>
+          <t>12:55</t>
+        </is>
+      </c>
+      <c r="F17" s="96" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="G17" s="96" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C18" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D18" s="97" t="inlineStr">
+        <is>
+          <t>新人社員教育</t>
+        </is>
+      </c>
+      <c r="E18" s="96" t="inlineStr">
+        <is>
+          <t>13:00</t>
+        </is>
+      </c>
+      <c r="F18" s="96" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="G18" s="96" t="n">
+        <v>120</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C19" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D19" s="103" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E19" s="95" t="inlineStr">
+        <is>
+          <t>15:00</t>
+        </is>
+      </c>
+      <c r="F19" s="95" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G15" s="95" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="104" t="inlineStr">
+      <c r="G19" s="95" t="n"/>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C16" s="93" t="n"/>
-      <c r="D16" s="93" t="n"/>
-      <c r="E16" s="93" t="n"/>
-      <c r="F16" s="93" t="n"/>
-      <c r="G16" s="94" t="n"/>
-    </row>
-    <row r="17" ht="18" customHeight="1" s="64">
-      <c r="B17" s="79" t="inlineStr">
+      <c r="C20" s="93" t="n"/>
+      <c r="D20" s="93" t="n"/>
+      <c r="E20" s="93" t="n"/>
+      <c r="F20" s="93" t="n"/>
+      <c r="G20" s="94" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C17" s="79" t="inlineStr">
+      <c r="C21" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D17" s="79" t="inlineStr">
+      <c r="D21" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E17" s="79" t="inlineStr">
+      <c r="E21" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F17" s="79" t="inlineStr">
+      <c r="F21" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="18" customHeight="1" s="64">
-      <c r="B18" s="105" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C18" s="105" t="inlineStr">
+      <c r="C22" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D18" s="105" t="n">
+      <c r="D22" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="105" t="n">
+      <c r="E22" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="105" t="n">
+      <c r="F22" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" s="64">
-      <c r="B19" s="96" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C19" s="96" t="inlineStr">
+      <c r="C23" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D19" s="96" t="n">
-        <v>138</v>
-      </c>
-      <c r="E19" s="96" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="F19" s="96" t="n">
-        <v>54.1</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" s="64">
-      <c r="B20" s="98" t="inlineStr">
+      <c r="D23" s="96" t="n">
+        <v>263</v>
+      </c>
+      <c r="E23" s="96" t="n">
+        <v>4.4</v>
+      </c>
+      <c r="F23" s="96" t="n">
+        <v>62.6</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C20" s="98" t="inlineStr">
+      <c r="C24" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D20" s="98" t="n">
+      <c r="D24" s="98" t="n">
         <v>45</v>
       </c>
-      <c r="E20" s="98" t="n">
+      <c r="E24" s="98" t="n">
         <v>0.8</v>
       </c>
-      <c r="F20" s="98" t="n">
-        <v>17.6</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="106" t="inlineStr">
+      <c r="F24" s="98" t="n">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C21" s="106" t="inlineStr">
+      <c r="C25" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D21" s="106" t="n">
+      <c r="D25" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="106" t="n">
+      <c r="E25" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="106" t="n">
+      <c r="F25" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="100" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C22" s="100" t="inlineStr">
+      <c r="C26" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D22" s="100" t="n">
+      <c r="D26" s="100" t="n">
         <v>59</v>
       </c>
-      <c r="E22" s="100" t="n">
+      <c r="E26" s="100" t="n">
         <v>1</v>
       </c>
-      <c r="F22" s="100" t="n">
-        <v>23.1</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="95" t="inlineStr">
+      <c r="F26" s="100" t="n">
+        <v>14</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C23" s="95" t="inlineStr">
+      <c r="C27" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D23" s="95" t="n">
-        <v>13</v>
-      </c>
-      <c r="E23" s="95" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F23" s="95" t="n">
-        <v>5.1</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="107" t="inlineStr">
+      <c r="D27" s="95" t="n">
+        <v>53</v>
+      </c>
+      <c r="E27" s="95" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F27" s="95" t="n">
+        <v>12.6</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D24" s="107" t="n">
-        <v>255</v>
-      </c>
-      <c r="E24" s="107" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="F24" s="107" t="n">
+      <c r="D28" s="107" t="n">
+        <v>420</v>
+      </c>
+      <c r="E28" s="107" t="n">
+        <v>7</v>
+      </c>
+      <c r="F28" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-01: 治具確認 17:35-18:17, 調査結果メール連絡 18:17-
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -13172,7 +13172,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G31"/>
+  <dimension ref="A1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -13820,189 +13820,249 @@
       </c>
       <c r="F22" s="100" t="inlineStr">
         <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="G22" s="100" t="n">
+        <v>45</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C23" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D23" s="99" t="inlineStr">
+        <is>
+          <t>治具確認</t>
+        </is>
+      </c>
+      <c r="E23" s="98" t="inlineStr">
+        <is>
+          <t>17:35</t>
+        </is>
+      </c>
+      <c r="F23" s="98" t="inlineStr">
+        <is>
+          <t>18:17</t>
+        </is>
+      </c>
+      <c r="G23" s="98" t="n">
+        <v>42</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C24" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D24" s="101" t="inlineStr">
+        <is>
+          <t>調査結果メール連絡</t>
+        </is>
+      </c>
+      <c r="E24" s="100" t="inlineStr">
+        <is>
+          <t>18:17</t>
+        </is>
+      </c>
+      <c r="F24" s="100" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G22" s="100" t="n"/>
-    </row>
-    <row r="23">
-      <c r="B23" s="104" t="inlineStr">
+      <c r="G24" s="100" t="n"/>
+    </row>
+    <row r="25">
+      <c r="B25" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C23" s="93" t="n"/>
-      <c r="D23" s="93" t="n"/>
-      <c r="E23" s="93" t="n"/>
-      <c r="F23" s="93" t="n"/>
-      <c r="G23" s="94" t="n"/>
-    </row>
-    <row r="24">
-      <c r="B24" s="79" t="inlineStr">
+      <c r="C25" s="93" t="n"/>
+      <c r="D25" s="93" t="n"/>
+      <c r="E25" s="93" t="n"/>
+      <c r="F25" s="93" t="n"/>
+      <c r="G25" s="94" t="n"/>
+    </row>
+    <row r="26">
+      <c r="B26" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C24" s="79" t="inlineStr">
+      <c r="C26" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D24" s="79" t="inlineStr">
+      <c r="D26" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E24" s="79" t="inlineStr">
+      <c r="E26" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F24" s="79" t="inlineStr">
+      <c r="F26" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="105" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C25" s="105" t="inlineStr">
+      <c r="C27" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D25" s="105" t="n">
+      <c r="D27" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E25" s="105" t="n">
+      <c r="E27" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F25" s="105" t="n">
+      <c r="F27" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="96" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C26" s="96" t="inlineStr">
+      <c r="C28" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D26" s="96" t="n">
+      <c r="D28" s="96" t="n">
         <v>263</v>
       </c>
-      <c r="E26" s="96" t="n">
+      <c r="E28" s="96" t="n">
         <v>4.4</v>
       </c>
-      <c r="F26" s="96" t="n">
-        <v>49.6</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="98" t="inlineStr">
+      <c r="F28" s="96" t="n">
+        <v>42.6</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C27" s="98" t="inlineStr">
+      <c r="C29" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D27" s="98" t="n">
-        <v>145</v>
-      </c>
-      <c r="E27" s="98" t="n">
-        <v>2.4</v>
-      </c>
-      <c r="F27" s="98" t="n">
-        <v>27.4</v>
-      </c>
-    </row>
-    <row r="28">
-      <c r="B28" s="106" t="inlineStr">
+      <c r="D29" s="98" t="n">
+        <v>187</v>
+      </c>
+      <c r="E29" s="98" t="n">
+        <v>3.1</v>
+      </c>
+      <c r="F29" s="98" t="n">
+        <v>30.3</v>
+      </c>
+    </row>
+    <row r="30">
+      <c r="B30" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C28" s="106" t="inlineStr">
+      <c r="C30" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D28" s="106" t="n">
+      <c r="D30" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E28" s="106" t="n">
+      <c r="E30" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F28" s="106" t="n">
+      <c r="F30" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="100" t="inlineStr">
+    <row r="31">
+      <c r="B31" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C29" s="100" t="inlineStr">
+      <c r="C31" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D29" s="100" t="n">
-        <v>59</v>
-      </c>
-      <c r="E29" s="100" t="n">
-        <v>1</v>
-      </c>
-      <c r="F29" s="100" t="n">
-        <v>11.1</v>
-      </c>
-    </row>
-    <row r="30">
-      <c r="B30" s="95" t="inlineStr">
+      <c r="D31" s="100" t="n">
+        <v>104</v>
+      </c>
+      <c r="E31" s="100" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F31" s="100" t="n">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="32">
+      <c r="B32" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C30" s="95" t="inlineStr">
+      <c r="C32" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D30" s="95" t="n">
+      <c r="D32" s="95" t="n">
         <v>63</v>
       </c>
-      <c r="E30" s="95" t="n">
+      <c r="E32" s="95" t="n">
         <v>1.1</v>
       </c>
-      <c r="F30" s="95" t="n">
-        <v>11.9</v>
-      </c>
-    </row>
-    <row r="31">
-      <c r="B31" s="107" t="inlineStr">
+      <c r="F32" s="95" t="n">
+        <v>10.2</v>
+      </c>
+    </row>
+    <row r="33">
+      <c r="B33" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D31" s="107" t="n">
-        <v>530</v>
-      </c>
-      <c r="E31" s="107" t="n">
-        <v>8.800000000000001</v>
-      </c>
-      <c r="F31" s="107" t="n">
+      <c r="D33" s="107" t="n">
+        <v>617</v>
+      </c>
+      <c r="E33" s="107" t="n">
+        <v>10.3</v>
+      </c>
+      <c r="F33" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-01: close 調査結果メール連絡 18:17-18:26, 業務終了
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -13880,10 +13880,12 @@
       </c>
       <c r="F24" s="100" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G24" s="100" t="n"/>
+          <t>18:26</t>
+        </is>
+      </c>
+      <c r="G24" s="100" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="25">
       <c r="B25" s="104" t="inlineStr">
@@ -13963,7 +13965,7 @@
         <v>4.4</v>
       </c>
       <c r="F28" s="96" t="n">
-        <v>42.6</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29">
@@ -13984,7 +13986,7 @@
         <v>3.1</v>
       </c>
       <c r="F29" s="98" t="n">
-        <v>30.3</v>
+        <v>29.9</v>
       </c>
     </row>
     <row r="30">
@@ -14020,13 +14022,13 @@
         </is>
       </c>
       <c r="D31" s="100" t="n">
-        <v>104</v>
+        <v>113</v>
       </c>
       <c r="E31" s="100" t="n">
-        <v>1.7</v>
+        <v>1.9</v>
       </c>
       <c r="F31" s="100" t="n">
-        <v>16.9</v>
+        <v>18.1</v>
       </c>
     </row>
     <row r="32">
@@ -14047,7 +14049,7 @@
         <v>1.1</v>
       </c>
       <c r="F32" s="95" t="n">
-        <v>10.2</v>
+        <v>10.1</v>
       </c>
     </row>
     <row r="33">
@@ -14057,10 +14059,10 @@
         </is>
       </c>
       <c r="D33" s="107" t="n">
-        <v>617</v>
+        <v>626</v>
       </c>
       <c r="E33" s="107" t="n">
-        <v>10.3</v>
+        <v>10.4</v>
       </c>
       <c r="F33" s="107" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add 2026-06-02: new sheet, start ラジオ体操 7:59
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -22,14 +22,15 @@
     <sheet name="2026-05-28" sheetId="14" state="visible" r:id="rId14"/>
     <sheet name="2026-05-29" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-06-01" sheetId="16" state="visible" r:id="rId16"/>
+    <sheet name="2026-06-02" sheetId="17" state="visible" r:id="rId17"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId17"/>
     <externalReference r:id="rId18"/>
     <externalReference r:id="rId19"/>
     <externalReference r:id="rId20"/>
     <externalReference r:id="rId21"/>
     <externalReference r:id="rId22"/>
+    <externalReference r:id="rId23"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -13172,7 +13173,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G33"/>
+  <dimension ref="B1:G33"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14070,6 +14071,275 @@
     </row>
   </sheetData>
   <mergeCells count="1">
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet17.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G12"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="64" min="2" max="2"/>
+    <col width="18" customWidth="1" style="64" min="3" max="3"/>
+    <col width="42" customWidth="1" style="64" min="4" max="4"/>
+    <col width="8" customWidth="1" style="64" min="5" max="5"/>
+    <col width="8" customWidth="1" style="64" min="6" max="6"/>
+    <col width="12" customWidth="1" style="64" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" s="64">
+      <c r="B1" s="102" t="inlineStr">
+        <is>
+          <t>2026年6月2日（火）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="64">
+      <c r="B2" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C2" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D2" s="79" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E2" s="79" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F2" s="79" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G2" s="79" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="64">
+      <c r="B3" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C3" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D3" s="103" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E3" s="95" t="inlineStr">
+        <is>
+          <t>7:59</t>
+        </is>
+      </c>
+      <c r="F3" s="95" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G3" s="95" t="n"/>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="64">
+      <c r="B4" s="104" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C5" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D5" s="79" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E5" s="79" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F5" s="79" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="64">
+      <c r="B6" s="105" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C6" s="105" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D6" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C7" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D7" s="96" t="n">
+        <v>0</v>
+      </c>
+      <c r="E7" s="96" t="n">
+        <v>0</v>
+      </c>
+      <c r="F7" s="96" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C8" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D8" s="98" t="n">
+        <v>0</v>
+      </c>
+      <c r="E8" s="98" t="n">
+        <v>0</v>
+      </c>
+      <c r="F8" s="98" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C9" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D9" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E9" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F9" s="106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C10" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D10" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="E11" s="95" t="n">
+        <v>0</v>
+      </c>
+      <c r="F11" s="95" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="107" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="D12" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="107" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="107" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B4:G4"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-06-02: ラジオ体操close, 各職場朝礼, start 現場周り 8:06
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14083,7 +14083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G12"/>
+  <dimension ref="A1:G14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14100,6 +14100,11 @@
           <t>2026年6月2日（火）　業務記録</t>
         </is>
       </c>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="94" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1" s="64">
       <c r="B2" s="79" t="inlineStr">
@@ -14156,184 +14161,249 @@
       </c>
       <c r="F3" s="95" t="inlineStr">
         <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G3" s="95" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="64">
+      <c r="B4" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C4" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E4" s="96" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F4" s="96" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G4" s="96" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5">
+      <c r="B5" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C5" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E5" s="98" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F5" s="98" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G3" s="95" t="n"/>
-    </row>
-    <row r="4" ht="18" customHeight="1" s="64">
-      <c r="B4" s="104" t="inlineStr">
+      <c r="G5" s="98" t="n"/>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="64">
+      <c r="B6" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="B5" s="79" t="inlineStr">
+      <c r="C6" s="93" t="n"/>
+      <c r="D6" s="93" t="n"/>
+      <c r="E6" s="93" t="n"/>
+      <c r="F6" s="93" t="n"/>
+      <c r="G6" s="94" t="n"/>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C5" s="79" t="inlineStr">
+      <c r="C7" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D5" s="79" t="inlineStr">
+      <c r="D7" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E5" s="79" t="inlineStr">
+      <c r="E7" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F5" s="79" t="inlineStr">
+      <c r="F7" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="6" ht="18" customHeight="1" s="64">
-      <c r="B6" s="105" t="inlineStr">
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C6" s="105" t="inlineStr">
+      <c r="C8" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D6" s="105" t="n">
+      <c r="D8" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E6" s="105" t="n">
+      <c r="E8" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F6" s="105" t="n">
+      <c r="F8" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="7" ht="18" customHeight="1" s="64">
-      <c r="B7" s="96" t="inlineStr">
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C7" s="96" t="inlineStr">
+      <c r="C9" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D7" s="96" t="n">
+      <c r="D9" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="E7" s="96" t="n">
+      <c r="E9" s="96" t="n">
         <v>0</v>
       </c>
-      <c r="F7" s="96" t="n">
+      <c r="F9" s="96" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" s="64">
-      <c r="B8" s="98" t="inlineStr">
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C8" s="98" t="inlineStr">
+      <c r="C10" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D8" s="98" t="n">
+      <c r="D10" s="98" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="98" t="n">
+      <c r="E10" s="98" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="98" t="n">
+      <c r="F10" s="98" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="64">
-      <c r="B9" s="106" t="inlineStr">
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C9" s="106" t="inlineStr">
+      <c r="C11" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D9" s="106" t="n">
+      <c r="D11" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="106" t="n">
+      <c r="E11" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="106" t="n">
+      <c r="F11" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="64">
-      <c r="B10" s="100" t="inlineStr">
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C10" s="100" t="inlineStr">
+      <c r="C12" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D10" s="100" t="n">
+      <c r="D12" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="100" t="n">
+      <c r="E12" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="100" t="n">
+      <c r="F12" s="100" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="64">
-      <c r="B11" s="95" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C11" s="95" t="inlineStr">
+      <c r="C13" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D11" s="95" t="n">
+      <c r="D13" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="E11" s="95" t="n">
+      <c r="E13" s="95" t="n">
         <v>0</v>
       </c>
-      <c r="F11" s="95" t="n">
+      <c r="F13" s="95" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="107" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D12" s="107" t="n">
+      <c r="D14" s="107" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="107" t="n">
+      <c r="E14" s="107" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="107" t="n">
+      <c r="F14" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-02: close 現場周り 8:15, add 社長と面談 8:15-8:25
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14083,7 +14083,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G14"/>
+  <dimension ref="A1:G15"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14174,29 +14174,11 @@
           <t>②</t>
         </is>
       </c>
-      <c r="C4" s="96" t="inlineStr">
-        <is>
-          <t>社内マネジメント</t>
-        </is>
-      </c>
-      <c r="D4" s="97" t="inlineStr">
-        <is>
-          <t>各職場朝礼参加</t>
-        </is>
-      </c>
-      <c r="E4" s="96" t="inlineStr">
-        <is>
-          <t>8:03</t>
-        </is>
-      </c>
-      <c r="F4" s="96" t="inlineStr">
-        <is>
-          <t>8:06</t>
-        </is>
-      </c>
-      <c r="G4" s="96" t="n">
-        <v>3</v>
-      </c>
+      <c r="C4" s="93" t="n"/>
+      <c r="D4" s="93" t="n"/>
+      <c r="E4" s="93" t="n"/>
+      <c r="F4" s="93" t="n"/>
+      <c r="G4" s="94" t="n"/>
     </row>
     <row r="5">
       <c r="B5" s="98" t="inlineStr">
@@ -14221,189 +14203,221 @@
       </c>
       <c r="F5" s="98" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G5" s="98" t="n"/>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="G5" s="98" t="n">
+        <v>9</v>
+      </c>
     </row>
     <row r="6" ht="18" customHeight="1" s="64">
-      <c r="B6" s="104" t="inlineStr">
+      <c r="B6" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C6" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D6" s="97" t="inlineStr">
+        <is>
+          <t>社長と面談</t>
+        </is>
+      </c>
+      <c r="E6" s="96" t="inlineStr">
+        <is>
+          <t>8:15</t>
+        </is>
+      </c>
+      <c r="F6" s="96" t="inlineStr">
+        <is>
+          <t>8:25</t>
+        </is>
+      </c>
+      <c r="G6" s="96" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C6" s="93" t="n"/>
-      <c r="D6" s="93" t="n"/>
-      <c r="E6" s="93" t="n"/>
-      <c r="F6" s="93" t="n"/>
-      <c r="G6" s="94" t="n"/>
-    </row>
-    <row r="7" ht="18" customHeight="1" s="64">
-      <c r="B7" s="79" t="inlineStr">
+      <c r="C7" s="93" t="n"/>
+      <c r="D7" s="93" t="n"/>
+      <c r="E7" s="93" t="n"/>
+      <c r="F7" s="93" t="n"/>
+      <c r="G7" s="94" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C7" s="79" t="inlineStr">
+      <c r="C8" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D7" s="79" t="inlineStr">
+      <c r="D8" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E7" s="79" t="inlineStr">
+      <c r="E8" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F7" s="79" t="inlineStr">
+      <c r="F8" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="8" ht="18" customHeight="1" s="64">
-      <c r="B8" s="105" t="inlineStr">
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C8" s="105" t="inlineStr">
+      <c r="C9" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D8" s="105" t="n">
+      <c r="D9" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E8" s="105" t="n">
+      <c r="E9" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F8" s="105" t="n">
+      <c r="F9" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="64">
-      <c r="B9" s="96" t="inlineStr">
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C9" s="96" t="inlineStr">
+      <c r="C10" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D9" s="96" t="n">
+      <c r="D10" s="96" t="n">
+        <v>13</v>
+      </c>
+      <c r="E10" s="96" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F10" s="96" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C11" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D11" s="98" t="n">
+        <v>9</v>
+      </c>
+      <c r="E11" s="98" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F11" s="98" t="n">
+        <v>34.6</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C12" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D12" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="96" t="n">
+      <c r="E12" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="96" t="n">
+      <c r="F12" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="64">
-      <c r="B10" s="98" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C10" s="98" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D10" s="98" t="n">
+    <row r="13">
+      <c r="B13" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C13" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D13" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="98" t="n">
+      <c r="E13" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="98" t="n">
+      <c r="F13" s="100" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="64">
-      <c r="B11" s="106" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C11" s="106" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D11" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="106" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="100" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C12" s="100" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D12" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="100" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="95" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C13" s="95" t="inlineStr">
+      <c r="C14" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D13" s="95" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="95" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="95" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="107" t="inlineStr">
+      <c r="D14" s="95" t="n">
+        <v>4</v>
+      </c>
+      <c r="E14" s="95" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F14" s="95" t="n">
+        <v>15.4</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D14" s="107" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="107" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="107" t="n">
+      <c r="D15" s="107" t="n">
+        <v>26</v>
+      </c>
+      <c r="E15" s="107" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F15" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-02: 打ち合わせ 8:30-8:36, 現場周り 8:36-8:45, start 現場軽作業 8:45
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -668,7 +668,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="108">
+  <cellXfs count="109">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -934,6 +934,9 @@
     </xf>
     <xf numFmtId="0" fontId="29" fillId="21" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="27" fillId="20" borderId="12" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+      <alignment horizontal="left" vertical="center" wrapText="1"/>
     </xf>
   </cellXfs>
   <cellStyles count="1">
@@ -14083,7 +14086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G15"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14241,183 +14244,271 @@
       </c>
     </row>
     <row r="7" ht="18" customHeight="1" s="64">
-      <c r="B7" s="104" t="inlineStr">
+      <c r="B7" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C7" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D7" s="97" t="inlineStr">
+        <is>
+          <t>現場社員と打ち合わせ</t>
+        </is>
+      </c>
+      <c r="E7" s="96" t="inlineStr">
+        <is>
+          <t>8:30</t>
+        </is>
+      </c>
+      <c r="F7" s="96" t="inlineStr">
+        <is>
+          <t>8:36</t>
+        </is>
+      </c>
+      <c r="G7" s="96" t="n">
+        <v>6</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C8" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D8" s="99" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E8" s="98" t="inlineStr">
+        <is>
+          <t>8:36</t>
+        </is>
+      </c>
+      <c r="F8" s="98" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="G8" s="98" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C9" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D9" s="108" t="inlineStr">
+        <is>
+          <t>現場軽作業</t>
+        </is>
+      </c>
+      <c r="E9" s="106" t="inlineStr">
+        <is>
+          <t>8:45</t>
+        </is>
+      </c>
+      <c r="F9" s="106" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G9" s="106" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C7" s="93" t="n"/>
-      <c r="D7" s="93" t="n"/>
-      <c r="E7" s="93" t="n"/>
-      <c r="F7" s="93" t="n"/>
-      <c r="G7" s="94" t="n"/>
-    </row>
-    <row r="8" ht="18" customHeight="1" s="64">
-      <c r="B8" s="79" t="inlineStr">
+      <c r="C10" s="93" t="n"/>
+      <c r="D10" s="93" t="n"/>
+      <c r="E10" s="93" t="n"/>
+      <c r="F10" s="93" t="n"/>
+      <c r="G10" s="94" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C8" s="79" t="inlineStr">
+      <c r="C11" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D8" s="79" t="inlineStr">
+      <c r="D11" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E8" s="79" t="inlineStr">
+      <c r="E11" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F8" s="79" t="inlineStr">
+      <c r="F11" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="18" customHeight="1" s="64">
-      <c r="B9" s="105" t="inlineStr">
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C9" s="105" t="inlineStr">
+      <c r="C12" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D9" s="105" t="n">
+      <c r="D12" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E9" s="105" t="n">
+      <c r="E12" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F9" s="105" t="n">
+      <c r="F12" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="64">
-      <c r="B10" s="96" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C10" s="96" t="inlineStr">
+      <c r="C13" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D10" s="96" t="n">
-        <v>13</v>
-      </c>
-      <c r="E10" s="96" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F10" s="96" t="n">
-        <v>50</v>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1" s="64">
-      <c r="B11" s="98" t="inlineStr">
+      <c r="D13" s="96" t="n">
+        <v>19</v>
+      </c>
+      <c r="E13" s="96" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F13" s="96" t="n">
+        <v>46.3</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C11" s="98" t="inlineStr">
+      <c r="C14" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D11" s="98" t="n">
-        <v>9</v>
-      </c>
-      <c r="E11" s="98" t="n">
+      <c r="D14" s="98" t="n">
+        <v>18</v>
+      </c>
+      <c r="E14" s="98" t="n">
+        <v>0.3</v>
+      </c>
+      <c r="F14" s="98" t="n">
+        <v>43.9</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C15" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D15" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C16" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D16" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F16" s="100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C17" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D17" s="95" t="n">
+        <v>4</v>
+      </c>
+      <c r="E17" s="95" t="n">
         <v>0.1</v>
       </c>
-      <c r="F11" s="98" t="n">
-        <v>34.6</v>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="106" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C12" s="106" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D12" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="E12" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="F12" s="106" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="13">
-      <c r="B13" s="100" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C13" s="100" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D13" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="E13" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="F13" s="100" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="95" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="C14" s="95" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D14" s="95" t="n">
-        <v>4</v>
-      </c>
-      <c r="E14" s="95" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F14" s="95" t="n">
-        <v>15.4</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="107" t="inlineStr">
+      <c r="F17" s="95" t="n">
+        <v>9.800000000000001</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D15" s="107" t="n">
-        <v>26</v>
-      </c>
-      <c r="E15" s="107" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F15" s="107" t="n">
+      <c r="D18" s="107" t="n">
+        <v>41</v>
+      </c>
+      <c r="E18" s="107" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F18" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-02: close 現場軽作業 8:45-9:20, start 検査表チェック 9:20
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14086,7 +14086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14326,189 +14326,219 @@
       </c>
       <c r="F9" s="106" t="inlineStr">
         <is>
+          <t>9:20</t>
+        </is>
+      </c>
+      <c r="G9" s="106" t="n">
+        <v>35</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C10" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D10" s="99" t="inlineStr">
+        <is>
+          <t>検査表チェック</t>
+        </is>
+      </c>
+      <c r="E10" s="98" t="inlineStr">
+        <is>
+          <t>9:20</t>
+        </is>
+      </c>
+      <c r="F10" s="98" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G9" s="106" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" s="64">
-      <c r="B10" s="104" t="inlineStr">
+      <c r="G10" s="98" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C10" s="93" t="n"/>
-      <c r="D10" s="93" t="n"/>
-      <c r="E10" s="93" t="n"/>
-      <c r="F10" s="93" t="n"/>
-      <c r="G10" s="94" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1" s="64">
-      <c r="B11" s="79" t="inlineStr">
+      <c r="C11" s="93" t="n"/>
+      <c r="D11" s="93" t="n"/>
+      <c r="E11" s="93" t="n"/>
+      <c r="F11" s="93" t="n"/>
+      <c r="G11" s="94" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C11" s="79" t="inlineStr">
+      <c r="C12" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D11" s="79" t="inlineStr">
+      <c r="D12" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E11" s="79" t="inlineStr">
+      <c r="E12" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F11" s="79" t="inlineStr">
+      <c r="F12" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="105" t="inlineStr">
+    <row r="13">
+      <c r="B13" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C12" s="105" t="inlineStr">
+      <c r="C13" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D12" s="105" t="n">
+      <c r="D13" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="105" t="n">
+      <c r="E13" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="105" t="n">
+      <c r="F13" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="96" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C13" s="96" t="inlineStr">
+      <c r="C14" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D13" s="96" t="n">
+      <c r="D14" s="96" t="n">
         <v>19</v>
       </c>
-      <c r="E13" s="96" t="n">
+      <c r="E14" s="96" t="n">
         <v>0.3</v>
       </c>
-      <c r="F13" s="96" t="n">
-        <v>46.3</v>
-      </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="98" t="inlineStr">
+      <c r="F14" s="96" t="n">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="15">
+      <c r="B15" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C14" s="98" t="inlineStr">
+      <c r="C15" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D14" s="98" t="n">
+      <c r="D15" s="98" t="n">
         <v>18</v>
       </c>
-      <c r="E14" s="98" t="n">
+      <c r="E15" s="98" t="n">
         <v>0.3</v>
       </c>
-      <c r="F14" s="98" t="n">
-        <v>43.9</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="106" t="inlineStr">
+      <c r="F15" s="98" t="n">
+        <v>23.7</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C15" s="106" t="inlineStr">
+      <c r="C16" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D15" s="106" t="n">
+      <c r="D16" s="106" t="n">
+        <v>35</v>
+      </c>
+      <c r="E16" s="106" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F16" s="106" t="n">
+        <v>46.1</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C17" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D17" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="106" t="n">
+      <c r="E17" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="106" t="n">
+      <c r="F17" s="100" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="16">
-      <c r="B16" s="100" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C16" s="100" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D16" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="F16" s="100" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="95" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C17" s="95" t="inlineStr">
+      <c r="C18" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D17" s="95" t="n">
+      <c r="D18" s="95" t="n">
         <v>4</v>
       </c>
-      <c r="E17" s="95" t="n">
+      <c r="E18" s="95" t="n">
         <v>0.1</v>
       </c>
-      <c r="F17" s="95" t="n">
-        <v>9.800000000000001</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="107" t="inlineStr">
+      <c r="F18" s="95" t="n">
+        <v>5.3</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D18" s="107" t="n">
-        <v>41</v>
-      </c>
-      <c r="E18" s="107" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F18" s="107" t="n">
+      <c r="D19" s="107" t="n">
+        <v>76</v>
+      </c>
+      <c r="E19" s="107" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F19" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-02: 検査表チェック 9:20-10:00, 休憩 10:00-10:10
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14086,7 +14086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G19"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14356,189 +14356,221 @@
       </c>
       <c r="F10" s="98" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G10" s="98" t="n"/>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="G10" s="98" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="11" ht="18" customHeight="1" s="64">
-      <c r="B11" s="104" t="inlineStr">
+      <c r="B11" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C11" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D11" s="103" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E11" s="95" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F11" s="95" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G11" s="95" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C11" s="93" t="n"/>
-      <c r="D11" s="93" t="n"/>
-      <c r="E11" s="93" t="n"/>
-      <c r="F11" s="93" t="n"/>
-      <c r="G11" s="94" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="79" t="inlineStr">
+      <c r="C12" s="93" t="n"/>
+      <c r="D12" s="93" t="n"/>
+      <c r="E12" s="93" t="n"/>
+      <c r="F12" s="93" t="n"/>
+      <c r="G12" s="94" t="n"/>
+    </row>
+    <row r="13">
+      <c r="B13" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C12" s="79" t="inlineStr">
+      <c r="C13" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D12" s="79" t="inlineStr">
+      <c r="D13" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E12" s="79" t="inlineStr">
+      <c r="E13" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F12" s="79" t="inlineStr">
+      <c r="F13" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="B13" s="105" t="inlineStr">
+    <row r="14">
+      <c r="B14" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C13" s="105" t="inlineStr">
+      <c r="C14" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D13" s="105" t="n">
+      <c r="D14" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="105" t="n">
+      <c r="E14" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="105" t="n">
+      <c r="F14" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="96" t="inlineStr">
+    <row r="15">
+      <c r="B15" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C14" s="96" t="inlineStr">
+      <c r="C15" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D14" s="96" t="n">
+      <c r="D15" s="96" t="n">
         <v>19</v>
       </c>
-      <c r="E14" s="96" t="n">
+      <c r="E15" s="96" t="n">
         <v>0.3</v>
       </c>
-      <c r="F14" s="96" t="n">
-        <v>25</v>
-      </c>
-    </row>
-    <row r="15">
-      <c r="B15" s="98" t="inlineStr">
+      <c r="F15" s="96" t="n">
+        <v>15.1</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="B16" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C15" s="98" t="inlineStr">
+      <c r="C16" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D15" s="98" t="n">
-        <v>18</v>
-      </c>
-      <c r="E15" s="98" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F15" s="98" t="n">
-        <v>23.7</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="106" t="inlineStr">
+      <c r="D16" s="98" t="n">
+        <v>58</v>
+      </c>
+      <c r="E16" s="98" t="n">
+        <v>1</v>
+      </c>
+      <c r="F16" s="98" t="n">
+        <v>46</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C16" s="106" t="inlineStr">
+      <c r="C17" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D16" s="106" t="n">
+      <c r="D17" s="106" t="n">
         <v>35</v>
       </c>
-      <c r="E16" s="106" t="n">
+      <c r="E17" s="106" t="n">
         <v>0.6</v>
       </c>
-      <c r="F16" s="106" t="n">
-        <v>46.1</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="100" t="inlineStr">
+      <c r="F17" s="106" t="n">
+        <v>27.8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C17" s="100" t="inlineStr">
+      <c r="C18" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D17" s="100" t="n">
+      <c r="D18" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="100" t="n">
+      <c r="E18" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="100" t="n">
+      <c r="F18" s="100" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="95" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C18" s="95" t="inlineStr">
+      <c r="C19" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D18" s="95" t="n">
-        <v>4</v>
-      </c>
-      <c r="E18" s="95" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F18" s="95" t="n">
-        <v>5.3</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="107" t="inlineStr">
+      <c r="D19" s="95" t="n">
+        <v>14</v>
+      </c>
+      <c r="E19" s="95" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F19" s="95" t="n">
+        <v>11.1</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D19" s="107" t="n">
-        <v>76</v>
-      </c>
-      <c r="E19" s="107" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="F19" s="107" t="n">
+      <c r="D20" s="107" t="n">
+        <v>126</v>
+      </c>
+      <c r="E20" s="107" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F20" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-02: 標準作業書作成会議 10:10-12:08, start 昼休憩 12:08
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14086,7 +14086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14394,183 +14394,241 @@
       </c>
     </row>
     <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="104" t="inlineStr">
+      <c r="B12" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C12" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
+        <is>
+          <t>標準作業書作成 会議</t>
+        </is>
+      </c>
+      <c r="E12" s="96" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F12" s="96" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="G12" s="96" t="n">
+        <v>118</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="B13" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="103" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E13" s="95" t="inlineStr">
+        <is>
+          <t>12:08</t>
+        </is>
+      </c>
+      <c r="F13" s="95" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G13" s="95" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C12" s="93" t="n"/>
-      <c r="D12" s="93" t="n"/>
-      <c r="E12" s="93" t="n"/>
-      <c r="F12" s="93" t="n"/>
-      <c r="G12" s="94" t="n"/>
-    </row>
-    <row r="13">
-      <c r="B13" s="79" t="inlineStr">
+      <c r="C14" s="93" t="n"/>
+      <c r="D14" s="93" t="n"/>
+      <c r="E14" s="93" t="n"/>
+      <c r="F14" s="93" t="n"/>
+      <c r="G14" s="94" t="n"/>
+    </row>
+    <row r="15">
+      <c r="B15" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C13" s="79" t="inlineStr">
+      <c r="C15" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D13" s="79" t="inlineStr">
+      <c r="D15" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E13" s="79" t="inlineStr">
+      <c r="E15" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F13" s="79" t="inlineStr">
+      <c r="F15" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="B14" s="105" t="inlineStr">
+    <row r="16">
+      <c r="B16" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C14" s="105" t="inlineStr">
+      <c r="C16" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D14" s="105" t="n">
+      <c r="D16" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="105" t="n">
+      <c r="E16" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="105" t="n">
+      <c r="F16" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15">
-      <c r="B15" s="96" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C15" s="96" t="inlineStr">
+      <c r="C17" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D15" s="96" t="n">
-        <v>19</v>
-      </c>
-      <c r="E15" s="96" t="n">
-        <v>0.3</v>
-      </c>
-      <c r="F15" s="96" t="n">
-        <v>15.1</v>
-      </c>
-    </row>
-    <row r="16">
-      <c r="B16" s="98" t="inlineStr">
+      <c r="D17" s="96" t="n">
+        <v>137</v>
+      </c>
+      <c r="E17" s="96" t="n">
+        <v>2.3</v>
+      </c>
+      <c r="F17" s="96" t="n">
+        <v>56.1</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C16" s="98" t="inlineStr">
+      <c r="C18" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D16" s="98" t="n">
+      <c r="D18" s="98" t="n">
         <v>58</v>
       </c>
-      <c r="E16" s="98" t="n">
+      <c r="E18" s="98" t="n">
         <v>1</v>
       </c>
-      <c r="F16" s="98" t="n">
-        <v>46</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="106" t="inlineStr">
+      <c r="F18" s="98" t="n">
+        <v>23.8</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C17" s="106" t="inlineStr">
+      <c r="C19" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D17" s="106" t="n">
+      <c r="D19" s="106" t="n">
         <v>35</v>
       </c>
-      <c r="E17" s="106" t="n">
+      <c r="E19" s="106" t="n">
         <v>0.6</v>
       </c>
-      <c r="F17" s="106" t="n">
-        <v>27.8</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="100" t="inlineStr">
+      <c r="F19" s="106" t="n">
+        <v>14.3</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C18" s="100" t="inlineStr">
+      <c r="C20" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D18" s="100" t="n">
+      <c r="D20" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="100" t="n">
+      <c r="E20" s="100" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="100" t="n">
+      <c r="F20" s="100" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="95" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C19" s="95" t="inlineStr">
+      <c r="C21" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D19" s="95" t="n">
+      <c r="D21" s="95" t="n">
         <v>14</v>
       </c>
-      <c r="E19" s="95" t="n">
+      <c r="E21" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F19" s="95" t="n">
-        <v>11.1</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="107" t="inlineStr">
+      <c r="F21" s="95" t="n">
+        <v>5.7</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D20" s="107" t="n">
-        <v>126</v>
-      </c>
-      <c r="E20" s="107" t="n">
-        <v>2.1</v>
-      </c>
-      <c r="F20" s="107" t="n">
+      <c r="D22" s="107" t="n">
+        <v>244</v>
+      </c>
+      <c r="E22" s="107" t="n">
+        <v>4.1</v>
+      </c>
+      <c r="F22" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-02: fix duplicates, 話し合い 14:25-14:33, resume メール事務処理 14:33
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14086,7 +14086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G27"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14177,11 +14177,29 @@
           <t>②</t>
         </is>
       </c>
-      <c r="C4" s="93" t="n"/>
-      <c r="D4" s="93" t="n"/>
-      <c r="E4" s="93" t="n"/>
-      <c r="F4" s="93" t="n"/>
-      <c r="G4" s="94" t="n"/>
+      <c r="C4" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E4" s="96" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F4" s="96" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G4" s="96" t="n">
+        <v>3</v>
+      </c>
     </row>
     <row r="5">
       <c r="B5" s="98" t="inlineStr">
@@ -14536,195 +14554,254 @@
       </c>
       <c r="F16" s="100" t="inlineStr">
         <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="G16" s="100" t="n">
+        <v>76</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C17" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
+        <is>
+          <t>現場社員と話し合い</t>
+        </is>
+      </c>
+      <c r="E17" s="96" t="inlineStr">
+        <is>
+          <t>14:25</t>
+        </is>
+      </c>
+      <c r="F17" s="96" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="G17" s="96" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C18" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D18" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック・事務処理</t>
+        </is>
+      </c>
+      <c r="E18" s="100" t="inlineStr">
+        <is>
+          <t>14:33</t>
+        </is>
+      </c>
+      <c r="F18" s="100" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G16" s="100" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="104" t="inlineStr">
+      <c r="G18" s="100" t="n"/>
+    </row>
+    <row r="19">
+      <c r="B19" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C17" s="93" t="n"/>
-      <c r="D17" s="93" t="n"/>
-      <c r="E17" s="93" t="n"/>
-      <c r="F17" s="93" t="n"/>
-      <c r="G17" s="94" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="79" t="inlineStr">
+      <c r="C19" s="93" t="n"/>
+      <c r="D19" s="93" t="n"/>
+      <c r="E19" s="93" t="n"/>
+      <c r="F19" s="93" t="n"/>
+      <c r="G19" s="94" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C18" s="79" t="inlineStr">
+      <c r="C20" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D18" s="79" t="inlineStr">
+      <c r="D20" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E18" s="79" t="inlineStr">
+      <c r="E20" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F18" s="79" t="inlineStr">
+      <c r="F20" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="105" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C19" s="105" t="inlineStr">
+      <c r="C21" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D19" s="105" t="n">
+      <c r="D21" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="105" t="n">
+      <c r="E21" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="105" t="n">
+      <c r="F21" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="96" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C20" s="96" t="inlineStr">
+      <c r="C22" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D20" s="96" t="n">
-        <v>137</v>
-      </c>
-      <c r="E20" s="96" t="n">
-        <v>2.3</v>
-      </c>
-      <c r="F20" s="96" t="n">
-        <v>44.9</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="98" t="inlineStr">
+      <c r="D22" s="96" t="n">
+        <v>145</v>
+      </c>
+      <c r="E22" s="96" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F22" s="96" t="n">
+        <v>37.3</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C21" s="98" t="inlineStr">
+      <c r="C23" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D21" s="98" t="n">
+      <c r="D23" s="98" t="n">
         <v>74</v>
       </c>
-      <c r="E21" s="98" t="n">
+      <c r="E23" s="98" t="n">
         <v>1.2</v>
       </c>
-      <c r="F21" s="98" t="n">
-        <v>24.3</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="106" t="inlineStr">
+      <c r="F23" s="98" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C22" s="106" t="inlineStr">
+      <c r="C24" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D22" s="106" t="n">
+      <c r="D24" s="106" t="n">
         <v>35</v>
       </c>
-      <c r="E22" s="106" t="n">
+      <c r="E24" s="106" t="n">
         <v>0.6</v>
       </c>
-      <c r="F22" s="106" t="n">
-        <v>11.5</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="100" t="inlineStr">
+      <c r="F24" s="106" t="n">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C23" s="100" t="inlineStr">
+      <c r="C25" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D23" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="E23" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="F23" s="100" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="95" t="inlineStr">
+      <c r="D25" s="100" t="n">
+        <v>76</v>
+      </c>
+      <c r="E25" s="100" t="n">
+        <v>1.3</v>
+      </c>
+      <c r="F25" s="100" t="n">
+        <v>19.5</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C24" s="95" t="inlineStr">
+      <c r="C26" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D24" s="95" t="n">
+      <c r="D26" s="95" t="n">
         <v>59</v>
       </c>
-      <c r="E24" s="95" t="n">
+      <c r="E26" s="95" t="n">
         <v>1</v>
       </c>
-      <c r="F24" s="95" t="n">
-        <v>19.3</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="107" t="inlineStr">
+      <c r="F26" s="95" t="n">
+        <v>15.2</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D25" s="107" t="n">
-        <v>305</v>
-      </c>
-      <c r="E25" s="107" t="n">
-        <v>5.1</v>
-      </c>
-      <c r="F25" s="107" t="n">
+      <c r="D27" s="107" t="n">
+        <v>389</v>
+      </c>
+      <c r="E27" s="107" t="n">
+        <v>6.5</v>
+      </c>
+      <c r="F27" s="107" t="n">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B4:G4"/>
+  <mergeCells count="1">
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-06-02: close メール事務処理 14:33-15:21, start 見積もり業務 15:21
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14086,7 +14086,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G27"/>
+  <dimension ref="A1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14614,189 +14614,219 @@
       </c>
       <c r="F18" s="100" t="inlineStr">
         <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="G18" s="100" t="n">
+        <v>48</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="101" t="inlineStr">
+        <is>
+          <t>見積もり業務</t>
+        </is>
+      </c>
+      <c r="E19" s="100" t="inlineStr">
+        <is>
+          <t>15:21</t>
+        </is>
+      </c>
+      <c r="F19" s="100" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G18" s="100" t="n"/>
-    </row>
-    <row r="19">
-      <c r="B19" s="104" t="inlineStr">
+      <c r="G19" s="100" t="n"/>
+    </row>
+    <row r="20">
+      <c r="B20" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C19" s="93" t="n"/>
-      <c r="D19" s="93" t="n"/>
-      <c r="E19" s="93" t="n"/>
-      <c r="F19" s="93" t="n"/>
-      <c r="G19" s="94" t="n"/>
-    </row>
-    <row r="20">
-      <c r="B20" s="79" t="inlineStr">
+      <c r="C20" s="93" t="n"/>
+      <c r="D20" s="93" t="n"/>
+      <c r="E20" s="93" t="n"/>
+      <c r="F20" s="93" t="n"/>
+      <c r="G20" s="94" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C20" s="79" t="inlineStr">
+      <c r="C21" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D20" s="79" t="inlineStr">
+      <c r="D21" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E20" s="79" t="inlineStr">
+      <c r="E21" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F20" s="79" t="inlineStr">
+      <c r="F21" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="105" t="inlineStr">
+    <row r="22">
+      <c r="B22" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C21" s="105" t="inlineStr">
+      <c r="C22" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D21" s="105" t="n">
+      <c r="D22" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E21" s="105" t="n">
+      <c r="E22" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F21" s="105" t="n">
+      <c r="F22" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="22">
-      <c r="B22" s="96" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C22" s="96" t="inlineStr">
+      <c r="C23" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D22" s="96" t="n">
+      <c r="D23" s="96" t="n">
         <v>145</v>
       </c>
-      <c r="E22" s="96" t="n">
+      <c r="E23" s="96" t="n">
         <v>2.4</v>
       </c>
-      <c r="F22" s="96" t="n">
-        <v>37.3</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="98" t="inlineStr">
+      <c r="F23" s="96" t="n">
+        <v>33.2</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C23" s="98" t="inlineStr">
+      <c r="C24" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D23" s="98" t="n">
+      <c r="D24" s="98" t="n">
         <v>74</v>
       </c>
-      <c r="E23" s="98" t="n">
+      <c r="E24" s="98" t="n">
         <v>1.2</v>
       </c>
-      <c r="F23" s="98" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="106" t="inlineStr">
+      <c r="F24" s="98" t="n">
+        <v>16.9</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C24" s="106" t="inlineStr">
+      <c r="C25" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D24" s="106" t="n">
+      <c r="D25" s="106" t="n">
         <v>35</v>
       </c>
-      <c r="E24" s="106" t="n">
+      <c r="E25" s="106" t="n">
         <v>0.6</v>
       </c>
-      <c r="F24" s="106" t="n">
-        <v>9</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="100" t="inlineStr">
+      <c r="F25" s="106" t="n">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C25" s="100" t="inlineStr">
+      <c r="C26" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D25" s="100" t="n">
-        <v>76</v>
-      </c>
-      <c r="E25" s="100" t="n">
-        <v>1.3</v>
-      </c>
-      <c r="F25" s="100" t="n">
-        <v>19.5</v>
-      </c>
-    </row>
-    <row r="26">
-      <c r="B26" s="95" t="inlineStr">
+      <c r="D26" s="100" t="n">
+        <v>124</v>
+      </c>
+      <c r="E26" s="100" t="n">
+        <v>2.1</v>
+      </c>
+      <c r="F26" s="100" t="n">
+        <v>28.4</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C26" s="95" t="inlineStr">
+      <c r="C27" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D26" s="95" t="n">
+      <c r="D27" s="95" t="n">
         <v>59</v>
       </c>
-      <c r="E26" s="95" t="n">
+      <c r="E27" s="95" t="n">
         <v>1</v>
       </c>
-      <c r="F26" s="95" t="n">
-        <v>15.2</v>
-      </c>
-    </row>
-    <row r="27">
-      <c r="B27" s="107" t="inlineStr">
+      <c r="F27" s="95" t="n">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D27" s="107" t="n">
-        <v>389</v>
-      </c>
-      <c r="E27" s="107" t="n">
-        <v>6.5</v>
-      </c>
-      <c r="F27" s="107" t="n">
+      <c r="D28" s="107" t="n">
+        <v>437</v>
+      </c>
+      <c r="E28" s="107" t="n">
+        <v>7.3</v>
+      </c>
+      <c r="F28" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-02: close 見積もり業務 15:21-18:00, 業務終了
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14644,10 +14644,12 @@
       </c>
       <c r="F19" s="100" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G19" s="100" t="n"/>
+          <t>18:00</t>
+        </is>
+      </c>
+      <c r="G19" s="100" t="n">
+        <v>159</v>
+      </c>
     </row>
     <row r="20">
       <c r="B20" s="104" t="inlineStr">
@@ -14727,7 +14729,7 @@
         <v>2.4</v>
       </c>
       <c r="F23" s="96" t="n">
-        <v>33.2</v>
+        <v>24.3</v>
       </c>
     </row>
     <row r="24">
@@ -14748,7 +14750,7 @@
         <v>1.2</v>
       </c>
       <c r="F24" s="98" t="n">
-        <v>16.9</v>
+        <v>12.4</v>
       </c>
     </row>
     <row r="25">
@@ -14769,7 +14771,7 @@
         <v>0.6</v>
       </c>
       <c r="F25" s="106" t="n">
-        <v>8</v>
+        <v>5.9</v>
       </c>
     </row>
     <row r="26">
@@ -14784,13 +14786,13 @@
         </is>
       </c>
       <c r="D26" s="100" t="n">
-        <v>124</v>
+        <v>283</v>
       </c>
       <c r="E26" s="100" t="n">
-        <v>2.1</v>
+        <v>4.7</v>
       </c>
       <c r="F26" s="100" t="n">
-        <v>28.4</v>
+        <v>47.5</v>
       </c>
     </row>
     <row r="27">
@@ -14811,7 +14813,7 @@
         <v>1</v>
       </c>
       <c r="F27" s="95" t="n">
-        <v>13.5</v>
+        <v>9.9</v>
       </c>
     </row>
     <row r="28">
@@ -14821,10 +14823,10 @@
         </is>
       </c>
       <c r="D28" s="107" t="n">
-        <v>437</v>
+        <v>596</v>
       </c>
       <c r="E28" s="107" t="n">
-        <v>7.3</v>
+        <v>9.9</v>
       </c>
       <c r="F28" s="107" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add 2026-06-03: new sheet, tasks 7:59-9:20, メール対応 in progress
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -23,14 +23,15 @@
     <sheet name="2026-05-29" sheetId="15" state="visible" r:id="rId15"/>
     <sheet name="2026-06-01" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="2026-06-02" sheetId="17" state="visible" r:id="rId17"/>
+    <sheet name="2026-06-03" sheetId="18" state="visible" r:id="rId18"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId18"/>
     <externalReference r:id="rId19"/>
     <externalReference r:id="rId20"/>
     <externalReference r:id="rId21"/>
     <externalReference r:id="rId22"/>
     <externalReference r:id="rId23"/>
+    <externalReference r:id="rId24"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -14086,7 +14087,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G28"/>
+  <dimension ref="B1:G28"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14834,6 +14835,395 @@
     </row>
   </sheetData>
   <mergeCells count="1">
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
+<file path=xl/worksheets/sheet18.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G16"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="64" min="2" max="2"/>
+    <col width="18" customWidth="1" style="64" min="3" max="3"/>
+    <col width="42" customWidth="1" style="64" min="4" max="4"/>
+    <col width="8" customWidth="1" style="64" min="5" max="5"/>
+    <col width="8" customWidth="1" style="64" min="6" max="6"/>
+    <col width="12" customWidth="1" style="64" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" s="64">
+      <c r="B1" s="102" t="inlineStr">
+        <is>
+          <t>2026年6月3日（水）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="64">
+      <c r="B2" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C2" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D2" s="79" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E2" s="79" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F2" s="79" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G2" s="79" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="64">
+      <c r="B3" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C3" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D3" s="103" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E3" s="95" t="inlineStr">
+        <is>
+          <t>7:59</t>
+        </is>
+      </c>
+      <c r="F3" s="95" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G3" s="95" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="64">
+      <c r="B4" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C4" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E4" s="96" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F4" s="96" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G4" s="96" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="64">
+      <c r="B5" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C5" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E5" s="98" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F5" s="98" t="inlineStr">
+        <is>
+          <t>8:30</t>
+        </is>
+      </c>
+      <c r="G5" s="98" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="64">
+      <c r="B6" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C6" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D6" s="97" t="inlineStr">
+        <is>
+          <t>5S推進委員会 事前調査</t>
+        </is>
+      </c>
+      <c r="E6" s="96" t="inlineStr">
+        <is>
+          <t>8:30</t>
+        </is>
+      </c>
+      <c r="F6" s="96" t="inlineStr">
+        <is>
+          <t>9:20</t>
+        </is>
+      </c>
+      <c r="G6" s="96" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C7" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D7" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック・返信・客先確認メール</t>
+        </is>
+      </c>
+      <c r="E7" s="100" t="inlineStr">
+        <is>
+          <t>9:20</t>
+        </is>
+      </c>
+      <c r="F7" s="100" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G7" s="100" t="n"/>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="104" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C9" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D9" s="79" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E9" s="79" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F9" s="79" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="105" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C10" s="105" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D10" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E10" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F10" s="105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C11" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D11" s="96" t="n">
+        <v>53</v>
+      </c>
+      <c r="E11" s="96" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F11" s="96" t="n">
+        <v>65.40000000000001</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C12" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D12" s="98" t="n">
+        <v>24</v>
+      </c>
+      <c r="E12" s="98" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F12" s="98" t="n">
+        <v>29.6</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C13" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D13" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E13" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F13" s="106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C14" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D14" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="E14" s="100" t="n">
+        <v>0</v>
+      </c>
+      <c r="F14" s="100" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C15" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D15" s="95" t="n">
+        <v>4</v>
+      </c>
+      <c r="E15" s="95" t="n">
+        <v>0.1</v>
+      </c>
+      <c r="F15" s="95" t="n">
+        <v>4.9</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="107" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="D16" s="107" t="n">
+        <v>81</v>
+      </c>
+      <c r="E16" s="107" t="n">
+        <v>1.4</v>
+      </c>
+      <c r="F16" s="107" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B8:G8"/>
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-06-03: close メール対応 9:20-10:00, 休憩 10:00-10:10
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G16"/>
+  <dimension ref="A1:G17"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -14864,6 +14864,11 @@
           <t>2026年6月3日（水）　業務記録</t>
         </is>
       </c>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="94" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1" s="64">
       <c r="B2" s="79" t="inlineStr">
@@ -15040,184 +15045,221 @@
       </c>
       <c r="F7" s="100" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G7" s="100" t="n"/>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="G7" s="100" t="n">
+        <v>40</v>
+      </c>
     </row>
     <row r="8" ht="18" customHeight="1" s="64">
-      <c r="B8" s="104" t="inlineStr">
+      <c r="B8" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C8" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D8" s="103" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E8" s="95" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F8" s="95" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G8" s="95" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9">
+      <c r="B9" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="79" t="inlineStr">
+      <c r="C9" s="93" t="n"/>
+      <c r="D9" s="93" t="n"/>
+      <c r="E9" s="93" t="n"/>
+      <c r="F9" s="93" t="n"/>
+      <c r="G9" s="94" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C9" s="79" t="inlineStr">
+      <c r="C10" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D9" s="79" t="inlineStr">
+      <c r="D10" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E9" s="79" t="inlineStr">
+      <c r="E10" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F9" s="79" t="inlineStr">
+      <c r="F10" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="18" customHeight="1" s="64">
-      <c r="B10" s="105" t="inlineStr">
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C10" s="105" t="inlineStr">
+      <c r="C11" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D10" s="105" t="n">
+      <c r="D11" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E10" s="105" t="n">
+      <c r="E11" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F10" s="105" t="n">
+      <c r="F11" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="11" ht="18" customHeight="1" s="64">
-      <c r="B11" s="96" t="inlineStr">
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C11" s="96" t="inlineStr">
+      <c r="C12" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D11" s="96" t="n">
+      <c r="D12" s="96" t="n">
         <v>53</v>
       </c>
-      <c r="E11" s="96" t="n">
+      <c r="E12" s="96" t="n">
         <v>0.9</v>
       </c>
-      <c r="F11" s="96" t="n">
-        <v>65.40000000000001</v>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="98" t="inlineStr">
+      <c r="F12" s="96" t="n">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C12" s="98" t="inlineStr">
+      <c r="C13" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D12" s="98" t="n">
+      <c r="D13" s="98" t="n">
         <v>24</v>
       </c>
-      <c r="E12" s="98" t="n">
+      <c r="E13" s="98" t="n">
         <v>0.4</v>
       </c>
-      <c r="F12" s="98" t="n">
-        <v>29.6</v>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="64">
-      <c r="B13" s="106" t="inlineStr">
+      <c r="F13" s="98" t="n">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C13" s="106" t="inlineStr">
+      <c r="C14" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D13" s="106" t="n">
+      <c r="D14" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E13" s="106" t="n">
+      <c r="E14" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F13" s="106" t="n">
+      <c r="F14" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="100" t="inlineStr">
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C14" s="100" t="inlineStr">
+      <c r="C15" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D14" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="100" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="100" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="95" t="inlineStr">
+      <c r="D15" s="100" t="n">
+        <v>40</v>
+      </c>
+      <c r="E15" s="100" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F15" s="100" t="n">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C15" s="95" t="inlineStr">
+      <c r="C16" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D15" s="95" t="n">
-        <v>4</v>
-      </c>
-      <c r="E15" s="95" t="n">
-        <v>0.1</v>
-      </c>
-      <c r="F15" s="95" t="n">
-        <v>4.9</v>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="107" t="inlineStr">
+      <c r="D16" s="95" t="n">
+        <v>14</v>
+      </c>
+      <c r="E16" s="95" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F16" s="95" t="n">
+        <v>10.7</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D16" s="107" t="n">
-        <v>81</v>
-      </c>
-      <c r="E16" s="107" t="n">
-        <v>1.4</v>
-      </c>
-      <c r="F16" s="107" t="n">
+      <c r="D17" s="107" t="n">
+        <v>131</v>
+      </c>
+      <c r="E17" s="107" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F17" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-03: start 5S推進委員会 事前検討会 10:10
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G17"/>
+  <dimension ref="A1:G18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15058,208 +15058,218 @@
           <t>⑥</t>
         </is>
       </c>
-      <c r="C8" s="95" t="inlineStr">
+      <c r="C8" s="93" t="n"/>
+      <c r="D8" s="93" t="n"/>
+      <c r="E8" s="93" t="n"/>
+      <c r="F8" s="93" t="n"/>
+      <c r="G8" s="94" t="n"/>
+    </row>
+    <row r="9">
+      <c r="B9" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C9" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D9" s="97" t="inlineStr">
+        <is>
+          <t>5S推進委員会 事前検討会</t>
+        </is>
+      </c>
+      <c r="E9" s="96" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F9" s="96" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G9" s="96" t="n"/>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="104" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+      <c r="C10" s="93" t="n"/>
+      <c r="D10" s="93" t="n"/>
+      <c r="E10" s="93" t="n"/>
+      <c r="F10" s="93" t="n"/>
+      <c r="G10" s="94" t="n"/>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C11" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D11" s="79" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E11" s="79" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F11" s="79" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="105" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C12" s="105" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D12" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E12" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F12" s="105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C13" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D13" s="96" t="n">
+        <v>53</v>
+      </c>
+      <c r="E13" s="96" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F13" s="96" t="n">
+        <v>40.5</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C14" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D14" s="98" t="n">
+        <v>24</v>
+      </c>
+      <c r="E14" s="98" t="n">
+        <v>0.4</v>
+      </c>
+      <c r="F14" s="98" t="n">
+        <v>18.3</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C15" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D15" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C16" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D16" s="100" t="n">
+        <v>40</v>
+      </c>
+      <c r="E16" s="100" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F16" s="100" t="n">
+        <v>30.5</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C17" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D8" s="103" t="inlineStr">
-        <is>
-          <t>休憩</t>
-        </is>
-      </c>
-      <c r="E8" s="95" t="inlineStr">
-        <is>
-          <t>10:00</t>
-        </is>
-      </c>
-      <c r="F8" s="95" t="inlineStr">
-        <is>
-          <t>10:10</t>
-        </is>
-      </c>
-      <c r="G8" s="95" t="n">
-        <v>10</v>
-      </c>
-    </row>
-    <row r="9">
-      <c r="B9" s="104" t="inlineStr">
-        <is>
-          <t>【カテゴリ別集計】</t>
-        </is>
-      </c>
-      <c r="C9" s="93" t="n"/>
-      <c r="D9" s="93" t="n"/>
-      <c r="E9" s="93" t="n"/>
-      <c r="F9" s="93" t="n"/>
-      <c r="G9" s="94" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" s="64">
-      <c r="B10" s="79" t="inlineStr">
-        <is>
-          <t>No.</t>
-        </is>
-      </c>
-      <c r="C10" s="79" t="inlineStr">
-        <is>
-          <t>カテゴリ名</t>
-        </is>
-      </c>
-      <c r="D10" s="79" t="inlineStr">
-        <is>
-          <t>合計（分）</t>
-        </is>
-      </c>
-      <c r="E10" s="79" t="inlineStr">
-        <is>
-          <t>合計（時間）</t>
-        </is>
-      </c>
-      <c r="F10" s="79" t="inlineStr">
-        <is>
-          <t>割合（%）</t>
-        </is>
-      </c>
-    </row>
-    <row r="11" ht="18" customHeight="1" s="64">
-      <c r="B11" s="105" t="inlineStr">
-        <is>
-          <t>①</t>
-        </is>
-      </c>
-      <c r="C11" s="105" t="inlineStr">
-        <is>
-          <t>経営・対外業務</t>
-        </is>
-      </c>
-      <c r="D11" s="105" t="n">
-        <v>0</v>
-      </c>
-      <c r="E11" s="105" t="n">
-        <v>0</v>
-      </c>
-      <c r="F11" s="105" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="96" t="inlineStr">
-        <is>
-          <t>②</t>
-        </is>
-      </c>
-      <c r="C12" s="96" t="inlineStr">
-        <is>
-          <t>社内マネジメント</t>
-        </is>
-      </c>
-      <c r="D12" s="96" t="n">
-        <v>53</v>
-      </c>
-      <c r="E12" s="96" t="n">
-        <v>0.9</v>
-      </c>
-      <c r="F12" s="96" t="n">
-        <v>40.5</v>
-      </c>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="64">
-      <c r="B13" s="98" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C13" s="98" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D13" s="98" t="n">
-        <v>24</v>
-      </c>
-      <c r="E13" s="98" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F13" s="98" t="n">
-        <v>18.3</v>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="106" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C14" s="106" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D14" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="E14" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="F14" s="106" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="100" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C15" s="100" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D15" s="100" t="n">
-        <v>40</v>
-      </c>
-      <c r="E15" s="100" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F15" s="100" t="n">
-        <v>30.5</v>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="95" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="C16" s="95" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D16" s="95" t="n">
+      <c r="D17" s="95" t="n">
         <v>14</v>
       </c>
-      <c r="E16" s="95" t="n">
+      <c r="E17" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F16" s="95" t="n">
+      <c r="F17" s="95" t="n">
         <v>10.7</v>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="107" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D17" s="107" t="n">
+      <c r="D18" s="107" t="n">
         <v>131</v>
       </c>
-      <c r="E17" s="107" t="n">
+      <c r="E18" s="107" t="n">
         <v>2.2</v>
       </c>
-      <c r="F17" s="107" t="n">
+      <c r="F18" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-03: 事前検討会 10:10-11:00, 現場周り 11:00-11:30, start 事務作業 11:30
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G18"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15087,189 +15087,249 @@
       </c>
       <c r="F9" s="96" t="inlineStr">
         <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="G9" s="96" t="n">
+        <v>50</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C10" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D10" s="99" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E10" s="98" t="inlineStr">
+        <is>
+          <t>11:00</t>
+        </is>
+      </c>
+      <c r="F10" s="98" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G10" s="98" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C11" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D11" s="101" t="inlineStr">
+        <is>
+          <t>事務作業</t>
+        </is>
+      </c>
+      <c r="E11" s="100" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="F11" s="100" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G9" s="96" t="n"/>
-    </row>
-    <row r="10" ht="18" customHeight="1" s="64">
-      <c r="B10" s="104" t="inlineStr">
+      <c r="G11" s="100" t="n"/>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C10" s="93" t="n"/>
-      <c r="D10" s="93" t="n"/>
-      <c r="E10" s="93" t="n"/>
-      <c r="F10" s="93" t="n"/>
-      <c r="G10" s="94" t="n"/>
-    </row>
-    <row r="11" ht="18" customHeight="1" s="64">
-      <c r="B11" s="79" t="inlineStr">
+      <c r="C12" s="93" t="n"/>
+      <c r="D12" s="93" t="n"/>
+      <c r="E12" s="93" t="n"/>
+      <c r="F12" s="93" t="n"/>
+      <c r="G12" s="94" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C11" s="79" t="inlineStr">
+      <c r="C13" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D11" s="79" t="inlineStr">
+      <c r="D13" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E11" s="79" t="inlineStr">
+      <c r="E13" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F11" s="79" t="inlineStr">
+      <c r="F13" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="105" t="inlineStr">
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C12" s="105" t="inlineStr">
+      <c r="C14" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D12" s="105" t="n">
+      <c r="D14" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E12" s="105" t="n">
+      <c r="E14" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F12" s="105" t="n">
+      <c r="F14" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="13" ht="18" customHeight="1" s="64">
-      <c r="B13" s="96" t="inlineStr">
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C13" s="96" t="inlineStr">
+      <c r="C15" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D13" s="96" t="n">
-        <v>53</v>
-      </c>
-      <c r="E13" s="96" t="n">
+      <c r="D15" s="96" t="n">
+        <v>103</v>
+      </c>
+      <c r="E15" s="96" t="n">
+        <v>1.7</v>
+      </c>
+      <c r="F15" s="96" t="n">
+        <v>48.8</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C16" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D16" s="98" t="n">
+        <v>54</v>
+      </c>
+      <c r="E16" s="98" t="n">
         <v>0.9</v>
       </c>
-      <c r="F13" s="96" t="n">
-        <v>40.5</v>
-      </c>
-    </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="98" t="inlineStr">
-        <is>
-          <t>③</t>
-        </is>
-      </c>
-      <c r="C14" s="98" t="inlineStr">
-        <is>
-          <t>現場管理・監督</t>
-        </is>
-      </c>
-      <c r="D14" s="98" t="n">
-        <v>24</v>
-      </c>
-      <c r="E14" s="98" t="n">
-        <v>0.4</v>
-      </c>
-      <c r="F14" s="98" t="n">
-        <v>18.3</v>
-      </c>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="106" t="inlineStr">
+      <c r="F16" s="98" t="n">
+        <v>25.6</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C15" s="106" t="inlineStr">
+      <c r="C17" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D15" s="106" t="n">
+      <c r="D17" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="106" t="n">
+      <c r="E17" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="106" t="n">
+      <c r="F17" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="100" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C16" s="100" t="inlineStr">
+      <c r="C18" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D16" s="100" t="n">
+      <c r="D18" s="100" t="n">
         <v>40</v>
       </c>
-      <c r="E16" s="100" t="n">
+      <c r="E18" s="100" t="n">
         <v>0.7</v>
       </c>
-      <c r="F16" s="100" t="n">
-        <v>30.5</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="95" t="inlineStr">
+      <c r="F18" s="100" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C17" s="95" t="inlineStr">
+      <c r="C19" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D17" s="95" t="n">
+      <c r="D19" s="95" t="n">
         <v>14</v>
       </c>
-      <c r="E17" s="95" t="n">
+      <c r="E19" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F17" s="95" t="n">
-        <v>10.7</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="107" t="inlineStr">
+      <c r="F19" s="95" t="n">
+        <v>6.6</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D18" s="107" t="n">
-        <v>131</v>
-      </c>
-      <c r="E18" s="107" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="F18" s="107" t="n">
+      <c r="D20" s="107" t="n">
+        <v>211</v>
+      </c>
+      <c r="E20" s="107" t="n">
+        <v>3.5</v>
+      </c>
+      <c r="F20" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-03: fix duplicates, 出荷品準備打ち合わせ 11:40-11:50, 事務作業再開 11:50
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G20"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15058,11 +15058,29 @@
           <t>⑥</t>
         </is>
       </c>
-      <c r="C8" s="93" t="n"/>
-      <c r="D8" s="93" t="n"/>
-      <c r="E8" s="93" t="n"/>
-      <c r="F8" s="93" t="n"/>
-      <c r="G8" s="94" t="n"/>
+      <c r="C8" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D8" s="103" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E8" s="95" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F8" s="95" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G8" s="95" t="n">
+        <v>10</v>
+      </c>
     </row>
     <row r="9">
       <c r="B9" s="96" t="inlineStr">
@@ -15147,195 +15165,254 @@
       </c>
       <c r="F11" s="100" t="inlineStr">
         <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="G11" s="100" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C12" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D12" s="97" t="inlineStr">
+        <is>
+          <t>出荷品準備 打ち合わせ</t>
+        </is>
+      </c>
+      <c r="E12" s="96" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="F12" s="96" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="G12" s="96" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C13" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D13" s="101" t="inlineStr">
+        <is>
+          <t>事務作業</t>
+        </is>
+      </c>
+      <c r="E13" s="100" t="inlineStr">
+        <is>
+          <t>11:50</t>
+        </is>
+      </c>
+      <c r="F13" s="100" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G11" s="100" t="n"/>
-    </row>
-    <row r="12" ht="18" customHeight="1" s="64">
-      <c r="B12" s="104" t="inlineStr">
+      <c r="G13" s="100" t="n"/>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C12" s="93" t="n"/>
-      <c r="D12" s="93" t="n"/>
-      <c r="E12" s="93" t="n"/>
-      <c r="F12" s="93" t="n"/>
-      <c r="G12" s="94" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="64">
-      <c r="B13" s="79" t="inlineStr">
+      <c r="C14" s="93" t="n"/>
+      <c r="D14" s="93" t="n"/>
+      <c r="E14" s="93" t="n"/>
+      <c r="F14" s="93" t="n"/>
+      <c r="G14" s="94" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C13" s="79" t="inlineStr">
+      <c r="C15" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D13" s="79" t="inlineStr">
+      <c r="D15" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E13" s="79" t="inlineStr">
+      <c r="E15" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F13" s="79" t="inlineStr">
+      <c r="F15" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="105" t="inlineStr">
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C14" s="105" t="inlineStr">
+      <c r="C16" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D14" s="105" t="n">
+      <c r="D16" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E14" s="105" t="n">
+      <c r="E16" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F14" s="105" t="n">
+      <c r="F16" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="96" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C15" s="96" t="inlineStr">
+      <c r="C17" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D15" s="96" t="n">
-        <v>103</v>
-      </c>
-      <c r="E15" s="96" t="n">
-        <v>1.7</v>
-      </c>
-      <c r="F15" s="96" t="n">
-        <v>48.8</v>
-      </c>
-    </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="98" t="inlineStr">
+      <c r="D17" s="96" t="n">
+        <v>113</v>
+      </c>
+      <c r="E17" s="96" t="n">
+        <v>1.9</v>
+      </c>
+      <c r="F17" s="96" t="n">
+        <v>48.9</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C16" s="98" t="inlineStr">
+      <c r="C18" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D16" s="98" t="n">
+      <c r="D18" s="98" t="n">
         <v>54</v>
       </c>
-      <c r="E16" s="98" t="n">
+      <c r="E18" s="98" t="n">
         <v>0.9</v>
       </c>
-      <c r="F16" s="98" t="n">
-        <v>25.6</v>
-      </c>
-    </row>
-    <row r="17">
-      <c r="B17" s="106" t="inlineStr">
+      <c r="F18" s="98" t="n">
+        <v>23.4</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C17" s="106" t="inlineStr">
+      <c r="C19" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D17" s="106" t="n">
+      <c r="D19" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="106" t="n">
+      <c r="E19" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="106" t="n">
+      <c r="F19" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="100" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C18" s="100" t="inlineStr">
+      <c r="C20" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D18" s="100" t="n">
-        <v>40</v>
-      </c>
-      <c r="E18" s="100" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F18" s="100" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="95" t="inlineStr">
+      <c r="D20" s="100" t="n">
+        <v>50</v>
+      </c>
+      <c r="E20" s="100" t="n">
+        <v>0.8</v>
+      </c>
+      <c r="F20" s="100" t="n">
+        <v>21.6</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C19" s="95" t="inlineStr">
+      <c r="C21" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D19" s="95" t="n">
+      <c r="D21" s="95" t="n">
         <v>14</v>
       </c>
-      <c r="E19" s="95" t="n">
+      <c r="E21" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F19" s="95" t="n">
-        <v>6.6</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="107" t="inlineStr">
+      <c r="F21" s="95" t="n">
+        <v>6.1</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D20" s="107" t="n">
-        <v>211</v>
-      </c>
-      <c r="E20" s="107" t="n">
-        <v>3.5</v>
-      </c>
-      <c r="F20" s="107" t="n">
+      <c r="D22" s="107" t="n">
+        <v>231</v>
+      </c>
+      <c r="E22" s="107" t="n">
+        <v>3.9</v>
+      </c>
+      <c r="F22" s="107" t="n">
         <v>100</v>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="2">
-    <mergeCell ref="B8:G8"/>
+  <mergeCells count="1">
     <mergeCell ref="B1:G1"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
Update 2026-06-03: close 事務作業 11:50-11:55, start 製品検査打ち合わせ 11:55
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="A1:G23"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15225,189 +15225,219 @@
       </c>
       <c r="F13" s="100" t="inlineStr">
         <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="G13" s="100" t="n">
+        <v>5</v>
+      </c>
+    </row>
+    <row r="14" ht="18" customHeight="1" s="64">
+      <c r="B14" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C14" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D14" s="97" t="inlineStr">
+        <is>
+          <t>製品検査 打ち合わせ</t>
+        </is>
+      </c>
+      <c r="E14" s="96" t="inlineStr">
+        <is>
+          <t>11:55</t>
+        </is>
+      </c>
+      <c r="F14" s="96" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G13" s="100" t="n"/>
-    </row>
-    <row r="14" ht="18" customHeight="1" s="64">
-      <c r="B14" s="104" t="inlineStr">
+      <c r="G14" s="96" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C14" s="93" t="n"/>
-      <c r="D14" s="93" t="n"/>
-      <c r="E14" s="93" t="n"/>
-      <c r="F14" s="93" t="n"/>
-      <c r="G14" s="94" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="79" t="inlineStr">
+      <c r="C15" s="93" t="n"/>
+      <c r="D15" s="93" t="n"/>
+      <c r="E15" s="93" t="n"/>
+      <c r="F15" s="93" t="n"/>
+      <c r="G15" s="94" t="n"/>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C15" s="79" t="inlineStr">
+      <c r="C16" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D15" s="79" t="inlineStr">
+      <c r="D16" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E15" s="79" t="inlineStr">
+      <c r="E16" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F15" s="79" t="inlineStr">
+      <c r="F16" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="105" t="inlineStr">
+    <row r="17">
+      <c r="B17" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C16" s="105" t="inlineStr">
+      <c r="C17" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D16" s="105" t="n">
+      <c r="D17" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E16" s="105" t="n">
+      <c r="E17" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F16" s="105" t="n">
+      <c r="F17" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="96" t="inlineStr">
+    <row r="18">
+      <c r="B18" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C17" s="96" t="inlineStr">
+      <c r="C18" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D17" s="96" t="n">
+      <c r="D18" s="96" t="n">
         <v>113</v>
       </c>
-      <c r="E17" s="96" t="n">
+      <c r="E18" s="96" t="n">
         <v>1.9</v>
       </c>
-      <c r="F17" s="96" t="n">
-        <v>48.9</v>
-      </c>
-    </row>
-    <row r="18">
-      <c r="B18" s="98" t="inlineStr">
+      <c r="F18" s="96" t="n">
+        <v>47.9</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C18" s="98" t="inlineStr">
+      <c r="C19" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D18" s="98" t="n">
+      <c r="D19" s="98" t="n">
         <v>54</v>
       </c>
-      <c r="E18" s="98" t="n">
+      <c r="E19" s="98" t="n">
         <v>0.9</v>
       </c>
-      <c r="F18" s="98" t="n">
-        <v>23.4</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="106" t="inlineStr">
+      <c r="F19" s="98" t="n">
+        <v>22.9</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C19" s="106" t="inlineStr">
+      <c r="C20" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D19" s="106" t="n">
+      <c r="D20" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="106" t="n">
+      <c r="E20" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="106" t="n">
+      <c r="F20" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="100" t="inlineStr">
+    <row r="21">
+      <c r="B21" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C20" s="100" t="inlineStr">
+      <c r="C21" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D20" s="100" t="n">
-        <v>50</v>
-      </c>
-      <c r="E20" s="100" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="F20" s="100" t="n">
-        <v>21.6</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="95" t="inlineStr">
+      <c r="D21" s="100" t="n">
+        <v>55</v>
+      </c>
+      <c r="E21" s="100" t="n">
+        <v>0.9</v>
+      </c>
+      <c r="F21" s="100" t="n">
+        <v>23.3</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C21" s="95" t="inlineStr">
+      <c r="C22" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D21" s="95" t="n">
+      <c r="D22" s="95" t="n">
         <v>14</v>
       </c>
-      <c r="E21" s="95" t="n">
+      <c r="E22" s="95" t="n">
         <v>0.2</v>
       </c>
-      <c r="F21" s="95" t="n">
-        <v>6.1</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="107" t="inlineStr">
+      <c r="F22" s="95" t="n">
+        <v>5.9</v>
+      </c>
+    </row>
+    <row r="23">
+      <c r="B23" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D22" s="107" t="n">
-        <v>231</v>
-      </c>
-      <c r="E22" s="107" t="n">
+      <c r="D23" s="107" t="n">
+        <v>236</v>
+      </c>
+      <c r="E23" s="107" t="n">
         <v>3.9</v>
       </c>
-      <c r="F22" s="107" t="n">
+      <c r="F23" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-03: 製品検査打ち合わせclose, 昼休憩 12:15-12:43, start 掃除 12:43
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G23"/>
+  <dimension ref="A1:G25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15255,189 +15255,249 @@
       </c>
       <c r="F14" s="96" t="inlineStr">
         <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="G14" s="96" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C15" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D15" s="103" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E15" s="95" t="inlineStr">
+        <is>
+          <t>12:15</t>
+        </is>
+      </c>
+      <c r="F15" s="95" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="G15" s="95" t="n">
+        <v>28</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C16" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D16" s="103" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E16" s="95" t="inlineStr">
+        <is>
+          <t>12:43</t>
+        </is>
+      </c>
+      <c r="F16" s="95" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G14" s="96" t="n"/>
-    </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="104" t="inlineStr">
+      <c r="G16" s="95" t="n"/>
+    </row>
+    <row r="17">
+      <c r="B17" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C15" s="93" t="n"/>
-      <c r="D15" s="93" t="n"/>
-      <c r="E15" s="93" t="n"/>
-      <c r="F15" s="93" t="n"/>
-      <c r="G15" s="94" t="n"/>
-    </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="79" t="inlineStr">
+      <c r="C17" s="93" t="n"/>
+      <c r="D17" s="93" t="n"/>
+      <c r="E17" s="93" t="n"/>
+      <c r="F17" s="93" t="n"/>
+      <c r="G17" s="94" t="n"/>
+    </row>
+    <row r="18">
+      <c r="B18" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C16" s="79" t="inlineStr">
+      <c r="C18" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D16" s="79" t="inlineStr">
+      <c r="D18" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E16" s="79" t="inlineStr">
+      <c r="E18" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F16" s="79" t="inlineStr">
+      <c r="F18" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="17">
-      <c r="B17" s="105" t="inlineStr">
+    <row r="19">
+      <c r="B19" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C17" s="105" t="inlineStr">
+      <c r="C19" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D17" s="105" t="n">
+      <c r="D19" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E17" s="105" t="n">
+      <c r="E19" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F17" s="105" t="n">
+      <c r="F19" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="18">
-      <c r="B18" s="96" t="inlineStr">
+    <row r="20">
+      <c r="B20" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C18" s="96" t="inlineStr">
+      <c r="C20" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D18" s="96" t="n">
-        <v>113</v>
-      </c>
-      <c r="E18" s="96" t="n">
-        <v>1.9</v>
-      </c>
-      <c r="F18" s="96" t="n">
-        <v>47.9</v>
-      </c>
-    </row>
-    <row r="19">
-      <c r="B19" s="98" t="inlineStr">
+      <c r="D20" s="96" t="n">
+        <v>133</v>
+      </c>
+      <c r="E20" s="96" t="n">
+        <v>2.2</v>
+      </c>
+      <c r="F20" s="96" t="n">
+        <v>46.8</v>
+      </c>
+    </row>
+    <row r="21">
+      <c r="B21" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C19" s="98" t="inlineStr">
+      <c r="C21" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D19" s="98" t="n">
+      <c r="D21" s="98" t="n">
         <v>54</v>
       </c>
-      <c r="E19" s="98" t="n">
+      <c r="E21" s="98" t="n">
         <v>0.9</v>
       </c>
-      <c r="F19" s="98" t="n">
-        <v>22.9</v>
-      </c>
-    </row>
-    <row r="20">
-      <c r="B20" s="106" t="inlineStr">
+      <c r="F21" s="98" t="n">
+        <v>19</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C20" s="106" t="inlineStr">
+      <c r="C22" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D20" s="106" t="n">
+      <c r="D22" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E20" s="106" t="n">
+      <c r="E22" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F20" s="106" t="n">
+      <c r="F22" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="21">
-      <c r="B21" s="100" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C21" s="100" t="inlineStr">
+      <c r="C23" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D21" s="100" t="n">
+      <c r="D23" s="100" t="n">
         <v>55</v>
       </c>
-      <c r="E21" s="100" t="n">
+      <c r="E23" s="100" t="n">
         <v>0.9</v>
       </c>
-      <c r="F21" s="100" t="n">
-        <v>23.3</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="95" t="inlineStr">
+      <c r="F23" s="100" t="n">
+        <v>19.4</v>
+      </c>
+    </row>
+    <row r="24">
+      <c r="B24" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C22" s="95" t="inlineStr">
+      <c r="C24" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D22" s="95" t="n">
-        <v>14</v>
-      </c>
-      <c r="E22" s="95" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F22" s="95" t="n">
-        <v>5.9</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="107" t="inlineStr">
+      <c r="D24" s="95" t="n">
+        <v>42</v>
+      </c>
+      <c r="E24" s="95" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F24" s="95" t="n">
+        <v>14.8</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D23" s="107" t="n">
-        <v>236</v>
-      </c>
-      <c r="E23" s="107" t="n">
-        <v>3.9</v>
-      </c>
-      <c r="F23" s="107" t="n">
+      <c r="D25" s="107" t="n">
+        <v>284</v>
+      </c>
+      <c r="E25" s="107" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F25" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-03: 掃除close, 社員話/5S委員会/現場周り/雑務PC作業 12:53-15:35+
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G25"/>
+  <dimension ref="A1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15315,189 +15315,309 @@
       </c>
       <c r="F16" s="95" t="inlineStr">
         <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="G16" s="95" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="17">
+      <c r="B17" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C17" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D17" s="97" t="inlineStr">
+        <is>
+          <t>社員との話し合い</t>
+        </is>
+      </c>
+      <c r="E17" s="96" t="inlineStr">
+        <is>
+          <t>12:53</t>
+        </is>
+      </c>
+      <c r="F17" s="96" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="G17" s="96" t="n">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="18">
+      <c r="B18" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C18" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D18" s="97" t="inlineStr">
+        <is>
+          <t>5S推進委員会</t>
+        </is>
+      </c>
+      <c r="E18" s="96" t="inlineStr">
+        <is>
+          <t>13:13</t>
+        </is>
+      </c>
+      <c r="F18" s="96" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="G18" s="96" t="n">
+        <v>53</v>
+      </c>
+    </row>
+    <row r="19">
+      <c r="B19" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C19" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D19" s="99" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E19" s="98" t="inlineStr">
+        <is>
+          <t>14:06</t>
+        </is>
+      </c>
+      <c r="F19" s="98" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="G19" s="98" t="n">
+        <v>89</v>
+      </c>
+    </row>
+    <row r="20">
+      <c r="B20" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C20" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D20" s="101" t="inlineStr">
+        <is>
+          <t>雑務・PC設定・データ移行</t>
+        </is>
+      </c>
+      <c r="E20" s="100" t="inlineStr">
+        <is>
+          <t>15:35</t>
+        </is>
+      </c>
+      <c r="F20" s="100" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G16" s="95" t="n"/>
-    </row>
-    <row r="17">
-      <c r="B17" s="104" t="inlineStr">
+      <c r="G20" s="100" t="n"/>
+    </row>
+    <row r="21">
+      <c r="B21" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C17" s="93" t="n"/>
-      <c r="D17" s="93" t="n"/>
-      <c r="E17" s="93" t="n"/>
-      <c r="F17" s="93" t="n"/>
-      <c r="G17" s="94" t="n"/>
-    </row>
-    <row r="18">
-      <c r="B18" s="79" t="inlineStr">
+      <c r="C21" s="93" t="n"/>
+      <c r="D21" s="93" t="n"/>
+      <c r="E21" s="93" t="n"/>
+      <c r="F21" s="93" t="n"/>
+      <c r="G21" s="94" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C18" s="79" t="inlineStr">
+      <c r="C22" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D18" s="79" t="inlineStr">
+      <c r="D22" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E18" s="79" t="inlineStr">
+      <c r="E22" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F18" s="79" t="inlineStr">
+      <c r="F22" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="19">
-      <c r="B19" s="105" t="inlineStr">
+    <row r="23">
+      <c r="B23" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C19" s="105" t="inlineStr">
+      <c r="C23" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D19" s="105" t="n">
+      <c r="D23" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E19" s="105" t="n">
+      <c r="E23" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F19" s="105" t="n">
+      <c r="F23" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="20">
-      <c r="B20" s="96" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C20" s="96" t="inlineStr">
+      <c r="C24" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D20" s="96" t="n">
-        <v>133</v>
-      </c>
-      <c r="E20" s="96" t="n">
-        <v>2.2</v>
-      </c>
-      <c r="F20" s="96" t="n">
-        <v>46.8</v>
-      </c>
-    </row>
-    <row r="21">
-      <c r="B21" s="98" t="inlineStr">
+      <c r="D24" s="96" t="n">
+        <v>206</v>
+      </c>
+      <c r="E24" s="96" t="n">
+        <v>3.4</v>
+      </c>
+      <c r="F24" s="96" t="n">
+        <v>45.2</v>
+      </c>
+    </row>
+    <row r="25">
+      <c r="B25" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C21" s="98" t="inlineStr">
+      <c r="C25" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D21" s="98" t="n">
-        <v>54</v>
-      </c>
-      <c r="E21" s="98" t="n">
+      <c r="D25" s="98" t="n">
+        <v>143</v>
+      </c>
+      <c r="E25" s="98" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F25" s="98" t="n">
+        <v>31.4</v>
+      </c>
+    </row>
+    <row r="26">
+      <c r="B26" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C26" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D26" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E26" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F26" s="106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="27">
+      <c r="B27" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C27" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D27" s="100" t="n">
+        <v>55</v>
+      </c>
+      <c r="E27" s="100" t="n">
         <v>0.9</v>
       </c>
-      <c r="F21" s="98" t="n">
-        <v>19</v>
-      </c>
-    </row>
-    <row r="22">
-      <c r="B22" s="106" t="inlineStr">
-        <is>
-          <t>④</t>
-        </is>
-      </c>
-      <c r="C22" s="106" t="inlineStr">
-        <is>
-          <t>現場直接作業</t>
-        </is>
-      </c>
-      <c r="D22" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="E22" s="106" t="n">
-        <v>0</v>
-      </c>
-      <c r="F22" s="106" t="n">
-        <v>0</v>
-      </c>
-    </row>
-    <row r="23">
-      <c r="B23" s="100" t="inlineStr">
-        <is>
-          <t>⑤</t>
-        </is>
-      </c>
-      <c r="C23" s="100" t="inlineStr">
-        <is>
-          <t>社内事務・管理</t>
-        </is>
-      </c>
-      <c r="D23" s="100" t="n">
-        <v>55</v>
-      </c>
-      <c r="E23" s="100" t="n">
+      <c r="F27" s="100" t="n">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="28">
+      <c r="B28" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C28" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D28" s="95" t="n">
+        <v>52</v>
+      </c>
+      <c r="E28" s="95" t="n">
         <v>0.9</v>
       </c>
-      <c r="F23" s="100" t="n">
-        <v>19.4</v>
-      </c>
-    </row>
-    <row r="24">
-      <c r="B24" s="95" t="inlineStr">
-        <is>
-          <t>⑥</t>
-        </is>
-      </c>
-      <c r="C24" s="95" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D24" s="95" t="n">
-        <v>42</v>
-      </c>
-      <c r="E24" s="95" t="n">
-        <v>0.7</v>
-      </c>
-      <c r="F24" s="95" t="n">
-        <v>14.8</v>
-      </c>
-    </row>
-    <row r="25">
-      <c r="B25" s="107" t="inlineStr">
+      <c r="F28" s="95" t="n">
+        <v>11.4</v>
+      </c>
+    </row>
+    <row r="29">
+      <c r="B29" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D25" s="107" t="n">
-        <v>284</v>
-      </c>
-      <c r="E25" s="107" t="n">
-        <v>4.7</v>
-      </c>
-      <c r="F25" s="107" t="n">
+      <c r="D29" s="107" t="n">
+        <v>456</v>
+      </c>
+      <c r="E29" s="107" t="n">
+        <v>7.6</v>
+      </c>
+      <c r="F29" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-03: close 雑務PC作業 15:35-17:13, 業務終了
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G29"/>
+  <dimension ref="B1:G29"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15435,10 +15435,12 @@
       </c>
       <c r="F20" s="100" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G20" s="100" t="n"/>
+          <t>17:13</t>
+        </is>
+      </c>
+      <c r="G20" s="100" t="n">
+        <v>98</v>
+      </c>
     </row>
     <row r="21">
       <c r="B21" s="104" t="inlineStr">
@@ -15518,7 +15520,7 @@
         <v>3.4</v>
       </c>
       <c r="F24" s="96" t="n">
-        <v>45.2</v>
+        <v>37.2</v>
       </c>
     </row>
     <row r="25">
@@ -15539,7 +15541,7 @@
         <v>2.4</v>
       </c>
       <c r="F25" s="98" t="n">
-        <v>31.4</v>
+        <v>25.8</v>
       </c>
     </row>
     <row r="26">
@@ -15575,13 +15577,13 @@
         </is>
       </c>
       <c r="D27" s="100" t="n">
-        <v>55</v>
+        <v>153</v>
       </c>
       <c r="E27" s="100" t="n">
-        <v>0.9</v>
+        <v>2.5</v>
       </c>
       <c r="F27" s="100" t="n">
-        <v>12.1</v>
+        <v>27.6</v>
       </c>
     </row>
     <row r="28">
@@ -15602,7 +15604,7 @@
         <v>0.9</v>
       </c>
       <c r="F28" s="95" t="n">
-        <v>11.4</v>
+        <v>9.4</v>
       </c>
     </row>
     <row r="29">
@@ -15612,10 +15614,10 @@
         </is>
       </c>
       <c r="D29" s="107" t="n">
-        <v>456</v>
+        <v>554</v>
       </c>
       <c r="E29" s="107" t="n">
-        <v>7.6</v>
+        <v>9.199999999999999</v>
       </c>
       <c r="F29" s="107" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Update 2026-06-03: start メールチェック 17:13
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G29"/>
+  <dimension ref="A1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15443,183 +15443,211 @@
       </c>
     </row>
     <row r="21">
-      <c r="B21" s="104" t="inlineStr">
+      <c r="B21" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C21" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D21" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック</t>
+        </is>
+      </c>
+      <c r="E21" s="100" t="inlineStr">
+        <is>
+          <t>17:13</t>
+        </is>
+      </c>
+      <c r="F21" s="100" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G21" s="100" t="n"/>
+    </row>
+    <row r="22">
+      <c r="B22" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-      <c r="C21" s="93" t="n"/>
-      <c r="D21" s="93" t="n"/>
-      <c r="E21" s="93" t="n"/>
-      <c r="F21" s="93" t="n"/>
-      <c r="G21" s="94" t="n"/>
-    </row>
-    <row r="22">
-      <c r="B22" s="79" t="inlineStr">
+      <c r="C22" s="93" t="n"/>
+      <c r="D22" s="93" t="n"/>
+      <c r="E22" s="93" t="n"/>
+      <c r="F22" s="93" t="n"/>
+      <c r="G22" s="94" t="n"/>
+    </row>
+    <row r="23">
+      <c r="B23" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C22" s="79" t="inlineStr">
+      <c r="C23" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D22" s="79" t="inlineStr">
+      <c r="D23" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E22" s="79" t="inlineStr">
+      <c r="E23" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F22" s="79" t="inlineStr">
+      <c r="F23" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="23">
-      <c r="B23" s="105" t="inlineStr">
+    <row r="24">
+      <c r="B24" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C23" s="105" t="inlineStr">
+      <c r="C24" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D23" s="105" t="n">
+      <c r="D24" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E23" s="105" t="n">
+      <c r="E24" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F23" s="105" t="n">
+      <c r="F24" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="24">
-      <c r="B24" s="96" t="inlineStr">
+    <row r="25">
+      <c r="B25" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C24" s="96" t="inlineStr">
+      <c r="C25" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D24" s="96" t="n">
+      <c r="D25" s="96" t="n">
         <v>206</v>
       </c>
-      <c r="E24" s="96" t="n">
+      <c r="E25" s="96" t="n">
         <v>3.4</v>
       </c>
-      <c r="F24" s="96" t="n">
+      <c r="F25" s="96" t="n">
         <v>37.2</v>
       </c>
     </row>
-    <row r="25">
-      <c r="B25" s="98" t="inlineStr">
+    <row r="26">
+      <c r="B26" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C25" s="98" t="inlineStr">
+      <c r="C26" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D25" s="98" t="n">
+      <c r="D26" s="98" t="n">
         <v>143</v>
       </c>
-      <c r="E25" s="98" t="n">
+      <c r="E26" s="98" t="n">
         <v>2.4</v>
       </c>
-      <c r="F25" s="98" t="n">
+      <c r="F26" s="98" t="n">
         <v>25.8</v>
       </c>
     </row>
-    <row r="26">
-      <c r="B26" s="106" t="inlineStr">
+    <row r="27">
+      <c r="B27" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C26" s="106" t="inlineStr">
+      <c r="C27" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D26" s="106" t="n">
+      <c r="D27" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E26" s="106" t="n">
+      <c r="E27" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F26" s="106" t="n">
+      <c r="F27" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="27">
-      <c r="B27" s="100" t="inlineStr">
+    <row r="28">
+      <c r="B28" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C27" s="100" t="inlineStr">
+      <c r="C28" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D27" s="100" t="n">
+      <c r="D28" s="100" t="n">
         <v>153</v>
       </c>
-      <c r="E27" s="100" t="n">
+      <c r="E28" s="100" t="n">
         <v>2.5</v>
       </c>
-      <c r="F27" s="100" t="n">
+      <c r="F28" s="100" t="n">
         <v>27.6</v>
       </c>
     </row>
-    <row r="28">
-      <c r="B28" s="95" t="inlineStr">
+    <row r="29">
+      <c r="B29" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C28" s="95" t="inlineStr">
+      <c r="C29" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D28" s="95" t="n">
+      <c r="D29" s="95" t="n">
         <v>52</v>
       </c>
-      <c r="E28" s="95" t="n">
+      <c r="E29" s="95" t="n">
         <v>0.9</v>
       </c>
-      <c r="F28" s="95" t="n">
+      <c r="F29" s="95" t="n">
         <v>9.4</v>
       </c>
     </row>
-    <row r="29">
-      <c r="B29" s="107" t="inlineStr">
+    <row r="30">
+      <c r="B30" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D29" s="107" t="n">
+      <c r="D30" s="107" t="n">
         <v>554</v>
       </c>
-      <c r="E29" s="107" t="n">
+      <c r="E30" s="107" t="n">
         <v>9.199999999999999</v>
       </c>
-      <c r="F29" s="107" t="n">
+      <c r="F30" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-03: close メールチェック 17:13-17:30, 業務終了
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -14847,7 +14847,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G30"/>
+  <dimension ref="B1:G30"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15465,10 +15465,12 @@
       </c>
       <c r="F21" s="100" t="inlineStr">
         <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G21" s="100" t="n"/>
+          <t>17:30</t>
+        </is>
+      </c>
+      <c r="G21" s="100" t="n">
+        <v>17</v>
+      </c>
     </row>
     <row r="22">
       <c r="B22" s="104" t="inlineStr">
@@ -15548,7 +15550,7 @@
         <v>3.4</v>
       </c>
       <c r="F25" s="96" t="n">
-        <v>37.2</v>
+        <v>36.1</v>
       </c>
     </row>
     <row r="26">
@@ -15569,7 +15571,7 @@
         <v>2.4</v>
       </c>
       <c r="F26" s="98" t="n">
-        <v>25.8</v>
+        <v>25</v>
       </c>
     </row>
     <row r="27">
@@ -15605,13 +15607,13 @@
         </is>
       </c>
       <c r="D28" s="100" t="n">
-        <v>153</v>
+        <v>170</v>
       </c>
       <c r="E28" s="100" t="n">
-        <v>2.5</v>
+        <v>2.8</v>
       </c>
       <c r="F28" s="100" t="n">
-        <v>27.6</v>
+        <v>29.8</v>
       </c>
     </row>
     <row r="29">
@@ -15632,7 +15634,7 @@
         <v>0.9</v>
       </c>
       <c r="F29" s="95" t="n">
-        <v>9.4</v>
+        <v>9.1</v>
       </c>
     </row>
     <row r="30">
@@ -15642,10 +15644,10 @@
         </is>
       </c>
       <c r="D30" s="107" t="n">
-        <v>554</v>
+        <v>571</v>
       </c>
       <c r="E30" s="107" t="n">
-        <v>9.199999999999999</v>
+        <v>9.5</v>
       </c>
       <c r="F30" s="107" t="n">
         <v>100</v>

</xml_diff>

<commit_message>
Add 2026-06-04: new sheet, tasks 7:59-12:11, 昼休憩 in progress
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -24,14 +24,15 @@
     <sheet name="2026-06-01" sheetId="16" state="visible" r:id="rId16"/>
     <sheet name="2026-06-02" sheetId="17" state="visible" r:id="rId17"/>
     <sheet name="2026-06-03" sheetId="18" state="visible" r:id="rId18"/>
+    <sheet name="2026-06-04" sheetId="19" state="visible" r:id="rId19"/>
   </sheets>
   <externalReferences>
-    <externalReference r:id="rId19"/>
     <externalReference r:id="rId20"/>
     <externalReference r:id="rId21"/>
     <externalReference r:id="rId22"/>
     <externalReference r:id="rId23"/>
     <externalReference r:id="rId24"/>
+    <externalReference r:id="rId25"/>
   </externalReferences>
   <definedNames>
     <definedName name="_13月">#REF!</definedName>
@@ -15661,6 +15662,545 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet19.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <sheetPr>
+    <outlinePr summaryBelow="1" summaryRight="1"/>
+    <pageSetUpPr/>
+  </sheetPr>
+  <dimension ref="B1:G21"/>
+  <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
+  <cols>
+    <col width="6" customWidth="1" style="64" min="2" max="2"/>
+    <col width="18" customWidth="1" style="64" min="3" max="3"/>
+    <col width="42" customWidth="1" style="64" min="4" max="4"/>
+    <col width="8" customWidth="1" style="64" min="5" max="5"/>
+    <col width="8" customWidth="1" style="64" min="6" max="6"/>
+    <col width="12" customWidth="1" style="64" min="7" max="7"/>
+  </cols>
+  <sheetData>
+    <row r="1" ht="24" customHeight="1" s="64">
+      <c r="B1" s="102" t="inlineStr">
+        <is>
+          <t>2026年6月4日（木）　業務記録</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" ht="20" customHeight="1" s="64">
+      <c r="B2" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C2" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D2" s="79" t="inlineStr">
+        <is>
+          <t>業務内容</t>
+        </is>
+      </c>
+      <c r="E2" s="79" t="inlineStr">
+        <is>
+          <t>開始</t>
+        </is>
+      </c>
+      <c r="F2" s="79" t="inlineStr">
+        <is>
+          <t>終了</t>
+        </is>
+      </c>
+      <c r="G2" s="79" t="inlineStr">
+        <is>
+          <t>所要時間（分）</t>
+        </is>
+      </c>
+    </row>
+    <row r="3" ht="18" customHeight="1" s="64">
+      <c r="B3" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C3" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D3" s="103" t="inlineStr">
+        <is>
+          <t>ラジオ体操</t>
+        </is>
+      </c>
+      <c r="E3" s="95" t="inlineStr">
+        <is>
+          <t>7:59</t>
+        </is>
+      </c>
+      <c r="F3" s="95" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="G3" s="95" t="n">
+        <v>4</v>
+      </c>
+    </row>
+    <row r="4" ht="18" customHeight="1" s="64">
+      <c r="B4" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C4" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D4" s="97" t="inlineStr">
+        <is>
+          <t>各職場朝礼参加</t>
+        </is>
+      </c>
+      <c r="E4" s="96" t="inlineStr">
+        <is>
+          <t>8:03</t>
+        </is>
+      </c>
+      <c r="F4" s="96" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="G4" s="96" t="n">
+        <v>3</v>
+      </c>
+    </row>
+    <row r="5" ht="18" customHeight="1" s="64">
+      <c r="B5" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C5" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D5" s="99" t="inlineStr">
+        <is>
+          <t>現場周り</t>
+        </is>
+      </c>
+      <c r="E5" s="98" t="inlineStr">
+        <is>
+          <t>8:06</t>
+        </is>
+      </c>
+      <c r="F5" s="98" t="inlineStr">
+        <is>
+          <t>8:30</t>
+        </is>
+      </c>
+      <c r="G5" s="98" t="n">
+        <v>24</v>
+      </c>
+    </row>
+    <row r="6" ht="18" customHeight="1" s="64">
+      <c r="B6" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C6" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D6" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック</t>
+        </is>
+      </c>
+      <c r="E6" s="100" t="inlineStr">
+        <is>
+          <t>8:30</t>
+        </is>
+      </c>
+      <c r="F6" s="100" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="G6" s="100" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="7" ht="18" customHeight="1" s="64">
+      <c r="B7" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C7" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D7" s="97" t="inlineStr">
+        <is>
+          <t>製造計画会議</t>
+        </is>
+      </c>
+      <c r="E7" s="96" t="inlineStr">
+        <is>
+          <t>9:00</t>
+        </is>
+      </c>
+      <c r="F7" s="96" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="G7" s="96" t="n">
+        <v>60</v>
+      </c>
+    </row>
+    <row r="8" ht="18" customHeight="1" s="64">
+      <c r="B8" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C8" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D8" s="103" t="inlineStr">
+        <is>
+          <t>休憩</t>
+        </is>
+      </c>
+      <c r="E8" s="95" t="inlineStr">
+        <is>
+          <t>10:00</t>
+        </is>
+      </c>
+      <c r="F8" s="95" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="G8" s="95" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="9" ht="18" customHeight="1" s="64">
+      <c r="B9" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C9" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D9" s="97" t="inlineStr">
+        <is>
+          <t>製造計画会議（続き）</t>
+        </is>
+      </c>
+      <c r="E9" s="96" t="inlineStr">
+        <is>
+          <t>10:10</t>
+        </is>
+      </c>
+      <c r="F9" s="96" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="G9" s="96" t="n">
+        <v>80</v>
+      </c>
+    </row>
+    <row r="10" ht="18" customHeight="1" s="64">
+      <c r="B10" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C10" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D10" s="99" t="inlineStr">
+        <is>
+          <t>現場指示</t>
+        </is>
+      </c>
+      <c r="E10" s="98" t="inlineStr">
+        <is>
+          <t>11:30</t>
+        </is>
+      </c>
+      <c r="F10" s="98" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="G10" s="98" t="n">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="11" ht="18" customHeight="1" s="64">
+      <c r="B11" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C11" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D11" s="101" t="inlineStr">
+        <is>
+          <t>メールチェック</t>
+        </is>
+      </c>
+      <c r="E11" s="100" t="inlineStr">
+        <is>
+          <t>11:40</t>
+        </is>
+      </c>
+      <c r="F11" s="100" t="inlineStr">
+        <is>
+          <t>12:11</t>
+        </is>
+      </c>
+      <c r="G11" s="100" t="n">
+        <v>31</v>
+      </c>
+    </row>
+    <row r="12" ht="18" customHeight="1" s="64">
+      <c r="B12" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C12" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D12" s="103" t="inlineStr">
+        <is>
+          <t>昼休憩</t>
+        </is>
+      </c>
+      <c r="E12" s="95" t="inlineStr">
+        <is>
+          <t>12:11</t>
+        </is>
+      </c>
+      <c r="F12" s="95" t="inlineStr">
+        <is>
+          <t>---</t>
+        </is>
+      </c>
+      <c r="G12" s="95" t="n"/>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="104" t="inlineStr">
+        <is>
+          <t>【カテゴリ別集計】</t>
+        </is>
+      </c>
+    </row>
+    <row r="14">
+      <c r="B14" s="79" t="inlineStr">
+        <is>
+          <t>No.</t>
+        </is>
+      </c>
+      <c r="C14" s="79" t="inlineStr">
+        <is>
+          <t>カテゴリ名</t>
+        </is>
+      </c>
+      <c r="D14" s="79" t="inlineStr">
+        <is>
+          <t>合計（分）</t>
+        </is>
+      </c>
+      <c r="E14" s="79" t="inlineStr">
+        <is>
+          <t>合計（時間）</t>
+        </is>
+      </c>
+      <c r="F14" s="79" t="inlineStr">
+        <is>
+          <t>割合（%）</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="105" t="inlineStr">
+        <is>
+          <t>①</t>
+        </is>
+      </c>
+      <c r="C15" s="105" t="inlineStr">
+        <is>
+          <t>経営・対外業務</t>
+        </is>
+      </c>
+      <c r="D15" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="E15" s="105" t="n">
+        <v>0</v>
+      </c>
+      <c r="F15" s="105" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="96" t="inlineStr">
+        <is>
+          <t>②</t>
+        </is>
+      </c>
+      <c r="C16" s="96" t="inlineStr">
+        <is>
+          <t>社内マネジメント</t>
+        </is>
+      </c>
+      <c r="D16" s="96" t="n">
+        <v>143</v>
+      </c>
+      <c r="E16" s="96" t="n">
+        <v>2.4</v>
+      </c>
+      <c r="F16" s="96" t="n">
+        <v>56.7</v>
+      </c>
+    </row>
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="98" t="inlineStr">
+        <is>
+          <t>③</t>
+        </is>
+      </c>
+      <c r="C17" s="98" t="inlineStr">
+        <is>
+          <t>現場管理・監督</t>
+        </is>
+      </c>
+      <c r="D17" s="98" t="n">
+        <v>34</v>
+      </c>
+      <c r="E17" s="98" t="n">
+        <v>0.6</v>
+      </c>
+      <c r="F17" s="98" t="n">
+        <v>13.5</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="106" t="inlineStr">
+        <is>
+          <t>④</t>
+        </is>
+      </c>
+      <c r="C18" s="106" t="inlineStr">
+        <is>
+          <t>現場直接作業</t>
+        </is>
+      </c>
+      <c r="D18" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="E18" s="106" t="n">
+        <v>0</v>
+      </c>
+      <c r="F18" s="106" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="100" t="inlineStr">
+        <is>
+          <t>⑤</t>
+        </is>
+      </c>
+      <c r="C19" s="100" t="inlineStr">
+        <is>
+          <t>社内事務・管理</t>
+        </is>
+      </c>
+      <c r="D19" s="100" t="n">
+        <v>61</v>
+      </c>
+      <c r="E19" s="100" t="n">
+        <v>1</v>
+      </c>
+      <c r="F19" s="100" t="n">
+        <v>24.2</v>
+      </c>
+    </row>
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C20" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D20" s="95" t="n">
+        <v>14</v>
+      </c>
+      <c r="E20" s="95" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="F20" s="95" t="n">
+        <v>5.6</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="64">
+      <c r="B21" s="107" t="inlineStr">
+        <is>
+          <t>合計</t>
+        </is>
+      </c>
+      <c r="D21" s="107" t="n">
+        <v>252</v>
+      </c>
+      <c r="E21" s="107" t="n">
+        <v>4.2</v>
+      </c>
+      <c r="F21" s="107" t="n">
+        <v>100</v>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="B13:G13"/>
+    <mergeCell ref="B1:G1"/>
+  </mergeCells>
+  <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <sheetPr>

</xml_diff>

<commit_message>
Update 2026-06-04: close 昼休憩 12:11-12:41, start 掃除 12:41
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -15668,7 +15668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="B1:G21"/>
+  <dimension ref="A1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -15685,6 +15685,11 @@
           <t>2026年6月4日（木）　業務記録</t>
         </is>
       </c>
+      <c r="C1" s="93" t="n"/>
+      <c r="D1" s="93" t="n"/>
+      <c r="E1" s="93" t="n"/>
+      <c r="F1" s="93" t="n"/>
+      <c r="G1" s="94" t="n"/>
     </row>
     <row r="2" ht="20" customHeight="1" s="64">
       <c r="B2" s="79" t="inlineStr">
@@ -16011,184 +16016,219 @@
       </c>
       <c r="F12" s="95" t="inlineStr">
         <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="G12" s="95" t="n">
+        <v>30</v>
+      </c>
+    </row>
+    <row r="13" ht="18" customHeight="1" s="64">
+      <c r="B13" s="95" t="inlineStr">
+        <is>
+          <t>⑥</t>
+        </is>
+      </c>
+      <c r="C13" s="95" t="inlineStr">
+        <is>
+          <t>定常・移動・休憩</t>
+        </is>
+      </c>
+      <c r="D13" s="103" t="inlineStr">
+        <is>
+          <t>掃除</t>
+        </is>
+      </c>
+      <c r="E13" s="95" t="inlineStr">
+        <is>
+          <t>12:41</t>
+        </is>
+      </c>
+      <c r="F13" s="95" t="inlineStr">
+        <is>
           <t>---</t>
         </is>
       </c>
-      <c r="G12" s="95" t="n"/>
-    </row>
-    <row r="13" ht="18" customHeight="1" s="64">
-      <c r="B13" s="104" t="inlineStr">
+      <c r="G13" s="95" t="n"/>
+    </row>
+    <row r="14">
+      <c r="B14" s="104" t="inlineStr">
         <is>
           <t>【カテゴリ別集計】</t>
         </is>
       </c>
-    </row>
-    <row r="14">
-      <c r="B14" s="79" t="inlineStr">
+      <c r="C14" s="93" t="n"/>
+      <c r="D14" s="93" t="n"/>
+      <c r="E14" s="93" t="n"/>
+      <c r="F14" s="93" t="n"/>
+      <c r="G14" s="94" t="n"/>
+    </row>
+    <row r="15" ht="18" customHeight="1" s="64">
+      <c r="B15" s="79" t="inlineStr">
         <is>
           <t>No.</t>
         </is>
       </c>
-      <c r="C14" s="79" t="inlineStr">
+      <c r="C15" s="79" t="inlineStr">
         <is>
           <t>カテゴリ名</t>
         </is>
       </c>
-      <c r="D14" s="79" t="inlineStr">
+      <c r="D15" s="79" t="inlineStr">
         <is>
           <t>合計（分）</t>
         </is>
       </c>
-      <c r="E14" s="79" t="inlineStr">
+      <c r="E15" s="79" t="inlineStr">
         <is>
           <t>合計（時間）</t>
         </is>
       </c>
-      <c r="F14" s="79" t="inlineStr">
+      <c r="F15" s="79" t="inlineStr">
         <is>
           <t>割合（%）</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="18" customHeight="1" s="64">
-      <c r="B15" s="105" t="inlineStr">
+    <row r="16" ht="18" customHeight="1" s="64">
+      <c r="B16" s="105" t="inlineStr">
         <is>
           <t>①</t>
         </is>
       </c>
-      <c r="C15" s="105" t="inlineStr">
+      <c r="C16" s="105" t="inlineStr">
         <is>
           <t>経営・対外業務</t>
         </is>
       </c>
-      <c r="D15" s="105" t="n">
+      <c r="D16" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="E15" s="105" t="n">
+      <c r="E16" s="105" t="n">
         <v>0</v>
       </c>
-      <c r="F15" s="105" t="n">
+      <c r="F16" s="105" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="16" ht="18" customHeight="1" s="64">
-      <c r="B16" s="96" t="inlineStr">
+    <row r="17" ht="18" customHeight="1" s="64">
+      <c r="B17" s="96" t="inlineStr">
         <is>
           <t>②</t>
         </is>
       </c>
-      <c r="C16" s="96" t="inlineStr">
+      <c r="C17" s="96" t="inlineStr">
         <is>
           <t>社内マネジメント</t>
         </is>
       </c>
-      <c r="D16" s="96" t="n">
+      <c r="D17" s="96" t="n">
         <v>143</v>
       </c>
-      <c r="E16" s="96" t="n">
+      <c r="E17" s="96" t="n">
         <v>2.4</v>
       </c>
-      <c r="F16" s="96" t="n">
-        <v>56.7</v>
-      </c>
-    </row>
-    <row r="17" ht="18" customHeight="1" s="64">
-      <c r="B17" s="98" t="inlineStr">
+      <c r="F17" s="96" t="n">
+        <v>50.7</v>
+      </c>
+    </row>
+    <row r="18" ht="18" customHeight="1" s="64">
+      <c r="B18" s="98" t="inlineStr">
         <is>
           <t>③</t>
         </is>
       </c>
-      <c r="C17" s="98" t="inlineStr">
+      <c r="C18" s="98" t="inlineStr">
         <is>
           <t>現場管理・監督</t>
         </is>
       </c>
-      <c r="D17" s="98" t="n">
+      <c r="D18" s="98" t="n">
         <v>34</v>
       </c>
-      <c r="E17" s="98" t="n">
+      <c r="E18" s="98" t="n">
         <v>0.6</v>
       </c>
-      <c r="F17" s="98" t="n">
-        <v>13.5</v>
-      </c>
-    </row>
-    <row r="18" ht="18" customHeight="1" s="64">
-      <c r="B18" s="106" t="inlineStr">
+      <c r="F18" s="98" t="n">
+        <v>12.1</v>
+      </c>
+    </row>
+    <row r="19" ht="18" customHeight="1" s="64">
+      <c r="B19" s="106" t="inlineStr">
         <is>
           <t>④</t>
         </is>
       </c>
-      <c r="C18" s="106" t="inlineStr">
+      <c r="C19" s="106" t="inlineStr">
         <is>
           <t>現場直接作業</t>
         </is>
       </c>
-      <c r="D18" s="106" t="n">
+      <c r="D19" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="E18" s="106" t="n">
+      <c r="E19" s="106" t="n">
         <v>0</v>
       </c>
-      <c r="F18" s="106" t="n">
+      <c r="F19" s="106" t="n">
         <v>0</v>
       </c>
     </row>
-    <row r="19" ht="18" customHeight="1" s="64">
-      <c r="B19" s="100" t="inlineStr">
+    <row r="20" ht="18" customHeight="1" s="64">
+      <c r="B20" s="100" t="inlineStr">
         <is>
           <t>⑤</t>
         </is>
       </c>
-      <c r="C19" s="100" t="inlineStr">
+      <c r="C20" s="100" t="inlineStr">
         <is>
           <t>社内事務・管理</t>
         </is>
       </c>
-      <c r="D19" s="100" t="n">
+      <c r="D20" s="100" t="n">
         <v>61</v>
       </c>
-      <c r="E19" s="100" t="n">
+      <c r="E20" s="100" t="n">
         <v>1</v>
       </c>
-      <c r="F19" s="100" t="n">
-        <v>24.2</v>
-      </c>
-    </row>
-    <row r="20" ht="18" customHeight="1" s="64">
-      <c r="B20" s="95" t="inlineStr">
+      <c r="F20" s="100" t="n">
+        <v>21.6</v>
+      </c>
+    </row>
+    <row r="21" ht="18" customHeight="1" s="64">
+      <c r="B21" s="95" t="inlineStr">
         <is>
           <t>⑥</t>
         </is>
       </c>
-      <c r="C20" s="95" t="inlineStr">
+      <c r="C21" s="95" t="inlineStr">
         <is>
           <t>定常・移動・休憩</t>
         </is>
       </c>
-      <c r="D20" s="95" t="n">
-        <v>14</v>
-      </c>
-      <c r="E20" s="95" t="n">
-        <v>0.2</v>
-      </c>
-      <c r="F20" s="95" t="n">
-        <v>5.6</v>
-      </c>
-    </row>
-    <row r="21" ht="18" customHeight="1" s="64">
-      <c r="B21" s="107" t="inlineStr">
+      <c r="D21" s="95" t="n">
+        <v>44</v>
+      </c>
+      <c r="E21" s="95" t="n">
+        <v>0.7</v>
+      </c>
+      <c r="F21" s="95" t="n">
+        <v>15.6</v>
+      </c>
+    </row>
+    <row r="22">
+      <c r="B22" s="107" t="inlineStr">
         <is>
           <t>合計</t>
         </is>
       </c>
-      <c r="D21" s="107" t="n">
-        <v>252</v>
-      </c>
-      <c r="E21" s="107" t="n">
-        <v>4.2</v>
-      </c>
-      <c r="F21" s="107" t="n">
+      <c r="D22" s="107" t="n">
+        <v>282</v>
+      </c>
+      <c r="E22" s="107" t="n">
+        <v>4.7</v>
+      </c>
+      <c r="F22" s="107" t="n">
         <v>100</v>
       </c>
     </row>

</xml_diff>

<commit_message>
Update 2026-06-04: 掃除 12:41-12:52, 現場周り 12:52-13:05, start 事務作業 13:05
https://claude.ai/code/session_01XKGWn6H6rA1soQpAVWBV9K
</commit_message>
<xml_diff>
--- a/業務記録.xlsx
+++ b/業務記録.xlsx
@@ -15668,7 +15668,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G22"/>
+  <dimension ref="B1:G22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" style="64" min="2" max="2"/>
@@ -16029,27 +16029,11 @@
           <t>⑥</t>
         </is>
       </c>
-      <c r="C13" s="95" t="inlineStr">
-        <is>
-          <t>定常・移動・休憩</t>
-        </is>
-      </c>
-      <c r="D13" s="103" t="inlineStr">
-        <is>
-          <t>掃除</t>
-        </is>
-      </c>
-      <c r="E13" s="95" t="inlineStr">
-        <is>
-          <t>12:41</t>
-        </is>
-      </c>
-      <c r="F13" s="95" t="inlineStr">
-        <is>
-          <t>---</t>
-        </is>
-      </c>
-      <c r="G13" s="95" t="n"/>
+      <c r="C13" s="93" t="n"/>
+      <c r="D13" s="93" t="n"/>
+      <c r="E13" s="93" t="n"/>
+      <c r="F13" s="93" t="n"/>
+      <c r="G13" s="94" t="n"/>
     </row>
     <row r="14">
       <c r="B14" s="104" t="inlineStr">
@@ -16129,7 +16113,7 @@
         <v>2.4</v>
       </c>
       <c r="F17" s="96" t="n">
-        <v>50.7</v>
+        <v>46.7</v>
       </c>
     </row>
     <row r="18" ht="18" customHeight="1" s="64">
@@ -16144,13 +16128,13 @@
         </is>
       </c>
       <c r="D18" s="98" t="n">
-        <v>34</v>
+        <v>47</v>
       </c>
       <c r="E18" s="98" t="n">
-        <v>0.6</v>
+        <v>0.8</v>
       </c>
       <c r="F18" s="98" t="n">
-        <v>12.1</v>
+        <v>15.4</v>
       </c>
     </row>
     <row r="19" ht="18" customHeight="1" s="64">
@@ -16192,7 +16176,7 @@
         <v>1</v>
       </c>
       <c r="F20" s="100" t="n">
-        <v>21.6</v>
+        <v>19.9</v>
       </c>
     </row>
     <row r="21" ht="18" customHeight="1" s="64">
@@ -16207,13 +16191,13 @@
         </is>
       </c>
       <c r="D21" s="95" t="n">
-        <v>44</v>
+        <v>55</v>
       </c>
       <c r="E21" s="95" t="n">
-        <v>0.7</v>
+        <v>0.9</v>
       </c>
       <c r="F21" s="95" t="n">
-        <v>15.6</v>
+        <v>18</v>
       </c>
     </row>
     <row r="22">
@@ -16223,10 +16207,10 @@
         </is>
       </c>
       <c r="D22" s="107" t="n">
-        <v>282</v>
+        <v>306</v>
       </c>
       <c r="E22" s="107" t="n">
-        <v>4.7</v>
+        <v>5.1</v>
       </c>
       <c r="F22" s="107" t="n">
         <v>100</v>

</xml_diff>